<commit_message>
Add Zone.Identifier file for template.docx to manage file transfer settings
</commit_message>
<xml_diff>
--- a/main/05_data_charting/data/Individual_Annotations.xlsx
+++ b/main/05_data_charting/data/Individual_Annotations.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\orincon\scoping-ml-wave-seismology\main\05_data_charting\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBE66586-DEE0-458E-8D40-DFB3A9E9E5B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AA02972-EE00-434F-A5B6-BEB531168360}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{115BB8D9-8B86-4726-97F8-E06477FD353D}"/>
+    <workbookView xWindow="-28935" yWindow="-135" windowWidth="29070" windowHeight="15750" xr2:uid="{115BB8D9-8B86-4726-97F8-E06477FD353D}"/>
   </bookViews>
   <sheets>
     <sheet name="Oscar" sheetId="4" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="694" uniqueCount="429">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="698" uniqueCount="431">
   <si>
     <t>Research gaps</t>
   </si>
@@ -1576,6 +1576,12 @@
   </si>
   <si>
     <t>2D and 3D</t>
+  </si>
+  <si>
+    <t>Not the case </t>
+  </si>
+  <si>
+    <t xml:space="preserve">The primary quantitative metric is the L2 norm of the difference between PINN-predicted and FDFD-reference scattered wavefields. </t>
   </si>
 </sst>
 </file>
@@ -1634,12 +1640,18 @@
       <family val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="3">
@@ -1682,7 +1694,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1709,6 +1721,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2116,94 +2134,104 @@
         <v>417</v>
       </c>
     </row>
-    <row r="2" spans="1:16" s="4" customFormat="1" ht="250.8" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+    <row r="2" spans="1:16" s="11" customFormat="1" ht="250.8" x14ac:dyDescent="0.25">
+      <c r="A2" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="10" t="s">
         <v>421</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="H2" s="10" t="s">
         <v>241</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="I2" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="J2" s="3" t="s">
+      <c r="J2" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="K2" s="3" t="s">
+      <c r="K2" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="L2" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="M2" s="3" t="s">
+      <c r="L2" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="M2" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="N2" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="O2" s="3" t="s">
+      <c r="N2" s="10" t="s">
+        <v>429</v>
+      </c>
+      <c r="O2" s="10" t="s">
         <v>58</v>
       </c>
+      <c r="P2" s="11" t="s">
+        <v>234</v>
+      </c>
     </row>
-    <row r="3" spans="1:16" s="4" customFormat="1" ht="184.8" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
+    <row r="3" spans="1:16" s="11" customFormat="1" ht="184.8" x14ac:dyDescent="0.25">
+      <c r="A3" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="10" t="s">
         <v>419</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="G3" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="H3" s="3" t="s">
+      <c r="G3" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="H3" s="10" t="s">
         <v>241</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="I3" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="J3" s="3" t="s">
+      <c r="J3" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="K3" s="3" t="s">
+      <c r="K3" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="L3" s="3" t="s">
+      <c r="L3" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="M3" s="3"/>
-      <c r="N3" s="3"/>
-      <c r="O3" s="3" t="s">
+      <c r="M3" s="10" t="s">
+        <v>429</v>
+      </c>
+      <c r="N3" s="10" t="s">
+        <v>429</v>
+      </c>
+      <c r="O3" s="10" t="s">
         <v>66</v>
+      </c>
+      <c r="P3" s="11" t="s">
+        <v>430</v>
       </c>
     </row>
     <row r="4" spans="1:16" s="4" customFormat="1" ht="201" customHeight="1" x14ac:dyDescent="0.25">
@@ -2294,7 +2322,7 @@
         <v>75</v>
       </c>
       <c r="N5" s="3" t="s">
-        <v>46</v>
+        <v>429</v>
       </c>
       <c r="O5" s="3" t="s">
         <v>76</v>
@@ -2341,7 +2369,7 @@
         <v>83</v>
       </c>
       <c r="N6" s="3" t="s">
-        <v>46</v>
+        <v>429</v>
       </c>
       <c r="O6" s="3" t="s">
         <v>84</v>
@@ -2388,7 +2416,7 @@
         <v>91</v>
       </c>
       <c r="N7" s="3" t="s">
-        <v>46</v>
+        <v>429</v>
       </c>
       <c r="O7" s="3" t="s">
         <v>92</v>
@@ -2435,7 +2463,7 @@
         <v>99</v>
       </c>
       <c r="N8" s="3" t="s">
-        <v>46</v>
+        <v>429</v>
       </c>
       <c r="O8" s="3" t="s">
         <v>100</v>
@@ -2482,7 +2510,7 @@
         <v>106</v>
       </c>
       <c r="N9" s="3" t="s">
-        <v>46</v>
+        <v>429</v>
       </c>
       <c r="O9" s="3" t="s">
         <v>107</v>
@@ -2529,7 +2557,7 @@
         <v>111</v>
       </c>
       <c r="N10" s="3" t="s">
-        <v>46</v>
+        <v>429</v>
       </c>
       <c r="O10" s="3" t="s">
         <v>112</v>
@@ -2576,7 +2604,7 @@
         <v>118</v>
       </c>
       <c r="N11" s="3" t="s">
-        <v>46</v>
+        <v>429</v>
       </c>
       <c r="O11" s="3" t="s">
         <v>119</v>
@@ -4251,6 +4279,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x01010009048CEEA230F14796749F6DFD5F5263" ma:contentTypeVersion="4" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="5105af4e7c1b0ed6cdb04338eaf51f7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="96457c7a-bdfc-427e-9d05-5faa5ab5244b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0baee1a300280ca08e7397f1756276d6" ns2:_="">
     <xsd:import namespace="96457c7a-bdfc-427e-9d05-5faa5ab5244b"/>
@@ -4394,22 +4437,24 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1160EB8C-E200-4916-A3B3-9BF8115D37F8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24F2579D-323E-48EA-8FED-D372AFFF0A04}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{75ADFBF6-8C74-4292-833E-68A026E87063}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4425,21 +4470,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1160EB8C-E200-4916-A3B3-9BF8115D37F8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24F2579D-323E-48EA-8FED-D372AFFF0A04}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Add temporary files for Yang et al. (2023) and Individual Annotations
</commit_message>
<xml_diff>
--- a/main/05_data_charting/data/Individual_Annotations.xlsx
+++ b/main/05_data_charting/data/Individual_Annotations.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\orincon\scoping-ml-wave-seismology\main\05_data_charting\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AA02972-EE00-434F-A5B6-BEB531168360}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7ACFCC5C-6447-41E6-A2C7-8CE639F0952A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28935" yWindow="-135" windowWidth="29070" windowHeight="15750" xr2:uid="{115BB8D9-8B86-4726-97F8-E06477FD353D}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{115BB8D9-8B86-4726-97F8-E06477FD353D}"/>
   </bookViews>
   <sheets>
     <sheet name="Oscar" sheetId="4" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="698" uniqueCount="431">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="699" uniqueCount="432">
   <si>
     <t>Research gaps</t>
   </si>
@@ -1582,6 +1582,9 @@
   </si>
   <si>
     <t xml:space="preserve">The primary quantitative metric is the L2 norm of the difference between PINN-predicted and FDFD-reference scattered wavefields. </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> L2 norm of the difference between U-NO prediction and FDM ground truth, divided by the L2 norm of the ground truth. </t>
   </si>
 </sst>
 </file>
@@ -2234,51 +2237,54 @@
         <v>430</v>
       </c>
     </row>
-    <row r="4" spans="1:16" s="4" customFormat="1" ht="201" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+    <row r="4" spans="1:16" s="11" customFormat="1" ht="201" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="E4" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="F4" s="3" t="s">
+      <c r="E4" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="F4" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="G4" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="H4" s="3" t="s">
+      <c r="G4" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="H4" s="10" t="s">
         <v>241</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="I4" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="J4" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="K4" s="3" t="s">
+      <c r="J4" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="K4" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="L4" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="M4" s="3" t="s">
+      <c r="L4" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="M4" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="N4" s="3" t="s">
+      <c r="N4" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="O4" s="3" t="s">
+      <c r="O4" s="10" t="s">
         <v>71</v>
+      </c>
+      <c r="P4" s="11" t="s">
+        <v>431</v>
       </c>
     </row>
     <row r="5" spans="1:16" s="4" customFormat="1" ht="210" customHeight="1" x14ac:dyDescent="0.25">
@@ -4279,18 +4285,18 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4438,18 +4444,18 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1160EB8C-E200-4916-A3B3-9BF8115D37F8}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24F2579D-323E-48EA-8FED-D372AFFF0A04}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24F2579D-323E-48EA-8FED-D372AFFF0A04}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1160EB8C-E200-4916-A3B3-9BF8115D37F8}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Remove temporary Yang et al. (2023) document and add new template file for data extraction
</commit_message>
<xml_diff>
--- a/main/05_data_charting/data/Individual_Annotations.xlsx
+++ b/main/05_data_charting/data/Individual_Annotations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\orincon\scoping-ml-wave-seismology\main\05_data_charting\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7ACFCC5C-6447-41E6-A2C7-8CE639F0952A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F30138CE-47E9-48E1-80CA-8EEDE41C96CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{115BB8D9-8B86-4726-97F8-E06477FD353D}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="699" uniqueCount="432">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="710" uniqueCount="446">
   <si>
     <t>Research gaps</t>
   </si>
@@ -367,9 +367,6 @@
     <t>Keras</t>
   </si>
   <si>
-    <t>MOS and Devito</t>
-  </si>
-  <si>
     <t>This technique may open new perspectives of development, in particular the extension to the 2-D and 3-D elastic case. Due to the performance demonstrated in the present work, such extension may be feasible and they can lead to efficient alternative to classical methods. Nonetheless, the complexity of such extension will require a complete revision of the design of the net.</t>
   </si>
   <si>
@@ -501,12 +498,6 @@
 3.  Multiple shots are used as channels in the network to increase data redundancy.
 4.The use of multiple shot gathers as input channels to improve data redundancy and reduce overfitting. 
 5. The paper is well-written. The proposed method is explained clearly; however, some details about the synthetic data used are missing and would be appropriate to include.</t>
-  </si>
-  <si>
-    <t>a modified FCN</t>
-  </si>
-  <si>
-    <t>has fewer parameters and thus is more efficient than DNNs.</t>
   </si>
   <si>
     <t>To limit the scope of this paper, we focus on 2D isotropic acoustic models with a uniform and constant density.</t>
@@ -1585,6 +1576,58 @@
   </si>
   <si>
     <t xml:space="preserve"> L2 norm of the difference between U-NO prediction and FDM ground truth, divided by the L2 norm of the ground truth. </t>
+  </si>
+  <si>
+    <t>Visual comparison of wavefields and spatial correlation coefficient maps</t>
+  </si>
+  <si>
+    <t>Visual comparison and comparison of the computational time</t>
+  </si>
+  <si>
+    <t>R2 coefficient determination and relative peak error</t>
+  </si>
+  <si>
+    <t>Mean Absolute Error and computational time</t>
+  </si>
+  <si>
+    <t>Relative Mean Square Error and Mean Absolute Error were used as metrics</t>
+  </si>
+  <si>
+    <t>Squared-error losses, wavefield difference fields
+and Prediction error maps</t>
+  </si>
+  <si>
+    <t>Goodness-of-Fit (GOF) as metric</t>
+  </si>
+  <si>
+    <t>Visual comparison with reference</t>
+  </si>
+  <si>
+    <t>Error metrics as mean squared error (MSE) and absolute error</t>
+  </si>
+  <si>
+    <t> Velocity parameter inversion problem</t>
+  </si>
+  <si>
+    <t> Velocity (P- and S-wave) and density inversion.</t>
+  </si>
+  <si>
+    <t> Not extensively discussed.</t>
+  </si>
+  <si>
+    <t> The synthetic data generated using finite differences (FD) were used to train two neural networks.</t>
+  </si>
+  <si>
+    <t>to estimate the P-wave velocity models directly from the prestack seismic traces</t>
+  </si>
+  <si>
+    <t>L2 error and visual comparison</t>
+  </si>
+  <si>
+    <t>A modified FCN</t>
+  </si>
+  <si>
+    <t>It has fewer parameters and thus is more efficient than DNNs.</t>
   </si>
 </sst>
 </file>
@@ -2089,52 +2132,52 @@
   <sheetData>
     <row r="1" spans="1:16" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
       <c r="C1" s="9" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="9" t="s">
+        <v>403</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>405</v>
+      </c>
+      <c r="F1" s="9" t="s">
+        <v>404</v>
+      </c>
+      <c r="G1" s="9" t="s">
         <v>406</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="H1" s="9" t="s">
+        <v>407</v>
+      </c>
+      <c r="I1" s="9" t="s">
         <v>408</v>
       </c>
-      <c r="F1" s="9" t="s">
-        <v>407</v>
-      </c>
-      <c r="G1" s="9" t="s">
+      <c r="J1" s="9" t="s">
         <v>409</v>
       </c>
-      <c r="H1" s="9" t="s">
+      <c r="K1" s="9" t="s">
         <v>410</v>
       </c>
-      <c r="I1" s="9" t="s">
+      <c r="L1" s="9" t="s">
         <v>411</v>
       </c>
-      <c r="J1" s="9" t="s">
+      <c r="M1" s="8" t="s">
         <v>412</v>
       </c>
-      <c r="K1" s="9" t="s">
+      <c r="N1" s="8" t="s">
         <v>413</v>
-      </c>
-      <c r="L1" s="9" t="s">
-        <v>414</v>
-      </c>
-      <c r="M1" s="8" t="s">
-        <v>415</v>
-      </c>
-      <c r="N1" s="8" t="s">
-        <v>416</v>
       </c>
       <c r="O1" s="8" t="s">
         <v>0</v>
       </c>
       <c r="P1" s="7" t="s">
-        <v>417</v>
+        <v>414</v>
       </c>
     </row>
     <row r="2" spans="1:16" s="11" customFormat="1" ht="250.8" x14ac:dyDescent="0.25">
@@ -2151,7 +2194,7 @@
         <v>53</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>421</v>
+        <v>418</v>
       </c>
       <c r="F2" s="10" t="s">
         <v>62</v>
@@ -2160,7 +2203,7 @@
         <v>54</v>
       </c>
       <c r="H2" s="10" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="I2" s="10" t="s">
         <v>48</v>
@@ -2178,13 +2221,13 @@
         <v>57</v>
       </c>
       <c r="N2" s="10" t="s">
-        <v>429</v>
+        <v>426</v>
       </c>
       <c r="O2" s="10" t="s">
         <v>58</v>
       </c>
       <c r="P2" s="11" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
     </row>
     <row r="3" spans="1:16" s="11" customFormat="1" ht="184.8" x14ac:dyDescent="0.25">
@@ -2201,7 +2244,7 @@
         <v>61</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>419</v>
+        <v>416</v>
       </c>
       <c r="F3" s="10" t="s">
         <v>62</v>
@@ -2210,7 +2253,7 @@
         <v>56</v>
       </c>
       <c r="H3" s="10" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="I3" s="10" t="s">
         <v>48</v>
@@ -2225,16 +2268,16 @@
         <v>65</v>
       </c>
       <c r="M3" s="10" t="s">
-        <v>429</v>
+        <v>426</v>
       </c>
       <c r="N3" s="10" t="s">
-        <v>429</v>
+        <v>426</v>
       </c>
       <c r="O3" s="10" t="s">
         <v>66</v>
       </c>
       <c r="P3" s="11" t="s">
-        <v>430</v>
+        <v>427</v>
       </c>
     </row>
     <row r="4" spans="1:16" s="11" customFormat="1" ht="201" customHeight="1" x14ac:dyDescent="0.25">
@@ -2260,7 +2303,7 @@
         <v>56</v>
       </c>
       <c r="H4" s="10" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="I4" s="10" t="s">
         <v>48</v>
@@ -2284,524 +2327,557 @@
         <v>71</v>
       </c>
       <c r="P4" s="11" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" s="11" customFormat="1" ht="210" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="E5" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="F5" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="G5" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="H5" s="10" t="s">
+        <v>238</v>
+      </c>
+      <c r="I5" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="J5" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="K5" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="L5" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="M5" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="N5" s="10" t="s">
+        <v>426</v>
+      </c>
+      <c r="O5" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="P5" s="11" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" s="11" customFormat="1" ht="250.8" x14ac:dyDescent="0.25">
+      <c r="A6" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>170</v>
+      </c>
+      <c r="F6" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="G6" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="H6" s="10" t="s">
+        <v>238</v>
+      </c>
+      <c r="I6" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="J6" s="10" t="s">
+        <v>82</v>
+      </c>
+      <c r="K6" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="L6" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="M6" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="N6" s="10" t="s">
+        <v>426</v>
+      </c>
+      <c r="O6" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="P6" s="11" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" s="11" customFormat="1" ht="250.8" x14ac:dyDescent="0.25">
+      <c r="A7" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>87</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>88</v>
+      </c>
+      <c r="F7" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="G7" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="H7" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="I7" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="J7" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="K7" s="10" t="s">
+        <v>420</v>
+      </c>
+      <c r="L7" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="M7" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="N7" s="10" t="s">
+        <v>426</v>
+      </c>
+      <c r="O7" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="P7" s="11" t="s">
         <v>431</v>
       </c>
     </row>
-    <row r="5" spans="1:16" s="4" customFormat="1" ht="210" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="F5" s="3" t="s">
+    <row r="8" spans="1:16" s="11" customFormat="1" ht="184.8" x14ac:dyDescent="0.25">
+      <c r="A8" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="C8" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="D8" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="E8" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="F8" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="G5" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>241</v>
-      </c>
-      <c r="I5" s="3" t="s">
+      <c r="G8" s="10" t="s">
+        <v>122</v>
+      </c>
+      <c r="H8" s="10" t="s">
+        <v>238</v>
+      </c>
+      <c r="I8" s="10" t="s">
+        <v>244</v>
+      </c>
+      <c r="J8" s="10" t="s">
+        <v>97</v>
+      </c>
+      <c r="K8" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="L8" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="M8" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="N8" s="10" t="s">
+        <v>426</v>
+      </c>
+      <c r="O8" s="10" t="s">
+        <v>99</v>
+      </c>
+      <c r="P8" s="11" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" s="11" customFormat="1" ht="303.60000000000002" x14ac:dyDescent="0.25">
+      <c r="A9" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>100</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="D9" s="10" t="s">
+        <v>102</v>
+      </c>
+      <c r="E9" s="10" t="s">
+        <v>235</v>
+      </c>
+      <c r="F9" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="G9" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="H9" s="10" t="s">
+        <v>415</v>
+      </c>
+      <c r="I9" s="10" t="s">
+        <v>244</v>
+      </c>
+      <c r="J9" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="K9" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="L9" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="M9" s="10" t="s">
+        <v>105</v>
+      </c>
+      <c r="N9" s="10" t="s">
+        <v>426</v>
+      </c>
+      <c r="O9" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="P9" s="11" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" s="11" customFormat="1" ht="211.2" x14ac:dyDescent="0.25">
+      <c r="A10" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>107</v>
+      </c>
+      <c r="C10" s="10" t="s">
+        <v>108</v>
+      </c>
+      <c r="D10" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="E10" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="F10" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="G10" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="H10" s="10" t="s">
+        <v>238</v>
+      </c>
+      <c r="I10" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="J5" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="K5" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="L5" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="M5" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="N5" s="3" t="s">
-        <v>429</v>
-      </c>
-      <c r="O5" s="3" t="s">
-        <v>76</v>
+      <c r="J10" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="K10" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="L10" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="M10" s="10" t="s">
+        <v>110</v>
+      </c>
+      <c r="N10" s="10" t="s">
+        <v>426</v>
+      </c>
+      <c r="O10" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="P10" s="11" t="s">
+        <v>434</v>
       </c>
     </row>
-    <row r="6" spans="1:16" s="4" customFormat="1" ht="250.8" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>241</v>
-      </c>
-      <c r="I6" s="3" t="s">
+    <row r="11" spans="1:16" s="11" customFormat="1" ht="198" x14ac:dyDescent="0.25">
+      <c r="A11" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>112</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>113</v>
+      </c>
+      <c r="D11" s="10" t="s">
+        <v>114</v>
+      </c>
+      <c r="E11" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="F11" s="10" t="s">
+        <v>115</v>
+      </c>
+      <c r="G11" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="H11" s="10" t="s">
+        <v>238</v>
+      </c>
+      <c r="I11" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="J6" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="K6" s="3" t="s">
+      <c r="J11" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="K11" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="L6" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="M6" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="N6" s="3" t="s">
-        <v>429</v>
-      </c>
-      <c r="O6" s="3" t="s">
-        <v>84</v>
+      <c r="L11" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="M11" s="10" t="s">
+        <v>117</v>
+      </c>
+      <c r="N11" s="10" t="s">
+        <v>426</v>
+      </c>
+      <c r="O11" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="P11" s="11" t="s">
+        <v>435</v>
       </c>
     </row>
-    <row r="7" spans="1:16" s="4" customFormat="1" ht="250.8" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="F7" s="3" t="s">
+    <row r="12" spans="1:16" s="11" customFormat="1" ht="264" x14ac:dyDescent="0.25">
+      <c r="A12" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>119</v>
+      </c>
+      <c r="C12" s="10" t="s">
+        <v>120</v>
+      </c>
+      <c r="D12" s="10" t="s">
+        <v>121</v>
+      </c>
+      <c r="E12" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="F12" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="G7" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="I7" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="J7" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="K7" s="3" t="s">
-        <v>423</v>
-      </c>
-      <c r="L7" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="M7" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="N7" s="3" t="s">
-        <v>429</v>
-      </c>
-      <c r="O7" s="3" t="s">
-        <v>92</v>
+      <c r="G12" s="10" t="s">
+        <v>122</v>
+      </c>
+      <c r="H12" s="10" t="s">
+        <v>238</v>
+      </c>
+      <c r="I12" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="J12" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="K12" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="L12" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="M12" s="10" t="s">
+        <v>124</v>
+      </c>
+      <c r="N12" s="10" t="s">
+        <v>125</v>
+      </c>
+      <c r="O12" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="P12" s="11" t="s">
+        <v>436</v>
       </c>
     </row>
-    <row r="8" spans="1:16" s="4" customFormat="1" ht="184.8" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="F8" s="3" t="s">
+    <row r="13" spans="1:16" s="11" customFormat="1" ht="303.60000000000002" x14ac:dyDescent="0.25">
+      <c r="A13" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="C13" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="D13" s="10" t="s">
+        <v>129</v>
+      </c>
+      <c r="E13" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="F13" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="G8" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="H8" s="3" t="s">
-        <v>241</v>
-      </c>
-      <c r="I8" s="3" t="s">
+      <c r="G13" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="H13" s="10" t="s">
+        <v>238</v>
+      </c>
+      <c r="I13" s="10" t="s">
+        <v>244</v>
+      </c>
+      <c r="J13" s="10" t="s">
+        <v>130</v>
+      </c>
+      <c r="K13" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="L13" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="M13" s="10" t="s">
+        <v>439</v>
+      </c>
+      <c r="N13" s="10" t="s">
+        <v>438</v>
+      </c>
+      <c r="O13" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="P13" s="11" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" s="11" customFormat="1" ht="198" x14ac:dyDescent="0.25">
+      <c r="A14" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="C14" s="10" t="s">
+        <v>444</v>
+      </c>
+      <c r="D14" s="10" t="s">
+        <v>445</v>
+      </c>
+      <c r="E14" s="10" t="s">
+        <v>235</v>
+      </c>
+      <c r="F14" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="G14" s="10" t="s">
+        <v>246</v>
+      </c>
+      <c r="H14" s="10" t="s">
+        <v>310</v>
+      </c>
+      <c r="I14" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="J14" s="10" t="s">
+        <v>440</v>
+      </c>
+      <c r="K14" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="L14" s="10" t="s">
+        <v>133</v>
+      </c>
+      <c r="M14" s="10" t="s">
+        <v>441</v>
+      </c>
+      <c r="N14" s="10" t="s">
+        <v>442</v>
+      </c>
+      <c r="O14" s="10" t="s">
+        <v>134</v>
+      </c>
+      <c r="P14" s="11" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" s="11" customFormat="1" ht="290.39999999999998" x14ac:dyDescent="0.25">
+      <c r="A15" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>135</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>245</v>
+      </c>
+      <c r="D15" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="E15" s="10" t="s">
+        <v>235</v>
+      </c>
+      <c r="F15" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="G15" s="10" t="s">
+        <v>246</v>
+      </c>
+      <c r="H15" s="10" t="s">
+        <v>238</v>
+      </c>
+      <c r="I15" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="J15" s="10" t="s">
         <v>247</v>
       </c>
-      <c r="J8" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="K8" s="3" t="s">
+      <c r="K15" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="L8" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="M8" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="N8" s="3" t="s">
-        <v>429</v>
-      </c>
-      <c r="O8" s="3" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="9" spans="1:16" s="4" customFormat="1" ht="303.60000000000002" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>238</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="H9" s="3" t="s">
-        <v>418</v>
-      </c>
-      <c r="I9" s="3" t="s">
-        <v>247</v>
-      </c>
-      <c r="J9" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="K9" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="L9" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="M9" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="N9" s="3" t="s">
-        <v>429</v>
-      </c>
-      <c r="O9" s="3" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="10" spans="1:16" s="4" customFormat="1" ht="211.2" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="G10" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="H10" s="3" t="s">
-        <v>241</v>
-      </c>
-      <c r="I10" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="J10" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="K10" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="L10" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="M10" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="N10" s="3" t="s">
-        <v>429</v>
-      </c>
-      <c r="O10" s="3" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="11" spans="1:16" s="4" customFormat="1" ht="198" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="G11" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="H11" s="3" t="s">
-        <v>241</v>
-      </c>
-      <c r="I11" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="J11" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="K11" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="L11" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="M11" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="N11" s="3" t="s">
-        <v>429</v>
-      </c>
-      <c r="O11" s="3" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="12" spans="1:16" s="4" customFormat="1" ht="264" x14ac:dyDescent="0.25">
-      <c r="A12" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="G12" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="H12" s="3" t="s">
-        <v>241</v>
-      </c>
-      <c r="I12" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="J12" s="3" t="s">
-        <v>124</v>
-      </c>
-      <c r="K12" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="L12" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="M12" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="N12" s="3" t="s">
-        <v>126</v>
-      </c>
-      <c r="O12" s="3" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="13" spans="1:16" s="4" customFormat="1" ht="303.60000000000002" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="G13" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="H13" s="3" t="s">
-        <v>241</v>
-      </c>
-      <c r="I13" s="3" t="s">
-        <v>247</v>
-      </c>
-      <c r="J13" s="3" t="s">
-        <v>131</v>
-      </c>
-      <c r="K13" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="L13" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="M13" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="N13" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="O13" s="3" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="14" spans="1:16" s="4" customFormat="1" ht="198" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>238</v>
-      </c>
-      <c r="F14" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="G14" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="H14" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="I14" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="J14" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="K14" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="L14" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="M14" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="N14" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="O14" s="3" t="s">
+      <c r="L15" s="10" t="s">
+        <v>248</v>
+      </c>
+      <c r="M15" s="10" t="s">
+        <v>249</v>
+      </c>
+      <c r="N15" s="10" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="15" spans="1:16" s="4" customFormat="1" ht="290.39999999999998" x14ac:dyDescent="0.25">
-      <c r="A15" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B15" s="3" t="s">
+      <c r="O15" s="10" t="s">
         <v>138</v>
       </c>
-      <c r="C15" s="3" t="s">
-        <v>248</v>
-      </c>
-      <c r="D15" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="E15" s="3" t="s">
-        <v>238</v>
-      </c>
-      <c r="F15" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="G15" s="3" t="s">
-        <v>249</v>
-      </c>
-      <c r="H15" s="3" t="s">
-        <v>241</v>
-      </c>
-      <c r="I15" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="J15" s="3" t="s">
-        <v>250</v>
-      </c>
-      <c r="K15" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="L15" s="3" t="s">
-        <v>251</v>
-      </c>
-      <c r="M15" s="3" t="s">
-        <v>252</v>
-      </c>
-      <c r="N15" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="O15" s="3" t="s">
-        <v>141</v>
+      <c r="P15" s="11" t="s">
+        <v>443</v>
       </c>
     </row>
     <row r="16" spans="1:16" s="4" customFormat="1" ht="132" x14ac:dyDescent="0.25">
@@ -2809,49 +2885,49 @@
         <v>16</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="E16" s="3" t="s">
         <v>56</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="I16" s="3" t="s">
         <v>48</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="K16" s="3" t="s">
         <v>49</v>
       </c>
       <c r="L16" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="M16" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="N16" s="3" t="s">
         <v>222</v>
       </c>
-      <c r="M16" s="3" t="s">
-        <v>223</v>
-      </c>
-      <c r="N16" s="3" t="s">
-        <v>225</v>
-      </c>
       <c r="O16" s="3" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="P16" s="3" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
     </row>
     <row r="17" spans="1:16" s="4" customFormat="1" ht="379.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2859,43 +2935,43 @@
         <v>17</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>419</v>
+        <v>416</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="G17" s="3" t="s">
         <v>56</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>418</v>
+        <v>415</v>
       </c>
       <c r="I17" s="3" t="s">
         <v>48</v>
       </c>
       <c r="J17" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="K17" s="3" t="s">
+        <v>422</v>
+      </c>
+      <c r="L17" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="M17" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="N17" s="3" t="s">
         <v>145</v>
-      </c>
-      <c r="K17" s="3" t="s">
-        <v>425</v>
-      </c>
-      <c r="L17" s="3" t="s">
-        <v>146</v>
-      </c>
-      <c r="M17" s="3" t="s">
-        <v>147</v>
-      </c>
-      <c r="N17" s="3" t="s">
-        <v>148</v>
       </c>
       <c r="O17" s="3" t="s">
         <v>46</v>
@@ -2906,49 +2982,49 @@
         <v>18</v>
       </c>
       <c r="B18" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>397</v>
+      </c>
+      <c r="G18" s="3" t="s">
         <v>149</v>
       </c>
-      <c r="C18" s="3" t="s">
-        <v>150</v>
-      </c>
-      <c r="D18" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="E18" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="F18" s="3" t="s">
-        <v>400</v>
-      </c>
-      <c r="G18" s="3" t="s">
-        <v>152</v>
-      </c>
       <c r="H18" s="3" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="I18" s="3" t="s">
         <v>48</v>
       </c>
       <c r="J18" s="3" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="K18" s="3" t="s">
         <v>49</v>
       </c>
       <c r="L18" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="M18" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="N18" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="O18" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="P18" s="4" t="s">
         <v>154</v>
-      </c>
-      <c r="M18" s="3" t="s">
-        <v>155</v>
-      </c>
-      <c r="N18" s="3" t="s">
-        <v>156</v>
-      </c>
-      <c r="O18" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="P18" s="4" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="19" spans="1:16" s="4" customFormat="1" ht="409.6" x14ac:dyDescent="0.25">
@@ -2956,13 +3032,13 @@
         <v>19</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="E19" s="3" t="s">
         <v>56</v>
@@ -2980,7 +3056,7 @@
         <v>48</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="K19" s="3" t="s">
         <v>49</v>
@@ -2995,7 +3071,7 @@
         <v>46</v>
       </c>
       <c r="O19" s="3" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
     <row r="20" spans="1:16" s="4" customFormat="1" ht="132" x14ac:dyDescent="0.25">
@@ -3003,49 +3079,49 @@
         <v>20</v>
       </c>
       <c r="B20" s="3" t="s">
+        <v>224</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>417</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="G20" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="H20" s="3" t="s">
+        <v>238</v>
+      </c>
+      <c r="I20" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="J20" s="3" t="s">
         <v>227</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>228</v>
-      </c>
-      <c r="D20" s="3" t="s">
-        <v>229</v>
-      </c>
-      <c r="E20" s="3" t="s">
-        <v>420</v>
-      </c>
-      <c r="F20" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="G20" s="3" t="s">
-        <v>204</v>
-      </c>
-      <c r="H20" s="3" t="s">
-        <v>241</v>
-      </c>
-      <c r="I20" s="3" t="s">
-        <v>247</v>
-      </c>
-      <c r="J20" s="3" t="s">
-        <v>230</v>
       </c>
       <c r="K20" s="3" t="s">
         <v>49</v>
       </c>
       <c r="L20" s="3" t="s">
+        <v>228</v>
+      </c>
+      <c r="M20" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="N20" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="O20" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="P20" s="4" t="s">
         <v>231</v>
-      </c>
-      <c r="M20" s="3" t="s">
-        <v>232</v>
-      </c>
-      <c r="N20" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="O20" s="3" t="s">
-        <v>233</v>
-      </c>
-      <c r="P20" s="4" t="s">
-        <v>234</v>
       </c>
     </row>
     <row r="21" spans="1:16" s="4" customFormat="1" ht="189" customHeight="1" x14ac:dyDescent="0.25">
@@ -3053,49 +3129,49 @@
         <v>21</v>
       </c>
       <c r="B21" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>234</v>
+      </c>
+      <c r="D21" s="3" t="s">
         <v>236</v>
       </c>
-      <c r="C21" s="3" t="s">
-        <v>237</v>
-      </c>
-      <c r="D21" s="3" t="s">
-        <v>239</v>
-      </c>
       <c r="E21" s="3" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="F21" s="3" t="s">
         <v>62</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="I21" s="3" t="s">
         <v>48</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="K21" s="3" t="s">
         <v>50</v>
       </c>
       <c r="L21" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="M21" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="N21" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="O21" s="3" t="s">
         <v>242</v>
       </c>
-      <c r="M21" s="3" t="s">
+      <c r="P21" s="4" t="s">
         <v>243</v>
-      </c>
-      <c r="N21" s="3" t="s">
-        <v>244</v>
-      </c>
-      <c r="O21" s="3" t="s">
-        <v>245</v>
-      </c>
-      <c r="P21" s="4" t="s">
-        <v>246</v>
       </c>
     </row>
     <row r="22" spans="1:16" s="4" customFormat="1" ht="250.8" x14ac:dyDescent="0.25">
@@ -3103,31 +3179,31 @@
         <v>22</v>
       </c>
       <c r="B22" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="F22" s="3" t="s">
         <v>163</v>
       </c>
-      <c r="C22" s="3" t="s">
-        <v>164</v>
-      </c>
-      <c r="D22" s="3" t="s">
-        <v>165</v>
-      </c>
-      <c r="E22" s="3" t="s">
+      <c r="G22" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="H22" s="3" t="s">
         <v>238</v>
-      </c>
-      <c r="F22" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="G22" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="H22" s="3" t="s">
-        <v>241</v>
       </c>
       <c r="I22" s="3" t="s">
         <v>47</v>
       </c>
       <c r="J22" s="3" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="K22" s="3" t="s">
         <v>49</v>
@@ -3136,64 +3212,64 @@
         <v>46</v>
       </c>
       <c r="M22" s="3" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="N22" s="3"/>
       <c r="O22" s="3" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="P22" s="3" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
     </row>
     <row r="23" spans="1:16" s="4" customFormat="1" ht="145.19999999999999" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="D23" s="3" t="s">
         <v>253</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="E23" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="F23" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="G23" s="3" t="s">
         <v>254</v>
       </c>
-      <c r="C23" s="3" t="s">
+      <c r="H23" s="3" t="s">
+        <v>419</v>
+      </c>
+      <c r="I23" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="J23" s="3" t="s">
         <v>255</v>
       </c>
-      <c r="D23" s="3" t="s">
+      <c r="K23" s="3" t="s">
+        <v>399</v>
+      </c>
+      <c r="L23" s="3" t="s">
         <v>256</v>
       </c>
-      <c r="E23" s="3" t="s">
-        <v>238</v>
-      </c>
-      <c r="F23" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="G23" s="3" t="s">
+      <c r="M23" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="N23" s="3" t="s">
+        <v>259</v>
+      </c>
+      <c r="O23" s="3" t="s">
         <v>257</v>
       </c>
-      <c r="H23" s="3" t="s">
-        <v>422</v>
-      </c>
-      <c r="I23" s="3" t="s">
-        <v>247</v>
-      </c>
-      <c r="J23" s="3" t="s">
+      <c r="P23" s="4" t="s">
         <v>258</v>
-      </c>
-      <c r="K23" s="3" t="s">
-        <v>402</v>
-      </c>
-      <c r="L23" s="3" t="s">
-        <v>259</v>
-      </c>
-      <c r="M23" s="3" t="s">
-        <v>263</v>
-      </c>
-      <c r="N23" s="3" t="s">
-        <v>262</v>
-      </c>
-      <c r="O23" s="3" t="s">
-        <v>260</v>
-      </c>
-      <c r="P23" s="4" t="s">
-        <v>261</v>
       </c>
     </row>
     <row r="24" spans="1:16" s="4" customFormat="1" ht="118.8" x14ac:dyDescent="0.25">
@@ -3201,49 +3277,49 @@
         <v>23</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="F24" s="3" t="s">
         <v>62</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="H24" s="3" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="I24" s="3" t="s">
         <v>48</v>
       </c>
       <c r="J24" s="3" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="K24" s="3" t="s">
         <v>50</v>
       </c>
       <c r="L24" s="3" t="s">
+        <v>265</v>
+      </c>
+      <c r="M24" s="3" t="s">
+        <v>266</v>
+      </c>
+      <c r="N24" s="3" t="s">
+        <v>267</v>
+      </c>
+      <c r="O24" s="3" t="s">
         <v>268</v>
       </c>
-      <c r="M24" s="3" t="s">
+      <c r="P24" s="4" t="s">
         <v>269</v>
-      </c>
-      <c r="N24" s="3" t="s">
-        <v>270</v>
-      </c>
-      <c r="O24" s="3" t="s">
-        <v>271</v>
-      </c>
-      <c r="P24" s="4" t="s">
-        <v>272</v>
       </c>
     </row>
     <row r="25" spans="1:16" s="4" customFormat="1" ht="184.8" x14ac:dyDescent="0.25">
@@ -3251,25 +3327,25 @@
         <v>24</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F25" s="3" t="s">
         <v>62</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="I25" s="3" t="s">
         <v>48</v>
@@ -3288,7 +3364,7 @@
       </c>
       <c r="N25" s="3"/>
       <c r="O25" s="3" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="26" spans="1:16" s="4" customFormat="1" ht="132" x14ac:dyDescent="0.25">
@@ -3296,25 +3372,25 @@
         <v>25</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>419</v>
+        <v>416</v>
       </c>
       <c r="F26" s="3" t="s">
         <v>62</v>
       </c>
       <c r="G26" s="3" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="H26" s="3" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="I26" s="3" t="s">
         <v>48</v>
@@ -3326,19 +3402,19 @@
         <v>49</v>
       </c>
       <c r="L26" s="3" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="M26" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="N26" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="O26" s="3" t="s">
+        <v>290</v>
+      </c>
+      <c r="P26" s="4" t="s">
         <v>292</v>
-      </c>
-      <c r="N26" s="3" t="s">
-        <v>296</v>
-      </c>
-      <c r="O26" s="3" t="s">
-        <v>293</v>
-      </c>
-      <c r="P26" s="4" t="s">
-        <v>295</v>
       </c>
     </row>
     <row r="27" spans="1:16" s="4" customFormat="1" ht="224.4" x14ac:dyDescent="0.25">
@@ -3346,46 +3422,46 @@
         <v>26</v>
       </c>
       <c r="B27" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="F27" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="G27" s="3" t="s">
         <v>175</v>
       </c>
-      <c r="C27" s="3" t="s">
+      <c r="H27" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="I27" s="3" t="s">
+        <v>424</v>
+      </c>
+      <c r="J27" s="3" t="s">
         <v>176</v>
-      </c>
-      <c r="D27" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="E27" s="3" t="s">
-        <v>419</v>
-      </c>
-      <c r="F27" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="G27" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="H27" s="3" t="s">
-        <v>290</v>
-      </c>
-      <c r="I27" s="3" t="s">
-        <v>427</v>
-      </c>
-      <c r="J27" s="3" t="s">
-        <v>179</v>
       </c>
       <c r="K27" s="3" t="s">
         <v>50</v>
       </c>
       <c r="L27" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="M27" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="N27" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="O27" s="3" t="s">
         <v>180</v>
-      </c>
-      <c r="M27" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="N27" s="3" t="s">
-        <v>182</v>
-      </c>
-      <c r="O27" s="3" t="s">
-        <v>183</v>
       </c>
     </row>
     <row r="28" spans="1:16" s="4" customFormat="1" ht="409.6" x14ac:dyDescent="0.25">
@@ -3393,49 +3469,49 @@
         <v>27</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="F28" s="3" t="s">
         <v>62</v>
       </c>
       <c r="G28" s="3" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="H28" s="3" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="I28" s="3" t="s">
         <v>48</v>
       </c>
       <c r="J28" s="3" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="K28" s="3" t="s">
         <v>49</v>
       </c>
       <c r="L28" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="M28" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="N28" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="O28" s="3" t="s">
         <v>189</v>
       </c>
-      <c r="M28" s="3" t="s">
+      <c r="P28" s="4" t="s">
         <v>190</v>
-      </c>
-      <c r="N28" s="3" t="s">
-        <v>191</v>
-      </c>
-      <c r="O28" s="3" t="s">
-        <v>192</v>
-      </c>
-      <c r="P28" s="4" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="29" spans="1:16" s="4" customFormat="1" ht="250.8" x14ac:dyDescent="0.25">
@@ -3443,49 +3519,49 @@
         <v>28</v>
       </c>
       <c r="B29" s="3" t="s">
+        <v>197</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>198</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="E29" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="F29" s="3" t="s">
         <v>200</v>
       </c>
-      <c r="C29" s="3" t="s">
+      <c r="G29" s="3" t="s">
         <v>201</v>
       </c>
-      <c r="D29" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="E29" s="3" t="s">
+      <c r="H29" s="3" t="s">
         <v>238</v>
-      </c>
-      <c r="F29" s="3" t="s">
-        <v>203</v>
-      </c>
-      <c r="G29" s="3" t="s">
-        <v>204</v>
-      </c>
-      <c r="H29" s="3" t="s">
-        <v>241</v>
       </c>
       <c r="I29" s="3" t="s">
         <v>48</v>
       </c>
       <c r="J29" s="3" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="K29" s="3" t="s">
         <v>49</v>
       </c>
       <c r="L29" s="3" t="s">
+        <v>203</v>
+      </c>
+      <c r="M29" s="5" t="s">
+        <v>271</v>
+      </c>
+      <c r="N29" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="O29" s="3" t="s">
         <v>206</v>
       </c>
-      <c r="M29" s="5" t="s">
-        <v>274</v>
-      </c>
-      <c r="N29" s="3" t="s">
-        <v>207</v>
-      </c>
-      <c r="O29" s="3" t="s">
-        <v>209</v>
-      </c>
       <c r="P29" s="4" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
     </row>
     <row r="30" spans="1:16" s="4" customFormat="1" ht="132" x14ac:dyDescent="0.25">
@@ -3493,13 +3569,13 @@
         <v>29</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="E30" s="3" t="s">
         <v>56</v>
@@ -3508,34 +3584,34 @@
         <v>62</v>
       </c>
       <c r="G30" s="3" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="H30" s="3" t="s">
-        <v>344</v>
+        <v>341</v>
       </c>
       <c r="I30" s="3" t="s">
         <v>48</v>
       </c>
       <c r="J30" s="3" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="K30" s="3" t="s">
         <v>50</v>
       </c>
       <c r="L30" s="3" t="s">
+        <v>210</v>
+      </c>
+      <c r="M30" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="N30" s="3" t="s">
+        <v>212</v>
+      </c>
+      <c r="O30" s="3" t="s">
+        <v>214</v>
+      </c>
+      <c r="P30" s="3" t="s">
         <v>213</v>
-      </c>
-      <c r="M30" s="3" t="s">
-        <v>214</v>
-      </c>
-      <c r="N30" s="3" t="s">
-        <v>215</v>
-      </c>
-      <c r="O30" s="3" t="s">
-        <v>217</v>
-      </c>
-      <c r="P30" s="3" t="s">
-        <v>216</v>
       </c>
     </row>
     <row r="31" spans="1:16" s="4" customFormat="1" ht="105.6" x14ac:dyDescent="0.25">
@@ -3543,49 +3619,49 @@
         <v>30</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="C31" s="3" t="s">
+        <v>273</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>274</v>
+      </c>
+      <c r="E31" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="F31" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="G31" s="3" t="s">
         <v>276</v>
       </c>
-      <c r="D31" s="3" t="s">
+      <c r="H31" s="3" t="s">
         <v>277</v>
-      </c>
-      <c r="E31" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="F31" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="G31" s="3" t="s">
-        <v>279</v>
-      </c>
-      <c r="H31" s="3" t="s">
-        <v>280</v>
       </c>
       <c r="I31" s="3" t="s">
         <v>48</v>
       </c>
       <c r="J31" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="K31" s="3" t="s">
+        <v>423</v>
+      </c>
+      <c r="L31" s="3" t="s">
+        <v>279</v>
+      </c>
+      <c r="M31" s="3" t="s">
+        <v>280</v>
+      </c>
+      <c r="N31" s="3" t="s">
         <v>281</v>
       </c>
-      <c r="K31" s="3" t="s">
-        <v>426</v>
-      </c>
-      <c r="L31" s="3" t="s">
+      <c r="O31" s="3" t="s">
         <v>282</v>
       </c>
-      <c r="M31" s="3" t="s">
+      <c r="P31" s="4" t="s">
         <v>283</v>
-      </c>
-      <c r="N31" s="3" t="s">
-        <v>284</v>
-      </c>
-      <c r="O31" s="3" t="s">
-        <v>285</v>
-      </c>
-      <c r="P31" s="4" t="s">
-        <v>286</v>
       </c>
     </row>
     <row r="32" spans="1:16" s="4" customFormat="1" ht="290.39999999999998" x14ac:dyDescent="0.25">
@@ -3593,13 +3669,13 @@
         <v>31</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="E32" s="3" t="s">
         <v>56</v>
@@ -3608,28 +3684,28 @@
         <v>62</v>
       </c>
       <c r="G32" s="3" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="H32" s="3" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="I32" s="3" t="s">
         <v>48</v>
       </c>
       <c r="J32" s="3" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="K32" s="3" t="s">
         <v>50</v>
       </c>
       <c r="L32" s="3" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="M32" s="3" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="N32" s="3" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="O32" s="3"/>
     </row>
@@ -3638,49 +3714,49 @@
         <v>32</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="F33" s="3" t="s">
         <v>62</v>
       </c>
       <c r="G33" s="3" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="H33" s="3" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="I33" s="3" t="s">
-        <v>428</v>
+        <v>425</v>
       </c>
       <c r="J33" s="3" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="K33" s="3" t="s">
         <v>49</v>
       </c>
       <c r="L33" s="3" t="s">
+        <v>301</v>
+      </c>
+      <c r="M33" s="3" t="s">
+        <v>302</v>
+      </c>
+      <c r="N33" s="3" t="s">
+        <v>303</v>
+      </c>
+      <c r="O33" s="3" t="s">
         <v>304</v>
       </c>
-      <c r="M33" s="3" t="s">
+      <c r="P33" s="4" t="s">
         <v>305</v>
-      </c>
-      <c r="N33" s="3" t="s">
-        <v>306</v>
-      </c>
-      <c r="O33" s="3" t="s">
-        <v>307</v>
-      </c>
-      <c r="P33" s="4" t="s">
-        <v>308</v>
       </c>
     </row>
     <row r="34" spans="1:16" s="4" customFormat="1" ht="79.2" x14ac:dyDescent="0.25">
@@ -3688,49 +3764,49 @@
         <v>33</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="C34" s="3" t="s">
+        <v>307</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>308</v>
+      </c>
+      <c r="E34" s="6" t="s">
+        <v>235</v>
+      </c>
+      <c r="F34" s="3" t="s">
+        <v>398</v>
+      </c>
+      <c r="G34" s="3" t="s">
+        <v>298</v>
+      </c>
+      <c r="H34" s="3" t="s">
         <v>310</v>
       </c>
-      <c r="D34" s="3" t="s">
+      <c r="I34" s="3" t="s">
+        <v>425</v>
+      </c>
+      <c r="J34" s="3" t="s">
         <v>311</v>
-      </c>
-      <c r="E34" s="6" t="s">
-        <v>238</v>
-      </c>
-      <c r="F34" s="3" t="s">
-        <v>401</v>
-      </c>
-      <c r="G34" s="3" t="s">
-        <v>301</v>
-      </c>
-      <c r="H34" s="3" t="s">
-        <v>313</v>
-      </c>
-      <c r="I34" s="3" t="s">
-        <v>428</v>
-      </c>
-      <c r="J34" s="3" t="s">
-        <v>314</v>
       </c>
       <c r="K34" s="3" t="s">
         <v>49</v>
       </c>
       <c r="L34" s="3" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="M34" s="3" t="s">
+        <v>312</v>
+      </c>
+      <c r="N34" s="3" t="s">
+        <v>313</v>
+      </c>
+      <c r="O34" s="3" t="s">
+        <v>314</v>
+      </c>
+      <c r="P34" s="4" t="s">
         <v>315</v>
-      </c>
-      <c r="N34" s="3" t="s">
-        <v>316</v>
-      </c>
-      <c r="O34" s="3" t="s">
-        <v>317</v>
-      </c>
-      <c r="P34" s="4" t="s">
-        <v>318</v>
       </c>
     </row>
     <row r="35" spans="1:16" s="4" customFormat="1" ht="92.4" x14ac:dyDescent="0.25">
@@ -3738,49 +3814,49 @@
         <v>34</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
       <c r="E35" s="3" t="s">
         <v>56</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="G35" s="3" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="H35" s="3" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="I35" s="3" t="s">
         <v>48</v>
       </c>
       <c r="J35" s="3" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="K35" s="3" t="s">
         <v>49</v>
       </c>
       <c r="L35" s="3" t="s">
+        <v>320</v>
+      </c>
+      <c r="M35" s="3" t="s">
+        <v>321</v>
+      </c>
+      <c r="N35" s="3" t="s">
+        <v>322</v>
+      </c>
+      <c r="O35" s="3" t="s">
         <v>323</v>
       </c>
-      <c r="M35" s="3" t="s">
+      <c r="P35" s="4" t="s">
         <v>324</v>
-      </c>
-      <c r="N35" s="3" t="s">
-        <v>325</v>
-      </c>
-      <c r="O35" s="3" t="s">
-        <v>326</v>
-      </c>
-      <c r="P35" s="4" t="s">
-        <v>327</v>
       </c>
     </row>
     <row r="36" spans="1:16" s="4" customFormat="1" ht="79.2" x14ac:dyDescent="0.25">
@@ -3788,49 +3864,49 @@
         <v>35</v>
       </c>
       <c r="B36" s="3" t="s">
+        <v>325</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>326</v>
+      </c>
+      <c r="D36" s="3" t="s">
+        <v>327</v>
+      </c>
+      <c r="E36" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="F36" s="3" t="s">
+        <v>329</v>
+      </c>
+      <c r="G36" s="3" t="s">
         <v>328</v>
       </c>
-      <c r="C36" s="3" t="s">
-        <v>329</v>
-      </c>
-      <c r="D36" s="3" t="s">
+      <c r="H36" s="3" t="s">
+        <v>238</v>
+      </c>
+      <c r="I36" s="3" t="s">
+        <v>425</v>
+      </c>
+      <c r="J36" s="3" t="s">
         <v>330</v>
-      </c>
-      <c r="E36" s="3" t="s">
-        <v>238</v>
-      </c>
-      <c r="F36" s="3" t="s">
-        <v>332</v>
-      </c>
-      <c r="G36" s="3" t="s">
-        <v>331</v>
-      </c>
-      <c r="H36" s="3" t="s">
-        <v>241</v>
-      </c>
-      <c r="I36" s="3" t="s">
-        <v>428</v>
-      </c>
-      <c r="J36" s="3" t="s">
-        <v>333</v>
       </c>
       <c r="K36" s="3" t="s">
         <v>64</v>
       </c>
       <c r="L36" s="3" t="s">
+        <v>331</v>
+      </c>
+      <c r="M36" s="3" t="s">
+        <v>332</v>
+      </c>
+      <c r="N36" s="3" t="s">
+        <v>333</v>
+      </c>
+      <c r="O36" s="3" t="s">
         <v>334</v>
       </c>
-      <c r="M36" s="3" t="s">
+      <c r="P36" s="4" t="s">
         <v>335</v>
-      </c>
-      <c r="N36" s="3" t="s">
-        <v>336</v>
-      </c>
-      <c r="O36" s="3" t="s">
-        <v>337</v>
-      </c>
-      <c r="P36" s="4" t="s">
-        <v>338</v>
       </c>
     </row>
     <row r="37" spans="1:16" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -3883,49 +3959,49 @@
         <v>37</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="C38" s="3" t="s">
+        <v>337</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>338</v>
+      </c>
+      <c r="E38" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="F38" s="3" t="s">
         <v>340</v>
       </c>
-      <c r="D38" s="3" t="s">
+      <c r="G38" s="3" t="s">
+        <v>298</v>
+      </c>
+      <c r="H38" s="3" t="s">
         <v>341</v>
-      </c>
-      <c r="E38" s="3" t="s">
-        <v>238</v>
-      </c>
-      <c r="F38" s="3" t="s">
-        <v>343</v>
-      </c>
-      <c r="G38" s="3" t="s">
-        <v>301</v>
-      </c>
-      <c r="H38" s="3" t="s">
-        <v>344</v>
       </c>
       <c r="I38" s="3" t="s">
         <v>48</v>
       </c>
       <c r="J38" s="3" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="K38" s="3" t="s">
         <v>49</v>
       </c>
       <c r="L38" s="3" t="s">
+        <v>342</v>
+      </c>
+      <c r="M38" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="N38" s="3" t="s">
+        <v>322</v>
+      </c>
+      <c r="O38" s="3" t="s">
+        <v>344</v>
+      </c>
+      <c r="P38" s="4" t="s">
         <v>345</v>
-      </c>
-      <c r="M38" s="3" t="s">
-        <v>346</v>
-      </c>
-      <c r="N38" s="3" t="s">
-        <v>325</v>
-      </c>
-      <c r="O38" s="3" t="s">
-        <v>347</v>
-      </c>
-      <c r="P38" s="4" t="s">
-        <v>348</v>
       </c>
     </row>
     <row r="39" spans="1:16" s="4" customFormat="1" ht="132" x14ac:dyDescent="0.25">
@@ -3933,49 +4009,49 @@
         <v>38</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="E39" s="3" t="s">
         <v>56</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
       <c r="G39" s="3" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="H39" s="3" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="I39" s="3" t="s">
         <v>48</v>
       </c>
       <c r="J39" s="3" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
       <c r="K39" s="3" t="s">
         <v>49</v>
       </c>
       <c r="L39" s="3" t="s">
-        <v>345</v>
+        <v>342</v>
       </c>
       <c r="M39" s="3" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
       <c r="N39" s="3" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="O39" s="3" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
       <c r="P39" s="4" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
     </row>
     <row r="40" spans="1:16" s="4" customFormat="1" ht="145.19999999999999" x14ac:dyDescent="0.25">
@@ -3983,49 +4059,49 @@
         <v>39</v>
       </c>
       <c r="B40" s="3" t="s">
+        <v>352</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>353</v>
+      </c>
+      <c r="D40" s="3" t="s">
+        <v>354</v>
+      </c>
+      <c r="E40" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="F40" s="3" t="s">
         <v>355</v>
       </c>
-      <c r="C40" s="3" t="s">
+      <c r="G40" s="3" t="s">
+        <v>298</v>
+      </c>
+      <c r="H40" s="3" t="s">
+        <v>238</v>
+      </c>
+      <c r="I40" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="J40" s="3" t="s">
         <v>356</v>
-      </c>
-      <c r="D40" s="3" t="s">
-        <v>357</v>
-      </c>
-      <c r="E40" s="3" t="s">
-        <v>419</v>
-      </c>
-      <c r="F40" s="3" t="s">
-        <v>358</v>
-      </c>
-      <c r="G40" s="3" t="s">
-        <v>301</v>
-      </c>
-      <c r="H40" s="3" t="s">
-        <v>241</v>
-      </c>
-      <c r="I40" s="3" t="s">
-        <v>247</v>
-      </c>
-      <c r="J40" s="3" t="s">
-        <v>359</v>
       </c>
       <c r="K40" s="3" t="s">
         <v>49</v>
       </c>
       <c r="L40" s="3" t="s">
+        <v>357</v>
+      </c>
+      <c r="M40" s="3" t="s">
+        <v>358</v>
+      </c>
+      <c r="N40" s="3" t="s">
+        <v>359</v>
+      </c>
+      <c r="O40" s="3" t="s">
         <v>360</v>
       </c>
-      <c r="M40" s="3" t="s">
+      <c r="P40" s="4" t="s">
         <v>361</v>
-      </c>
-      <c r="N40" s="3" t="s">
-        <v>362</v>
-      </c>
-      <c r="O40" s="3" t="s">
-        <v>363</v>
-      </c>
-      <c r="P40" s="4" t="s">
-        <v>364</v>
       </c>
     </row>
     <row r="41" spans="1:16" s="4" customFormat="1" ht="118.8" x14ac:dyDescent="0.25">
@@ -4033,49 +4109,49 @@
         <v>40</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="E41" s="3" t="s">
         <v>56</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
       <c r="G41" s="3" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="H41" s="3" t="s">
-        <v>344</v>
+        <v>341</v>
       </c>
       <c r="I41" s="3" t="s">
         <v>48</v>
       </c>
       <c r="J41" s="3" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="K41" s="3" t="s">
         <v>49</v>
       </c>
       <c r="L41" s="3" t="s">
-        <v>345</v>
+        <v>342</v>
       </c>
       <c r="M41" s="3" t="s">
+        <v>365</v>
+      </c>
+      <c r="N41" s="3" t="s">
+        <v>366</v>
+      </c>
+      <c r="O41" s="3" t="s">
+        <v>367</v>
+      </c>
+      <c r="P41" s="4" t="s">
         <v>368</v>
-      </c>
-      <c r="N41" s="3" t="s">
-        <v>369</v>
-      </c>
-      <c r="O41" s="3" t="s">
-        <v>370</v>
-      </c>
-      <c r="P41" s="4" t="s">
-        <v>371</v>
       </c>
     </row>
     <row r="42" spans="1:16" s="4" customFormat="1" ht="145.19999999999999" x14ac:dyDescent="0.25">
@@ -4083,49 +4159,49 @@
         <v>41</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="E42" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="F42" s="3" t="s">
+        <v>340</v>
+      </c>
+      <c r="G42" s="3" t="s">
+        <v>339</v>
+      </c>
+      <c r="H42" s="3" t="s">
         <v>238</v>
-      </c>
-      <c r="F42" s="3" t="s">
-        <v>343</v>
-      </c>
-      <c r="G42" s="3" t="s">
-        <v>342</v>
-      </c>
-      <c r="H42" s="3" t="s">
-        <v>241</v>
       </c>
       <c r="I42" s="3" t="s">
         <v>48</v>
       </c>
       <c r="J42" s="3" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
       <c r="K42" s="3" t="s">
         <v>49</v>
       </c>
       <c r="L42" s="3" t="s">
+        <v>373</v>
+      </c>
+      <c r="M42" s="3" t="s">
+        <v>374</v>
+      </c>
+      <c r="N42" s="3" t="s">
+        <v>375</v>
+      </c>
+      <c r="O42" s="3" t="s">
         <v>376</v>
       </c>
-      <c r="M42" s="3" t="s">
+      <c r="P42" s="4" t="s">
         <v>377</v>
-      </c>
-      <c r="N42" s="3" t="s">
-        <v>378</v>
-      </c>
-      <c r="O42" s="3" t="s">
-        <v>379</v>
-      </c>
-      <c r="P42" s="4" t="s">
-        <v>380</v>
       </c>
     </row>
     <row r="43" spans="1:16" s="4" customFormat="1" ht="145.19999999999999" x14ac:dyDescent="0.25">
@@ -4133,49 +4209,49 @@
         <v>42</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>381</v>
+        <v>378</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
       <c r="E43" s="3" t="s">
         <v>56</v>
       </c>
       <c r="F43" s="3" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
       <c r="G43" s="3" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="H43" s="3" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="I43" s="3" t="s">
         <v>48</v>
       </c>
       <c r="J43" s="3" t="s">
-        <v>384</v>
+        <v>381</v>
       </c>
       <c r="K43" s="3" t="s">
         <v>49</v>
       </c>
       <c r="L43" s="3" t="s">
+        <v>382</v>
+      </c>
+      <c r="M43" s="3" t="s">
+        <v>383</v>
+      </c>
+      <c r="N43" s="3" t="s">
+        <v>384</v>
+      </c>
+      <c r="O43" s="3" t="s">
         <v>385</v>
       </c>
-      <c r="M43" s="3" t="s">
+      <c r="P43" s="4" t="s">
         <v>386</v>
-      </c>
-      <c r="N43" s="3" t="s">
-        <v>387</v>
-      </c>
-      <c r="O43" s="3" t="s">
-        <v>388</v>
-      </c>
-      <c r="P43" s="4" t="s">
-        <v>389</v>
       </c>
     </row>
     <row r="44" spans="1:16" s="4" customFormat="1" ht="171.6" x14ac:dyDescent="0.25">
@@ -4183,49 +4259,49 @@
         <v>43</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>391</v>
+        <v>388</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>399</v>
+        <v>396</v>
       </c>
       <c r="E44" s="3" t="s">
         <v>56</v>
       </c>
       <c r="F44" s="3" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
       <c r="G44" s="3" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="H44" s="3" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="I44" s="3" t="s">
         <v>48</v>
       </c>
       <c r="J44" s="3" t="s">
+        <v>390</v>
+      </c>
+      <c r="K44" s="3" t="s">
+        <v>421</v>
+      </c>
+      <c r="L44" s="3" t="s">
+        <v>391</v>
+      </c>
+      <c r="M44" s="3" t="s">
+        <v>392</v>
+      </c>
+      <c r="N44" s="3" t="s">
         <v>393</v>
       </c>
-      <c r="K44" s="3" t="s">
-        <v>424</v>
-      </c>
-      <c r="L44" s="3" t="s">
+      <c r="O44" s="3" t="s">
         <v>394</v>
       </c>
-      <c r="M44" s="3" t="s">
+      <c r="P44" s="4" t="s">
         <v>395</v>
-      </c>
-      <c r="N44" s="3" t="s">
-        <v>396</v>
-      </c>
-      <c r="O44" s="3" t="s">
-        <v>397</v>
-      </c>
-      <c r="P44" s="4" t="s">
-        <v>398</v>
       </c>
     </row>
     <row r="45" spans="1:16" ht="145.19999999999999" x14ac:dyDescent="0.25">
@@ -4233,49 +4309,49 @@
         <v>44</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="E45" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="F45" s="3" t="s">
+        <v>340</v>
+      </c>
+      <c r="G45" s="3" t="s">
+        <v>339</v>
+      </c>
+      <c r="H45" s="3" t="s">
         <v>238</v>
-      </c>
-      <c r="F45" s="3" t="s">
-        <v>343</v>
-      </c>
-      <c r="G45" s="3" t="s">
-        <v>342</v>
-      </c>
-      <c r="H45" s="3" t="s">
-        <v>241</v>
       </c>
       <c r="I45" s="3" t="s">
         <v>48</v>
       </c>
       <c r="J45" s="3" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
       <c r="K45" s="3" t="s">
         <v>49</v>
       </c>
       <c r="L45" s="3" t="s">
+        <v>373</v>
+      </c>
+      <c r="M45" s="3" t="s">
+        <v>374</v>
+      </c>
+      <c r="N45" s="3" t="s">
+        <v>375</v>
+      </c>
+      <c r="O45" s="3" t="s">
         <v>376</v>
       </c>
-      <c r="M45" s="3" t="s">
+      <c r="P45" s="4" t="s">
         <v>377</v>
-      </c>
-      <c r="N45" s="3" t="s">
-        <v>378</v>
-      </c>
-      <c r="O45" s="3" t="s">
-        <v>379</v>
-      </c>
-      <c r="P45" s="4" t="s">
-        <v>380</v>
       </c>
     </row>
   </sheetData>
@@ -4285,18 +4361,18 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4444,18 +4520,18 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24F2579D-323E-48EA-8FED-D372AFFF0A04}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1160EB8C-E200-4916-A3B3-9BF8115D37F8}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1160EB8C-E200-4916-A3B3-9BF8115D37F8}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24F2579D-323E-48EA-8FED-D372AFFF0A04}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Update Individual Annotations files and remove unnecessary Zone.Identifier
</commit_message>
<xml_diff>
--- a/main/05_data_charting/data/Individual_Annotations.xlsx
+++ b/main/05_data_charting/data/Individual_Annotations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\orincon\scoping-ml-wave-seismology\main\05_data_charting\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F30138CE-47E9-48E1-80CA-8EEDE41C96CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1600E499-A9C5-4B50-B485-0BE916B41CF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{115BB8D9-8B86-4726-97F8-E06477FD353D}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="710" uniqueCount="446">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="712" uniqueCount="450">
   <si>
     <t>Research gaps</t>
   </si>
@@ -1112,9 +1112,6 @@
     <t> Extend to more realistic velocity models and acquisition setups.</t>
   </si>
   <si>
-    <t xml:space="preserve"> </t>
-  </si>
-  <si>
     <t>Visual comparison: RTM images vs surrogate predictions.</t>
   </si>
   <si>
@@ -1628,6 +1625,21 @@
   </si>
   <si>
     <t>It has fewer parameters and thus is more efficient than DNNs.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Only 2D acoustic cases are tested; scalability to 3D and elastic physics remains future work.</t>
+  </si>
+  <si>
+    <t>Agreement of dispersion curves and consistency of phase-velocity maps</t>
+  </si>
+  <si>
+    <t> Single-mode assumption</t>
+  </si>
+  <si>
+    <t>Relative error and comparison of reconstructed velocity models</t>
+  </si>
+  <si>
+    <t> Estimation of subsurface velocity fields from wavefield data.</t>
   </si>
 </sst>
 </file>
@@ -2132,52 +2144,52 @@
   <sheetData>
     <row r="1" spans="1:16" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
+        <v>400</v>
+      </c>
+      <c r="B1" s="8" t="s">
         <v>401</v>
-      </c>
-      <c r="B1" s="8" t="s">
-        <v>402</v>
       </c>
       <c r="C1" s="9" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="9" t="s">
+        <v>402</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>404</v>
+      </c>
+      <c r="F1" s="9" t="s">
         <v>403</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="G1" s="9" t="s">
         <v>405</v>
       </c>
-      <c r="F1" s="9" t="s">
-        <v>404</v>
-      </c>
-      <c r="G1" s="9" t="s">
+      <c r="H1" s="9" t="s">
         <v>406</v>
       </c>
-      <c r="H1" s="9" t="s">
+      <c r="I1" s="9" t="s">
         <v>407</v>
       </c>
-      <c r="I1" s="9" t="s">
+      <c r="J1" s="9" t="s">
         <v>408</v>
       </c>
-      <c r="J1" s="9" t="s">
+      <c r="K1" s="9" t="s">
         <v>409</v>
       </c>
-      <c r="K1" s="9" t="s">
+      <c r="L1" s="9" t="s">
         <v>410</v>
       </c>
-      <c r="L1" s="9" t="s">
+      <c r="M1" s="8" t="s">
         <v>411</v>
       </c>
-      <c r="M1" s="8" t="s">
+      <c r="N1" s="8" t="s">
         <v>412</v>
-      </c>
-      <c r="N1" s="8" t="s">
-        <v>413</v>
       </c>
       <c r="O1" s="8" t="s">
         <v>0</v>
       </c>
       <c r="P1" s="7" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
     </row>
     <row r="2" spans="1:16" s="11" customFormat="1" ht="250.8" x14ac:dyDescent="0.25">
@@ -2194,7 +2206,7 @@
         <v>53</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="F2" s="10" t="s">
         <v>62</v>
@@ -2221,7 +2233,7 @@
         <v>57</v>
       </c>
       <c r="N2" s="10" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="O2" s="10" t="s">
         <v>58</v>
@@ -2244,7 +2256,7 @@
         <v>61</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F3" s="10" t="s">
         <v>62</v>
@@ -2268,16 +2280,16 @@
         <v>65</v>
       </c>
       <c r="M3" s="10" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="N3" s="10" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="O3" s="10" t="s">
         <v>66</v>
       </c>
       <c r="P3" s="11" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="4" spans="1:16" s="11" customFormat="1" ht="201" customHeight="1" x14ac:dyDescent="0.25">
@@ -2327,7 +2339,7 @@
         <v>71</v>
       </c>
       <c r="P4" s="11" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
     </row>
     <row r="5" spans="1:16" s="11" customFormat="1" ht="210" customHeight="1" x14ac:dyDescent="0.25">
@@ -2371,13 +2383,13 @@
         <v>75</v>
       </c>
       <c r="N5" s="10" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="O5" s="10" t="s">
         <v>76</v>
       </c>
       <c r="P5" s="11" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="6" spans="1:16" s="11" customFormat="1" ht="250.8" x14ac:dyDescent="0.25">
@@ -2421,13 +2433,13 @@
         <v>83</v>
       </c>
       <c r="N6" s="10" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="O6" s="10" t="s">
         <v>84</v>
       </c>
       <c r="P6" s="11" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="7" spans="1:16" s="11" customFormat="1" ht="250.8" x14ac:dyDescent="0.25">
@@ -2462,7 +2474,7 @@
         <v>89</v>
       </c>
       <c r="K7" s="10" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="L7" s="10" t="s">
         <v>90</v>
@@ -2471,13 +2483,13 @@
         <v>91</v>
       </c>
       <c r="N7" s="10" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="O7" s="10" t="s">
         <v>92</v>
       </c>
       <c r="P7" s="11" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="8" spans="1:16" s="11" customFormat="1" ht="184.8" x14ac:dyDescent="0.25">
@@ -2521,13 +2533,13 @@
         <v>98</v>
       </c>
       <c r="N8" s="10" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="O8" s="10" t="s">
         <v>99</v>
       </c>
       <c r="P8" s="11" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
     </row>
     <row r="9" spans="1:16" s="11" customFormat="1" ht="303.60000000000002" x14ac:dyDescent="0.25">
@@ -2553,7 +2565,7 @@
         <v>56</v>
       </c>
       <c r="H9" s="10" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="I9" s="10" t="s">
         <v>244</v>
@@ -2571,13 +2583,13 @@
         <v>105</v>
       </c>
       <c r="N9" s="10" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="O9" s="10" t="s">
         <v>106</v>
       </c>
       <c r="P9" s="11" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
     </row>
     <row r="10" spans="1:16" s="11" customFormat="1" ht="211.2" x14ac:dyDescent="0.25">
@@ -2621,13 +2633,13 @@
         <v>110</v>
       </c>
       <c r="N10" s="10" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="O10" s="10" t="s">
         <v>111</v>
       </c>
       <c r="P10" s="11" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="11" spans="1:16" s="11" customFormat="1" ht="198" x14ac:dyDescent="0.25">
@@ -2671,13 +2683,13 @@
         <v>117</v>
       </c>
       <c r="N11" s="10" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="O11" s="10" t="s">
         <v>118</v>
       </c>
       <c r="P11" s="11" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="12" spans="1:16" s="11" customFormat="1" ht="264" x14ac:dyDescent="0.25">
@@ -2727,7 +2739,7 @@
         <v>126</v>
       </c>
       <c r="P12" s="11" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="13" spans="1:16" s="11" customFormat="1" ht="303.60000000000002" x14ac:dyDescent="0.25">
@@ -2768,16 +2780,16 @@
         <v>56</v>
       </c>
       <c r="M13" s="10" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="N13" s="10" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="O13" s="10" t="s">
         <v>131</v>
       </c>
       <c r="P13" s="11" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
     </row>
     <row r="14" spans="1:16" s="11" customFormat="1" ht="198" x14ac:dyDescent="0.25">
@@ -2788,10 +2800,10 @@
         <v>132</v>
       </c>
       <c r="C14" s="10" t="s">
+        <v>443</v>
+      </c>
+      <c r="D14" s="10" t="s">
         <v>444</v>
-      </c>
-      <c r="D14" s="10" t="s">
-        <v>445</v>
       </c>
       <c r="E14" s="10" t="s">
         <v>235</v>
@@ -2803,13 +2815,13 @@
         <v>246</v>
       </c>
       <c r="H14" s="10" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="I14" s="10" t="s">
         <v>48</v>
       </c>
       <c r="J14" s="10" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="K14" s="10" t="s">
         <v>49</v>
@@ -2818,16 +2830,16 @@
         <v>133</v>
       </c>
       <c r="M14" s="10" t="s">
+        <v>440</v>
+      </c>
+      <c r="N14" s="10" t="s">
         <v>441</v>
-      </c>
-      <c r="N14" s="10" t="s">
-        <v>442</v>
       </c>
       <c r="O14" s="10" t="s">
         <v>134</v>
       </c>
       <c r="P14" s="11" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
     </row>
     <row r="15" spans="1:16" s="11" customFormat="1" ht="290.39999999999998" x14ac:dyDescent="0.25">
@@ -2877,300 +2889,306 @@
         <v>138</v>
       </c>
       <c r="P15" s="11" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
     </row>
-    <row r="16" spans="1:16" s="4" customFormat="1" ht="132" x14ac:dyDescent="0.25">
-      <c r="A16" s="3" t="s">
+    <row r="16" spans="1:16" s="11" customFormat="1" ht="152.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B16" s="10" t="s">
         <v>223</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C16" s="10" t="s">
         <v>215</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="D16" s="10" t="s">
         <v>216</v>
       </c>
-      <c r="E16" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="F16" s="3" t="s">
+      <c r="E16" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="F16" s="10" t="s">
         <v>115</v>
       </c>
-      <c r="G16" s="3" t="s">
+      <c r="G16" s="10" t="s">
         <v>217</v>
       </c>
-      <c r="H16" s="3" t="s">
+      <c r="H16" s="10" t="s">
         <v>238</v>
       </c>
-      <c r="I16" s="3" t="s">
+      <c r="I16" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="J16" s="3" t="s">
+      <c r="J16" s="10" t="s">
         <v>218</v>
       </c>
-      <c r="K16" s="3" t="s">
+      <c r="K16" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="L16" s="3" t="s">
+      <c r="L16" s="10" t="s">
         <v>219</v>
       </c>
-      <c r="M16" s="3" t="s">
+      <c r="M16" s="10" t="s">
         <v>220</v>
       </c>
-      <c r="N16" s="3" t="s">
+      <c r="N16" s="10" t="s">
         <v>222</v>
       </c>
-      <c r="O16" s="3" t="s">
-        <v>291</v>
-      </c>
-      <c r="P16" s="3" t="s">
+      <c r="O16" s="10" t="s">
+        <v>445</v>
+      </c>
+      <c r="P16" s="10" t="s">
         <v>221</v>
       </c>
     </row>
-    <row r="17" spans="1:16" s="4" customFormat="1" ht="379.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="3" t="s">
+    <row r="17" spans="1:16" s="11" customFormat="1" ht="379.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="B17" s="10" t="s">
         <v>139</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="C17" s="10" t="s">
         <v>140</v>
       </c>
-      <c r="D17" s="3" t="s">
+      <c r="D17" s="10" t="s">
         <v>141</v>
       </c>
-      <c r="E17" s="3" t="s">
+      <c r="E17" s="10" t="s">
+        <v>415</v>
+      </c>
+      <c r="F17" s="10" t="s">
+        <v>396</v>
+      </c>
+      <c r="G17" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="H17" s="10" t="s">
+        <v>414</v>
+      </c>
+      <c r="I17" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="J17" s="10" t="s">
+        <v>142</v>
+      </c>
+      <c r="K17" s="10" t="s">
+        <v>421</v>
+      </c>
+      <c r="L17" s="10" t="s">
+        <v>143</v>
+      </c>
+      <c r="M17" s="10" t="s">
+        <v>144</v>
+      </c>
+      <c r="N17" s="10" t="s">
+        <v>145</v>
+      </c>
+      <c r="O17" s="10" t="s">
+        <v>447</v>
+      </c>
+      <c r="P17" s="11" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" s="11" customFormat="1" ht="304.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="B18" s="10" t="s">
+        <v>146</v>
+      </c>
+      <c r="C18" s="10" t="s">
+        <v>147</v>
+      </c>
+      <c r="D18" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="E18" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="F18" s="10" t="s">
+        <v>396</v>
+      </c>
+      <c r="G18" s="10" t="s">
+        <v>149</v>
+      </c>
+      <c r="H18" s="10" t="s">
+        <v>238</v>
+      </c>
+      <c r="I18" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="J18" s="10" t="s">
+        <v>150</v>
+      </c>
+      <c r="K18" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="L18" s="10" t="s">
+        <v>151</v>
+      </c>
+      <c r="M18" s="10" t="s">
+        <v>152</v>
+      </c>
+      <c r="N18" s="10" t="s">
+        <v>153</v>
+      </c>
+      <c r="O18" s="10" t="s">
+        <v>149</v>
+      </c>
+      <c r="P18" s="11" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="19" spans="1:16" s="11" customFormat="1" ht="409.6" x14ac:dyDescent="0.25">
+      <c r="A19" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="B19" s="10" t="s">
+        <v>155</v>
+      </c>
+      <c r="C19" s="10" t="s">
+        <v>156</v>
+      </c>
+      <c r="D19" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="E19" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="F19" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="G19" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="H19" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="I19" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="J19" s="10" t="s">
+        <v>158</v>
+      </c>
+      <c r="K19" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="L19" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="M19" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="N19" s="10" t="s">
+        <v>449</v>
+      </c>
+      <c r="O19" s="10" t="s">
+        <v>159</v>
+      </c>
+      <c r="P19" s="11" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16" s="11" customFormat="1" ht="132" x14ac:dyDescent="0.25">
+      <c r="A20" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="B20" s="10" t="s">
+        <v>224</v>
+      </c>
+      <c r="C20" s="10" t="s">
+        <v>225</v>
+      </c>
+      <c r="D20" s="10" t="s">
+        <v>226</v>
+      </c>
+      <c r="E20" s="10" t="s">
         <v>416</v>
       </c>
-      <c r="F17" s="3" t="s">
-        <v>397</v>
-      </c>
-      <c r="G17" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="H17" s="3" t="s">
-        <v>415</v>
-      </c>
-      <c r="I17" s="3" t="s">
+      <c r="F20" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="G20" s="10" t="s">
+        <v>201</v>
+      </c>
+      <c r="H20" s="10" t="s">
+        <v>238</v>
+      </c>
+      <c r="I20" s="10" t="s">
+        <v>244</v>
+      </c>
+      <c r="J20" s="10" t="s">
+        <v>227</v>
+      </c>
+      <c r="K20" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="L20" s="10" t="s">
+        <v>228</v>
+      </c>
+      <c r="M20" s="10" t="s">
+        <v>229</v>
+      </c>
+      <c r="N20" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="O20" s="10" t="s">
+        <v>230</v>
+      </c>
+      <c r="P20" s="11" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="21" spans="1:16" s="11" customFormat="1" ht="189" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="B21" s="10" t="s">
+        <v>233</v>
+      </c>
+      <c r="C21" s="10" t="s">
+        <v>234</v>
+      </c>
+      <c r="D21" s="10" t="s">
+        <v>236</v>
+      </c>
+      <c r="E21" s="10" t="s">
+        <v>235</v>
+      </c>
+      <c r="F21" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="G21" s="10" t="s">
+        <v>237</v>
+      </c>
+      <c r="H21" s="10" t="s">
+        <v>238</v>
+      </c>
+      <c r="I21" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="J17" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="K17" s="3" t="s">
-        <v>422</v>
-      </c>
-      <c r="L17" s="3" t="s">
-        <v>143</v>
-      </c>
-      <c r="M17" s="3" t="s">
-        <v>144</v>
-      </c>
-      <c r="N17" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="O17" s="3" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="18" spans="1:16" s="4" customFormat="1" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>146</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>147</v>
-      </c>
-      <c r="D18" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="E18" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="F18" s="3" t="s">
-        <v>397</v>
-      </c>
-      <c r="G18" s="3" t="s">
-        <v>149</v>
-      </c>
-      <c r="H18" s="3" t="s">
-        <v>238</v>
-      </c>
-      <c r="I18" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="J18" s="3" t="s">
-        <v>150</v>
-      </c>
-      <c r="K18" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="L18" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="M18" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="N18" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="O18" s="3" t="s">
-        <v>149</v>
-      </c>
-      <c r="P18" s="4" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="19" spans="1:16" s="4" customFormat="1" ht="409.6" x14ac:dyDescent="0.25">
-      <c r="A19" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>155</v>
-      </c>
-      <c r="C19" s="3" t="s">
-        <v>156</v>
-      </c>
-      <c r="D19" s="3" t="s">
-        <v>157</v>
-      </c>
-      <c r="E19" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="F19" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="G19" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="H19" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="I19" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="J19" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="K19" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="L19" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="M19" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="N19" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="O19" s="3" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="20" spans="1:16" s="4" customFormat="1" ht="132" x14ac:dyDescent="0.25">
-      <c r="A20" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>224</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>225</v>
-      </c>
-      <c r="D20" s="3" t="s">
-        <v>226</v>
-      </c>
-      <c r="E20" s="3" t="s">
-        <v>417</v>
-      </c>
-      <c r="F20" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="G20" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="H20" s="3" t="s">
-        <v>238</v>
-      </c>
-      <c r="I20" s="3" t="s">
-        <v>244</v>
-      </c>
-      <c r="J20" s="3" t="s">
-        <v>227</v>
-      </c>
-      <c r="K20" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="L20" s="3" t="s">
-        <v>228</v>
-      </c>
-      <c r="M20" s="3" t="s">
-        <v>229</v>
-      </c>
-      <c r="N20" s="3" t="s">
-        <v>232</v>
-      </c>
-      <c r="O20" s="3" t="s">
-        <v>230</v>
-      </c>
-      <c r="P20" s="4" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="21" spans="1:16" s="4" customFormat="1" ht="189" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>233</v>
-      </c>
-      <c r="C21" s="3" t="s">
-        <v>234</v>
-      </c>
-      <c r="D21" s="3" t="s">
-        <v>236</v>
-      </c>
-      <c r="E21" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="F21" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="G21" s="3" t="s">
-        <v>237</v>
-      </c>
-      <c r="H21" s="3" t="s">
-        <v>238</v>
-      </c>
-      <c r="I21" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="J21" s="3" t="s">
+      <c r="J21" s="10" t="s">
         <v>202</v>
       </c>
-      <c r="K21" s="3" t="s">
+      <c r="K21" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="L21" s="3" t="s">
+      <c r="L21" s="10" t="s">
         <v>239</v>
       </c>
-      <c r="M21" s="3" t="s">
+      <c r="M21" s="10" t="s">
         <v>240</v>
       </c>
-      <c r="N21" s="3" t="s">
+      <c r="N21" s="10" t="s">
         <v>241</v>
       </c>
-      <c r="O21" s="3" t="s">
+      <c r="O21" s="10" t="s">
         <v>242</v>
       </c>
-      <c r="P21" s="4" t="s">
+      <c r="P21" s="11" t="s">
         <v>243</v>
       </c>
     </row>
@@ -3245,7 +3263,7 @@
         <v>254</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="I23" s="3" t="s">
         <v>244</v>
@@ -3254,7 +3272,7 @@
         <v>255</v>
       </c>
       <c r="K23" s="3" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="L23" s="3" t="s">
         <v>256</v>
@@ -3327,7 +3345,7 @@
         <v>24</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="C25" s="3" t="s">
         <v>168</v>
@@ -3381,7 +3399,7 @@
         <v>286</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F26" s="3" t="s">
         <v>62</v>
@@ -3408,13 +3426,13 @@
         <v>289</v>
       </c>
       <c r="N26" s="3" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="O26" s="3" t="s">
         <v>290</v>
       </c>
       <c r="P26" s="4" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="27" spans="1:16" s="4" customFormat="1" ht="224.4" x14ac:dyDescent="0.25">
@@ -3431,7 +3449,7 @@
         <v>174</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F27" s="3" t="s">
         <v>115</v>
@@ -3443,7 +3461,7 @@
         <v>287</v>
       </c>
       <c r="I27" s="3" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="J27" s="3" t="s">
         <v>176</v>
@@ -3572,7 +3590,7 @@
         <v>207</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="D30" s="3" t="s">
         <v>208</v>
@@ -3587,7 +3605,7 @@
         <v>209</v>
       </c>
       <c r="H30" s="3" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="I30" s="3" t="s">
         <v>48</v>
@@ -3646,7 +3664,7 @@
         <v>278</v>
       </c>
       <c r="K31" s="3" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="L31" s="3" t="s">
         <v>279</v>
@@ -3714,13 +3732,13 @@
         <v>32</v>
       </c>
       <c r="B33" s="3" t="s">
+        <v>294</v>
+      </c>
+      <c r="C33" s="3" t="s">
         <v>295</v>
       </c>
-      <c r="C33" s="3" t="s">
+      <c r="D33" s="3" t="s">
         <v>296</v>
-      </c>
-      <c r="D33" s="3" t="s">
-        <v>297</v>
       </c>
       <c r="E33" s="3" t="s">
         <v>235</v>
@@ -3729,34 +3747,34 @@
         <v>62</v>
       </c>
       <c r="G33" s="3" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="H33" s="3" t="s">
         <v>287</v>
       </c>
       <c r="I33" s="3" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="J33" s="3" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="K33" s="3" t="s">
         <v>49</v>
       </c>
       <c r="L33" s="3" t="s">
+        <v>300</v>
+      </c>
+      <c r="M33" s="3" t="s">
         <v>301</v>
       </c>
-      <c r="M33" s="3" t="s">
+      <c r="N33" s="3" t="s">
         <v>302</v>
       </c>
-      <c r="N33" s="3" t="s">
+      <c r="O33" s="3" t="s">
         <v>303</v>
       </c>
-      <c r="O33" s="3" t="s">
+      <c r="P33" s="4" t="s">
         <v>304</v>
-      </c>
-      <c r="P33" s="4" t="s">
-        <v>305</v>
       </c>
     </row>
     <row r="34" spans="1:16" s="4" customFormat="1" ht="79.2" x14ac:dyDescent="0.25">
@@ -3764,31 +3782,31 @@
         <v>33</v>
       </c>
       <c r="B34" s="3" t="s">
+        <v>305</v>
+      </c>
+      <c r="C34" s="3" t="s">
         <v>306</v>
       </c>
-      <c r="C34" s="3" t="s">
+      <c r="D34" s="3" t="s">
         <v>307</v>
-      </c>
-      <c r="D34" s="3" t="s">
-        <v>308</v>
       </c>
       <c r="E34" s="6" t="s">
         <v>235</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="G34" s="3" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="H34" s="3" t="s">
+        <v>309</v>
+      </c>
+      <c r="I34" s="3" t="s">
+        <v>424</v>
+      </c>
+      <c r="J34" s="3" t="s">
         <v>310</v>
-      </c>
-      <c r="I34" s="3" t="s">
-        <v>425</v>
-      </c>
-      <c r="J34" s="3" t="s">
-        <v>311</v>
       </c>
       <c r="K34" s="3" t="s">
         <v>49</v>
@@ -3797,16 +3815,16 @@
         <v>202</v>
       </c>
       <c r="M34" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="N34" s="3" t="s">
         <v>312</v>
       </c>
-      <c r="N34" s="3" t="s">
+      <c r="O34" s="3" t="s">
         <v>313</v>
       </c>
-      <c r="O34" s="3" t="s">
+      <c r="P34" s="4" t="s">
         <v>314</v>
-      </c>
-      <c r="P34" s="4" t="s">
-        <v>315</v>
       </c>
     </row>
     <row r="35" spans="1:16" s="4" customFormat="1" ht="92.4" x14ac:dyDescent="0.25">
@@ -3814,22 +3832,22 @@
         <v>34</v>
       </c>
       <c r="B35" s="3" t="s">
+        <v>315</v>
+      </c>
+      <c r="C35" s="3" t="s">
         <v>316</v>
       </c>
-      <c r="C35" s="3" t="s">
+      <c r="D35" s="3" t="s">
         <v>317</v>
       </c>
-      <c r="D35" s="3" t="s">
-        <v>318</v>
-      </c>
       <c r="E35" s="3" t="s">
         <v>56</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="G35" s="3" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="H35" s="3" t="s">
         <v>238</v>
@@ -3838,25 +3856,25 @@
         <v>48</v>
       </c>
       <c r="J35" s="3" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="K35" s="3" t="s">
         <v>49</v>
       </c>
       <c r="L35" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="M35" s="3" t="s">
         <v>320</v>
       </c>
-      <c r="M35" s="3" t="s">
+      <c r="N35" s="3" t="s">
         <v>321</v>
       </c>
-      <c r="N35" s="3" t="s">
+      <c r="O35" s="3" t="s">
         <v>322</v>
       </c>
-      <c r="O35" s="3" t="s">
+      <c r="P35" s="4" t="s">
         <v>323</v>
-      </c>
-      <c r="P35" s="4" t="s">
-        <v>324</v>
       </c>
     </row>
     <row r="36" spans="1:16" s="4" customFormat="1" ht="79.2" x14ac:dyDescent="0.25">
@@ -3864,49 +3882,49 @@
         <v>35</v>
       </c>
       <c r="B36" s="3" t="s">
+        <v>324</v>
+      </c>
+      <c r="C36" s="3" t="s">
         <v>325</v>
       </c>
-      <c r="C36" s="3" t="s">
+      <c r="D36" s="3" t="s">
         <v>326</v>
-      </c>
-      <c r="D36" s="3" t="s">
-        <v>327</v>
       </c>
       <c r="E36" s="3" t="s">
         <v>235</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="G36" s="3" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="H36" s="3" t="s">
         <v>238</v>
       </c>
       <c r="I36" s="3" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="J36" s="3" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="K36" s="3" t="s">
         <v>64</v>
       </c>
       <c r="L36" s="3" t="s">
+        <v>330</v>
+      </c>
+      <c r="M36" s="3" t="s">
         <v>331</v>
       </c>
-      <c r="M36" s="3" t="s">
+      <c r="N36" s="3" t="s">
         <v>332</v>
       </c>
-      <c r="N36" s="3" t="s">
+      <c r="O36" s="3" t="s">
         <v>333</v>
       </c>
-      <c r="O36" s="3" t="s">
+      <c r="P36" s="4" t="s">
         <v>334</v>
-      </c>
-      <c r="P36" s="4" t="s">
-        <v>335</v>
       </c>
     </row>
     <row r="37" spans="1:16" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -3959,49 +3977,49 @@
         <v>37</v>
       </c>
       <c r="B38" s="3" t="s">
+        <v>335</v>
+      </c>
+      <c r="C38" s="3" t="s">
         <v>336</v>
       </c>
-      <c r="C38" s="3" t="s">
+      <c r="D38" s="3" t="s">
         <v>337</v>
-      </c>
-      <c r="D38" s="3" t="s">
-        <v>338</v>
       </c>
       <c r="E38" s="3" t="s">
         <v>235</v>
       </c>
       <c r="F38" s="3" t="s">
+        <v>339</v>
+      </c>
+      <c r="G38" s="3" t="s">
+        <v>297</v>
+      </c>
+      <c r="H38" s="3" t="s">
         <v>340</v>
-      </c>
-      <c r="G38" s="3" t="s">
-        <v>298</v>
-      </c>
-      <c r="H38" s="3" t="s">
-        <v>341</v>
       </c>
       <c r="I38" s="3" t="s">
         <v>48</v>
       </c>
       <c r="J38" s="3" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="K38" s="3" t="s">
         <v>49</v>
       </c>
       <c r="L38" s="3" t="s">
+        <v>341</v>
+      </c>
+      <c r="M38" s="3" t="s">
         <v>342</v>
       </c>
-      <c r="M38" s="3" t="s">
+      <c r="N38" s="3" t="s">
+        <v>321</v>
+      </c>
+      <c r="O38" s="3" t="s">
         <v>343</v>
       </c>
-      <c r="N38" s="3" t="s">
-        <v>322</v>
-      </c>
-      <c r="O38" s="3" t="s">
+      <c r="P38" s="4" t="s">
         <v>344</v>
-      </c>
-      <c r="P38" s="4" t="s">
-        <v>345</v>
       </c>
     </row>
     <row r="39" spans="1:16" s="4" customFormat="1" ht="132" x14ac:dyDescent="0.25">
@@ -4009,22 +4027,22 @@
         <v>38</v>
       </c>
       <c r="B39" s="3" t="s">
+        <v>345</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>347</v>
+      </c>
+      <c r="D39" s="3" t="s">
         <v>346</v>
       </c>
-      <c r="C39" s="3" t="s">
-        <v>348</v>
-      </c>
-      <c r="D39" s="3" t="s">
-        <v>347</v>
-      </c>
       <c r="E39" s="3" t="s">
         <v>56</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="G39" s="3" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="H39" s="3" t="s">
         <v>238</v>
@@ -4033,75 +4051,75 @@
         <v>48</v>
       </c>
       <c r="J39" s="3" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="K39" s="3" t="s">
         <v>49</v>
       </c>
       <c r="L39" s="3" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="M39" s="3" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="N39" s="3" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="O39" s="3" t="s">
+        <v>349</v>
+      </c>
+      <c r="P39" s="4" t="s">
         <v>350</v>
       </c>
-      <c r="P39" s="4" t="s">
+    </row>
+    <row r="40" spans="1:16" s="11" customFormat="1" ht="145.19999999999999" x14ac:dyDescent="0.25">
+      <c r="A40" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="B40" s="10" t="s">
         <v>351</v>
       </c>
-    </row>
-    <row r="40" spans="1:16" s="4" customFormat="1" ht="145.19999999999999" x14ac:dyDescent="0.25">
-      <c r="A40" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="B40" s="3" t="s">
+      <c r="C40" s="10" t="s">
         <v>352</v>
       </c>
-      <c r="C40" s="3" t="s">
+      <c r="D40" s="10" t="s">
         <v>353</v>
       </c>
-      <c r="D40" s="3" t="s">
+      <c r="E40" s="10" t="s">
+        <v>415</v>
+      </c>
+      <c r="F40" s="10" t="s">
         <v>354</v>
       </c>
-      <c r="E40" s="3" t="s">
-        <v>416</v>
-      </c>
-      <c r="F40" s="3" t="s">
+      <c r="G40" s="10" t="s">
+        <v>297</v>
+      </c>
+      <c r="H40" s="10" t="s">
+        <v>238</v>
+      </c>
+      <c r="I40" s="10" t="s">
+        <v>244</v>
+      </c>
+      <c r="J40" s="10" t="s">
         <v>355</v>
       </c>
-      <c r="G40" s="3" t="s">
-        <v>298</v>
-      </c>
-      <c r="H40" s="3" t="s">
-        <v>238</v>
-      </c>
-      <c r="I40" s="3" t="s">
-        <v>244</v>
-      </c>
-      <c r="J40" s="3" t="s">
+      <c r="K40" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="L40" s="10" t="s">
         <v>356</v>
       </c>
-      <c r="K40" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="L40" s="3" t="s">
+      <c r="M40" s="10" t="s">
         <v>357</v>
       </c>
-      <c r="M40" s="3" t="s">
+      <c r="N40" s="10" t="s">
         <v>358</v>
       </c>
-      <c r="N40" s="3" t="s">
+      <c r="O40" s="10" t="s">
         <v>359</v>
       </c>
-      <c r="O40" s="3" t="s">
+      <c r="P40" s="11" t="s">
         <v>360</v>
-      </c>
-      <c r="P40" s="4" t="s">
-        <v>361</v>
       </c>
     </row>
     <row r="41" spans="1:16" s="4" customFormat="1" ht="118.8" x14ac:dyDescent="0.25">
@@ -4109,25 +4127,25 @@
         <v>40</v>
       </c>
       <c r="B41" s="3" t="s">
+        <v>361</v>
+      </c>
+      <c r="C41" s="3" t="s">
         <v>362</v>
       </c>
-      <c r="C41" s="3" t="s">
+      <c r="D41" s="3" t="s">
         <v>363</v>
       </c>
-      <c r="D41" s="3" t="s">
-        <v>364</v>
-      </c>
       <c r="E41" s="3" t="s">
         <v>56</v>
       </c>
       <c r="F41" s="3" t="s">
+        <v>339</v>
+      </c>
+      <c r="G41" s="3" t="s">
+        <v>297</v>
+      </c>
+      <c r="H41" s="3" t="s">
         <v>340</v>
-      </c>
-      <c r="G41" s="3" t="s">
-        <v>298</v>
-      </c>
-      <c r="H41" s="3" t="s">
-        <v>341</v>
       </c>
       <c r="I41" s="3" t="s">
         <v>48</v>
@@ -4139,19 +4157,19 @@
         <v>49</v>
       </c>
       <c r="L41" s="3" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="M41" s="3" t="s">
+        <v>364</v>
+      </c>
+      <c r="N41" s="3" t="s">
         <v>365</v>
       </c>
-      <c r="N41" s="3" t="s">
+      <c r="O41" s="3" t="s">
         <v>366</v>
       </c>
-      <c r="O41" s="3" t="s">
+      <c r="P41" s="4" t="s">
         <v>367</v>
-      </c>
-      <c r="P41" s="4" t="s">
-        <v>368</v>
       </c>
     </row>
     <row r="42" spans="1:16" s="4" customFormat="1" ht="145.19999999999999" x14ac:dyDescent="0.25">
@@ -4159,22 +4177,22 @@
         <v>41</v>
       </c>
       <c r="B42" s="3" t="s">
+        <v>368</v>
+      </c>
+      <c r="C42" s="3" t="s">
         <v>369</v>
       </c>
-      <c r="C42" s="3" t="s">
+      <c r="D42" s="3" t="s">
         <v>370</v>
-      </c>
-      <c r="D42" s="3" t="s">
-        <v>371</v>
       </c>
       <c r="E42" s="3" t="s">
         <v>235</v>
       </c>
       <c r="F42" s="3" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="G42" s="3" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="H42" s="3" t="s">
         <v>238</v>
@@ -4183,25 +4201,25 @@
         <v>48</v>
       </c>
       <c r="J42" s="3" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="K42" s="3" t="s">
         <v>49</v>
       </c>
       <c r="L42" s="3" t="s">
+        <v>372</v>
+      </c>
+      <c r="M42" s="3" t="s">
         <v>373</v>
       </c>
-      <c r="M42" s="3" t="s">
+      <c r="N42" s="3" t="s">
         <v>374</v>
       </c>
-      <c r="N42" s="3" t="s">
+      <c r="O42" s="3" t="s">
         <v>375</v>
       </c>
-      <c r="O42" s="3" t="s">
+      <c r="P42" s="4" t="s">
         <v>376</v>
-      </c>
-      <c r="P42" s="4" t="s">
-        <v>377</v>
       </c>
     </row>
     <row r="43" spans="1:16" s="4" customFormat="1" ht="145.19999999999999" x14ac:dyDescent="0.25">
@@ -4209,19 +4227,19 @@
         <v>42</v>
       </c>
       <c r="B43" s="3" t="s">
+        <v>377</v>
+      </c>
+      <c r="C43" s="3" t="s">
         <v>378</v>
       </c>
-      <c r="C43" s="3" t="s">
+      <c r="D43" s="3" t="s">
         <v>379</v>
       </c>
-      <c r="D43" s="3" t="s">
-        <v>380</v>
-      </c>
       <c r="E43" s="3" t="s">
         <v>56</v>
       </c>
       <c r="F43" s="3" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="G43" s="3" t="s">
         <v>275</v>
@@ -4233,25 +4251,25 @@
         <v>48</v>
       </c>
       <c r="J43" s="3" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="K43" s="3" t="s">
         <v>49</v>
       </c>
       <c r="L43" s="3" t="s">
+        <v>381</v>
+      </c>
+      <c r="M43" s="3" t="s">
         <v>382</v>
       </c>
-      <c r="M43" s="3" t="s">
+      <c r="N43" s="3" t="s">
         <v>383</v>
       </c>
-      <c r="N43" s="3" t="s">
+      <c r="O43" s="3" t="s">
         <v>384</v>
       </c>
-      <c r="O43" s="3" t="s">
+      <c r="P43" s="4" t="s">
         <v>385</v>
-      </c>
-      <c r="P43" s="4" t="s">
-        <v>386</v>
       </c>
     </row>
     <row r="44" spans="1:16" s="4" customFormat="1" ht="171.6" x14ac:dyDescent="0.25">
@@ -4259,49 +4277,49 @@
         <v>43</v>
       </c>
       <c r="B44" s="3" t="s">
+        <v>386</v>
+      </c>
+      <c r="C44" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="C44" s="3" t="s">
+      <c r="D44" s="3" t="s">
+        <v>395</v>
+      </c>
+      <c r="E44" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="F44" s="3" t="s">
         <v>388</v>
       </c>
-      <c r="D44" s="3" t="s">
-        <v>396</v>
-      </c>
-      <c r="E44" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="F44" s="3" t="s">
-        <v>389</v>
-      </c>
       <c r="G44" s="3" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="H44" s="3" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="I44" s="3" t="s">
         <v>48</v>
       </c>
       <c r="J44" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="K44" s="3" t="s">
+        <v>420</v>
+      </c>
+      <c r="L44" s="3" t="s">
         <v>390</v>
       </c>
-      <c r="K44" s="3" t="s">
-        <v>421</v>
-      </c>
-      <c r="L44" s="3" t="s">
+      <c r="M44" s="3" t="s">
         <v>391</v>
       </c>
-      <c r="M44" s="3" t="s">
+      <c r="N44" s="3" t="s">
         <v>392</v>
       </c>
-      <c r="N44" s="3" t="s">
+      <c r="O44" s="3" t="s">
         <v>393</v>
       </c>
-      <c r="O44" s="3" t="s">
+      <c r="P44" s="4" t="s">
         <v>394</v>
-      </c>
-      <c r="P44" s="4" t="s">
-        <v>395</v>
       </c>
     </row>
     <row r="45" spans="1:16" ht="145.19999999999999" x14ac:dyDescent="0.25">
@@ -4309,22 +4327,22 @@
         <v>44</v>
       </c>
       <c r="B45" s="3" t="s">
+        <v>368</v>
+      </c>
+      <c r="C45" s="3" t="s">
         <v>369</v>
       </c>
-      <c r="C45" s="3" t="s">
+      <c r="D45" s="3" t="s">
         <v>370</v>
-      </c>
-      <c r="D45" s="3" t="s">
-        <v>371</v>
       </c>
       <c r="E45" s="3" t="s">
         <v>235</v>
       </c>
       <c r="F45" s="3" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="G45" s="3" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="H45" s="3" t="s">
         <v>238</v>
@@ -4333,25 +4351,25 @@
         <v>48</v>
       </c>
       <c r="J45" s="3" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="K45" s="3" t="s">
         <v>49</v>
       </c>
       <c r="L45" s="3" t="s">
+        <v>372</v>
+      </c>
+      <c r="M45" s="3" t="s">
         <v>373</v>
       </c>
-      <c r="M45" s="3" t="s">
+      <c r="N45" s="3" t="s">
         <v>374</v>
       </c>
-      <c r="N45" s="3" t="s">
+      <c r="O45" s="3" t="s">
         <v>375</v>
       </c>
-      <c r="O45" s="3" t="s">
+      <c r="P45" s="4" t="s">
         <v>376</v>
-      </c>
-      <c r="P45" s="4" t="s">
-        <v>377</v>
       </c>
     </row>
   </sheetData>
@@ -4361,18 +4379,18 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4520,18 +4538,18 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1160EB8C-E200-4916-A3B3-9BF8115D37F8}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24F2579D-323E-48EA-8FED-D372AFFF0A04}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24F2579D-323E-48EA-8FED-D372AFFF0A04}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1160EB8C-E200-4916-A3B3-9BF8115D37F8}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Add new template and individual annotations files for data extraction
</commit_message>
<xml_diff>
--- a/main/05_data_charting/data/Individual_Annotations.xlsx
+++ b/main/05_data_charting/data/Individual_Annotations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\orincon\scoping-ml-wave-seismology\main\05_data_charting\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5339867D-9FB7-4755-9A24-7C4909730176}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E1DFBFF-5CE3-415B-9780-6C6921C7F2F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{115BB8D9-8B86-4726-97F8-E06477FD353D}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="716" uniqueCount="456">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="718" uniqueCount="458">
   <si>
     <t>Research gaps</t>
   </si>
@@ -1658,6 +1658,12 @@
   </si>
   <si>
     <t>Pixel accuracy and Intersection over Union (IOU)</t>
+  </si>
+  <si>
+    <t>Mean Squared Error (MSE),  Structural Similarity Index (SSIM) and Data misfit (L2 norm)</t>
+  </si>
+  <si>
+    <t>Extension to density inversion</t>
   </si>
 </sst>
 </file>
@@ -1787,9 +1793,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1813,6 +1816,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2170,1842 +2176,1847 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="6" t="s">
         <v>400</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="5" t="s">
         <v>401</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="6" t="s">
         <v>402</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="E1" s="6" t="s">
         <v>404</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="F1" s="6" t="s">
         <v>403</v>
       </c>
-      <c r="G1" s="7" t="s">
+      <c r="G1" s="6" t="s">
         <v>405</v>
       </c>
-      <c r="H1" s="7" t="s">
+      <c r="H1" s="6" t="s">
         <v>406</v>
       </c>
-      <c r="I1" s="7" t="s">
+      <c r="I1" s="6" t="s">
         <v>407</v>
       </c>
-      <c r="J1" s="7" t="s">
+      <c r="J1" s="6" t="s">
         <v>408</v>
       </c>
-      <c r="K1" s="7" t="s">
+      <c r="K1" s="6" t="s">
         <v>409</v>
       </c>
-      <c r="L1" s="7" t="s">
+      <c r="L1" s="6" t="s">
         <v>410</v>
       </c>
-      <c r="M1" s="6" t="s">
+      <c r="M1" s="5" t="s">
         <v>411</v>
       </c>
-      <c r="N1" s="6" t="s">
+      <c r="N1" s="5" t="s">
         <v>412</v>
       </c>
-      <c r="O1" s="6" t="s">
+      <c r="O1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="P1" s="5" t="s">
+      <c r="P1" s="4" t="s">
         <v>413</v>
       </c>
     </row>
-    <row r="2" spans="1:16" s="9" customFormat="1" ht="250.8" x14ac:dyDescent="0.25">
-      <c r="A2" s="8" t="s">
+    <row r="2" spans="1:16" s="8" customFormat="1" ht="250.8" x14ac:dyDescent="0.25">
+      <c r="A2" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C2" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="D2" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="E2" s="7" t="s">
         <v>417</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="F2" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="G2" s="8" t="s">
+      <c r="G2" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="H2" s="8" t="s">
+      <c r="H2" s="7" t="s">
         <v>238</v>
       </c>
-      <c r="I2" s="8" t="s">
+      <c r="I2" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="J2" s="8" t="s">
+      <c r="J2" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="K2" s="8" t="s">
+      <c r="K2" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="L2" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="M2" s="8" t="s">
+      <c r="L2" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="M2" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="N2" s="8" t="s">
+      <c r="N2" s="7" t="s">
         <v>425</v>
       </c>
-      <c r="O2" s="8" t="s">
+      <c r="O2" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="P2" s="9" t="s">
+      <c r="P2" s="8" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="3" spans="1:16" s="9" customFormat="1" ht="184.8" x14ac:dyDescent="0.25">
-      <c r="A3" s="8" t="s">
+    <row r="3" spans="1:16" s="8" customFormat="1" ht="184.8" x14ac:dyDescent="0.25">
+      <c r="A3" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D3" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="E3" s="7" t="s">
         <v>415</v>
       </c>
-      <c r="F3" s="8" t="s">
+      <c r="F3" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="G3" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="H3" s="8" t="s">
+      <c r="G3" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="H3" s="7" t="s">
         <v>238</v>
       </c>
-      <c r="I3" s="8" t="s">
+      <c r="I3" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="J3" s="8" t="s">
+      <c r="J3" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="K3" s="8" t="s">
+      <c r="K3" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="L3" s="8" t="s">
+      <c r="L3" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="M3" s="8" t="s">
+      <c r="M3" s="7" t="s">
         <v>425</v>
       </c>
-      <c r="N3" s="8" t="s">
+      <c r="N3" s="7" t="s">
         <v>425</v>
       </c>
-      <c r="O3" s="8" t="s">
+      <c r="O3" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="P3" s="9" t="s">
+      <c r="P3" s="8" t="s">
         <v>426</v>
       </c>
     </row>
-    <row r="4" spans="1:16" s="9" customFormat="1" ht="201" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="8" t="s">
+    <row r="4" spans="1:16" s="8" customFormat="1" ht="201" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D4" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="E4" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="F4" s="8" t="s">
+      <c r="E4" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="F4" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="G4" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="H4" s="8" t="s">
+      <c r="G4" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="H4" s="7" t="s">
         <v>238</v>
       </c>
-      <c r="I4" s="8" t="s">
+      <c r="I4" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="J4" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="K4" s="8" t="s">
+      <c r="J4" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="K4" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="L4" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="M4" s="8" t="s">
+      <c r="L4" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="M4" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="N4" s="8" t="s">
+      <c r="N4" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="O4" s="8" t="s">
+      <c r="O4" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="P4" s="9" t="s">
+      <c r="P4" s="8" t="s">
         <v>427</v>
       </c>
     </row>
-    <row r="5" spans="1:16" s="9" customFormat="1" ht="210" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="8" t="s">
+    <row r="5" spans="1:16" s="8" customFormat="1" ht="210" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="C5" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="D5" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="E5" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="F5" s="8" t="s">
+      <c r="E5" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="F5" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="G5" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="H5" s="8" t="s">
+      <c r="G5" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="H5" s="7" t="s">
         <v>238</v>
       </c>
-      <c r="I5" s="8" t="s">
+      <c r="I5" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="J5" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="K5" s="8" t="s">
+      <c r="J5" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="K5" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="L5" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="M5" s="8" t="s">
+      <c r="L5" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="M5" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="N5" s="8" t="s">
+      <c r="N5" s="7" t="s">
         <v>425</v>
       </c>
-      <c r="O5" s="8" t="s">
+      <c r="O5" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="P5" s="9" t="s">
+      <c r="P5" s="8" t="s">
         <v>428</v>
       </c>
     </row>
-    <row r="6" spans="1:16" s="9" customFormat="1" ht="250.8" x14ac:dyDescent="0.25">
-      <c r="A6" s="8" t="s">
+    <row r="6" spans="1:16" s="8" customFormat="1" ht="250.8" x14ac:dyDescent="0.25">
+      <c r="A6" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="C6" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="D6" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="E6" s="7" t="s">
         <v>170</v>
       </c>
-      <c r="F6" s="8" t="s">
+      <c r="F6" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="G6" s="8" t="s">
+      <c r="G6" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="H6" s="8" t="s">
+      <c r="H6" s="7" t="s">
         <v>238</v>
       </c>
-      <c r="I6" s="8" t="s">
+      <c r="I6" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="J6" s="8" t="s">
+      <c r="J6" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="K6" s="8" t="s">
+      <c r="K6" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="L6" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="M6" s="8" t="s">
+      <c r="L6" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="M6" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="N6" s="8" t="s">
+      <c r="N6" s="7" t="s">
         <v>425</v>
       </c>
-      <c r="O6" s="8" t="s">
+      <c r="O6" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="P6" s="9" t="s">
+      <c r="P6" s="8" t="s">
         <v>429</v>
       </c>
     </row>
-    <row r="7" spans="1:16" s="9" customFormat="1" ht="250.8" x14ac:dyDescent="0.25">
-      <c r="A7" s="8" t="s">
+    <row r="7" spans="1:16" s="8" customFormat="1" ht="250.8" x14ac:dyDescent="0.25">
+      <c r="A7" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="C7" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="D7" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="E7" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="F7" s="8" t="s">
+      <c r="F7" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="G7" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="H7" s="8" t="s">
+      <c r="G7" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="H7" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="I7" s="8" t="s">
+      <c r="I7" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="J7" s="8" t="s">
+      <c r="J7" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="K7" s="8" t="s">
+      <c r="K7" s="7" t="s">
         <v>419</v>
       </c>
-      <c r="L7" s="8" t="s">
+      <c r="L7" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="M7" s="8" t="s">
+      <c r="M7" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="N7" s="8" t="s">
+      <c r="N7" s="7" t="s">
         <v>425</v>
       </c>
-      <c r="O7" s="8" t="s">
+      <c r="O7" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="P7" s="9" t="s">
+      <c r="P7" s="8" t="s">
         <v>430</v>
       </c>
     </row>
-    <row r="8" spans="1:16" s="9" customFormat="1" ht="184.8" x14ac:dyDescent="0.25">
-      <c r="A8" s="8" t="s">
+    <row r="8" spans="1:16" s="8" customFormat="1" ht="184.8" x14ac:dyDescent="0.25">
+      <c r="A8" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="D8" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="E8" s="8" t="s">
+      <c r="E8" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="F8" s="8" t="s">
+      <c r="F8" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="G8" s="8" t="s">
+      <c r="G8" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="H8" s="8" t="s">
+      <c r="H8" s="7" t="s">
         <v>238</v>
       </c>
-      <c r="I8" s="8" t="s">
+      <c r="I8" s="7" t="s">
         <v>244</v>
       </c>
-      <c r="J8" s="8" t="s">
+      <c r="J8" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="K8" s="8" t="s">
+      <c r="K8" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="L8" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="M8" s="8" t="s">
+      <c r="L8" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="M8" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="N8" s="8" t="s">
+      <c r="N8" s="7" t="s">
         <v>425</v>
       </c>
-      <c r="O8" s="8" t="s">
+      <c r="O8" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="P8" s="9" t="s">
+      <c r="P8" s="8" t="s">
         <v>431</v>
       </c>
     </row>
-    <row r="9" spans="1:16" s="9" customFormat="1" ht="303.60000000000002" x14ac:dyDescent="0.25">
-      <c r="A9" s="8" t="s">
+    <row r="9" spans="1:16" s="8" customFormat="1" ht="303.60000000000002" x14ac:dyDescent="0.25">
+      <c r="A9" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="B9" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="C9" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="D9" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="E9" s="8" t="s">
+      <c r="E9" s="7" t="s">
         <v>235</v>
       </c>
-      <c r="F9" s="8" t="s">
+      <c r="F9" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="G9" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="H9" s="8" t="s">
+      <c r="G9" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="H9" s="7" t="s">
         <v>414</v>
       </c>
-      <c r="I9" s="8" t="s">
+      <c r="I9" s="7" t="s">
         <v>244</v>
       </c>
-      <c r="J9" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="K9" s="8" t="s">
+      <c r="J9" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="K9" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="L9" s="8" t="s">
+      <c r="L9" s="7" t="s">
         <v>104</v>
       </c>
-      <c r="M9" s="8" t="s">
+      <c r="M9" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="N9" s="8" t="s">
+      <c r="N9" s="7" t="s">
         <v>425</v>
       </c>
-      <c r="O9" s="8" t="s">
+      <c r="O9" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="P9" s="9" t="s">
+      <c r="P9" s="8" t="s">
         <v>432</v>
       </c>
     </row>
-    <row r="10" spans="1:16" s="9" customFormat="1" ht="211.2" x14ac:dyDescent="0.25">
-      <c r="A10" s="8" t="s">
+    <row r="10" spans="1:16" s="8" customFormat="1" ht="211.2" x14ac:dyDescent="0.25">
+      <c r="A10" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="B10" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="C10" s="8" t="s">
+      <c r="C10" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="D10" s="8" t="s">
+      <c r="D10" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="E10" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="F10" s="8" t="s">
+      <c r="E10" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="F10" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="G10" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="H10" s="8" t="s">
+      <c r="G10" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="H10" s="7" t="s">
         <v>238</v>
       </c>
-      <c r="I10" s="8" t="s">
+      <c r="I10" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="J10" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="K10" s="8" t="s">
+      <c r="J10" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="K10" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="L10" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="M10" s="8" t="s">
+      <c r="L10" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="M10" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="N10" s="8" t="s">
+      <c r="N10" s="7" t="s">
         <v>425</v>
       </c>
-      <c r="O10" s="8" t="s">
+      <c r="O10" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="P10" s="9" t="s">
+      <c r="P10" s="8" t="s">
         <v>433</v>
       </c>
     </row>
-    <row r="11" spans="1:16" s="9" customFormat="1" ht="198" x14ac:dyDescent="0.25">
-      <c r="A11" s="8" t="s">
+    <row r="11" spans="1:16" s="8" customFormat="1" ht="198" x14ac:dyDescent="0.25">
+      <c r="A11" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="B11" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="C11" s="8" t="s">
+      <c r="C11" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="D11" s="8" t="s">
+      <c r="D11" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="E11" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="F11" s="8" t="s">
+      <c r="E11" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="F11" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="G11" s="8" t="s">
+      <c r="G11" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="H11" s="8" t="s">
+      <c r="H11" s="7" t="s">
         <v>238</v>
       </c>
-      <c r="I11" s="8" t="s">
+      <c r="I11" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="J11" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="K11" s="8" t="s">
+      <c r="J11" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="K11" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="L11" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="M11" s="8" t="s">
+      <c r="L11" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="M11" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="N11" s="8" t="s">
+      <c r="N11" s="7" t="s">
         <v>425</v>
       </c>
-      <c r="O11" s="8" t="s">
+      <c r="O11" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="P11" s="9" t="s">
+      <c r="P11" s="8" t="s">
         <v>434</v>
       </c>
     </row>
-    <row r="12" spans="1:16" s="9" customFormat="1" ht="264" x14ac:dyDescent="0.25">
-      <c r="A12" s="8" t="s">
+    <row r="12" spans="1:16" s="8" customFormat="1" ht="264" x14ac:dyDescent="0.25">
+      <c r="A12" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="B12" s="7" t="s">
         <v>119</v>
       </c>
-      <c r="C12" s="8" t="s">
+      <c r="C12" s="7" t="s">
         <v>120</v>
       </c>
-      <c r="D12" s="8" t="s">
+      <c r="D12" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="E12" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="F12" s="8" t="s">
+      <c r="E12" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="F12" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="G12" s="8" t="s">
+      <c r="G12" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="H12" s="8" t="s">
+      <c r="H12" s="7" t="s">
         <v>238</v>
       </c>
-      <c r="I12" s="8" t="s">
+      <c r="I12" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="J12" s="8" t="s">
+      <c r="J12" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="K12" s="8" t="s">
+      <c r="K12" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="L12" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="M12" s="8" t="s">
+      <c r="L12" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="M12" s="7" t="s">
         <v>124</v>
       </c>
-      <c r="N12" s="8" t="s">
+      <c r="N12" s="7" t="s">
         <v>125</v>
       </c>
-      <c r="O12" s="8" t="s">
+      <c r="O12" s="7" t="s">
         <v>126</v>
       </c>
-      <c r="P12" s="9" t="s">
+      <c r="P12" s="8" t="s">
         <v>435</v>
       </c>
     </row>
-    <row r="13" spans="1:16" s="9" customFormat="1" ht="303.60000000000002" x14ac:dyDescent="0.25">
-      <c r="A13" s="8" t="s">
+    <row r="13" spans="1:16" s="8" customFormat="1" ht="303.60000000000002" x14ac:dyDescent="0.25">
+      <c r="A13" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="B13" s="8" t="s">
+      <c r="B13" s="7" t="s">
         <v>127</v>
       </c>
-      <c r="C13" s="8" t="s">
+      <c r="C13" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="D13" s="8" t="s">
+      <c r="D13" s="7" t="s">
         <v>129</v>
       </c>
-      <c r="E13" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="F13" s="8" t="s">
+      <c r="E13" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="F13" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="G13" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="H13" s="8" t="s">
+      <c r="G13" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="H13" s="7" t="s">
         <v>238</v>
       </c>
-      <c r="I13" s="8" t="s">
+      <c r="I13" s="7" t="s">
         <v>244</v>
       </c>
-      <c r="J13" s="8" t="s">
+      <c r="J13" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="K13" s="8" t="s">
+      <c r="K13" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="L13" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="M13" s="8" t="s">
+      <c r="L13" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="M13" s="7" t="s">
         <v>438</v>
       </c>
-      <c r="N13" s="8" t="s">
+      <c r="N13" s="7" t="s">
         <v>437</v>
       </c>
-      <c r="O13" s="8" t="s">
+      <c r="O13" s="7" t="s">
         <v>131</v>
       </c>
-      <c r="P13" s="9" t="s">
+      <c r="P13" s="8" t="s">
         <v>436</v>
       </c>
     </row>
-    <row r="14" spans="1:16" s="9" customFormat="1" ht="198" x14ac:dyDescent="0.25">
-      <c r="A14" s="8" t="s">
+    <row r="14" spans="1:16" s="8" customFormat="1" ht="198" x14ac:dyDescent="0.25">
+      <c r="A14" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="B14" s="8" t="s">
+      <c r="B14" s="7" t="s">
         <v>132</v>
       </c>
-      <c r="C14" s="8" t="s">
+      <c r="C14" s="7" t="s">
         <v>443</v>
       </c>
-      <c r="D14" s="8" t="s">
+      <c r="D14" s="7" t="s">
         <v>444</v>
       </c>
-      <c r="E14" s="8" t="s">
+      <c r="E14" s="7" t="s">
         <v>235</v>
       </c>
-      <c r="F14" s="8" t="s">
+      <c r="F14" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="G14" s="8" t="s">
+      <c r="G14" s="7" t="s">
         <v>246</v>
       </c>
-      <c r="H14" s="8" t="s">
+      <c r="H14" s="7" t="s">
         <v>309</v>
       </c>
-      <c r="I14" s="8" t="s">
+      <c r="I14" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="J14" s="8" t="s">
+      <c r="J14" s="7" t="s">
         <v>439</v>
       </c>
-      <c r="K14" s="8" t="s">
+      <c r="K14" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="L14" s="8" t="s">
+      <c r="L14" s="7" t="s">
         <v>133</v>
       </c>
-      <c r="M14" s="8" t="s">
+      <c r="M14" s="7" t="s">
         <v>440</v>
       </c>
-      <c r="N14" s="8" t="s">
+      <c r="N14" s="7" t="s">
         <v>441</v>
       </c>
-      <c r="O14" s="8" t="s">
+      <c r="O14" s="7" t="s">
         <v>134</v>
       </c>
-      <c r="P14" s="9" t="s">
+      <c r="P14" s="8" t="s">
         <v>442</v>
       </c>
     </row>
-    <row r="15" spans="1:16" s="9" customFormat="1" ht="290.39999999999998" x14ac:dyDescent="0.25">
-      <c r="A15" s="8" t="s">
+    <row r="15" spans="1:16" s="8" customFormat="1" ht="290.39999999999998" x14ac:dyDescent="0.25">
+      <c r="A15" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="B15" s="8" t="s">
+      <c r="B15" s="7" t="s">
         <v>135</v>
       </c>
-      <c r="C15" s="8" t="s">
+      <c r="C15" s="7" t="s">
         <v>245</v>
       </c>
-      <c r="D15" s="8" t="s">
+      <c r="D15" s="7" t="s">
         <v>136</v>
       </c>
-      <c r="E15" s="8" t="s">
+      <c r="E15" s="7" t="s">
         <v>235</v>
       </c>
-      <c r="F15" s="8" t="s">
+      <c r="F15" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="G15" s="8" t="s">
+      <c r="G15" s="7" t="s">
         <v>246</v>
       </c>
-      <c r="H15" s="8" t="s">
+      <c r="H15" s="7" t="s">
         <v>238</v>
       </c>
-      <c r="I15" s="8" t="s">
+      <c r="I15" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="J15" s="8" t="s">
+      <c r="J15" s="7" t="s">
         <v>247</v>
       </c>
-      <c r="K15" s="8" t="s">
+      <c r="K15" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="L15" s="8" t="s">
+      <c r="L15" s="7" t="s">
         <v>248</v>
       </c>
-      <c r="M15" s="8" t="s">
+      <c r="M15" s="7" t="s">
         <v>249</v>
       </c>
-      <c r="N15" s="8" t="s">
+      <c r="N15" s="7" t="s">
         <v>137</v>
       </c>
-      <c r="O15" s="8" t="s">
+      <c r="O15" s="7" t="s">
         <v>138</v>
       </c>
-      <c r="P15" s="9" t="s">
+      <c r="P15" s="8" t="s">
         <v>442</v>
       </c>
     </row>
-    <row r="16" spans="1:16" s="9" customFormat="1" ht="152.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="8" t="s">
+    <row r="16" spans="1:16" s="8" customFormat="1" ht="152.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B16" s="8" t="s">
+      <c r="B16" s="7" t="s">
         <v>223</v>
       </c>
-      <c r="C16" s="8" t="s">
+      <c r="C16" s="7" t="s">
         <v>215</v>
       </c>
-      <c r="D16" s="8" t="s">
+      <c r="D16" s="7" t="s">
         <v>216</v>
       </c>
-      <c r="E16" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="F16" s="8" t="s">
+      <c r="E16" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="F16" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="G16" s="8" t="s">
+      <c r="G16" s="7" t="s">
         <v>217</v>
       </c>
-      <c r="H16" s="8" t="s">
+      <c r="H16" s="7" t="s">
         <v>238</v>
       </c>
-      <c r="I16" s="8" t="s">
+      <c r="I16" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="J16" s="8" t="s">
+      <c r="J16" s="7" t="s">
         <v>218</v>
       </c>
-      <c r="K16" s="8" t="s">
+      <c r="K16" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="L16" s="8" t="s">
+      <c r="L16" s="7" t="s">
         <v>219</v>
       </c>
-      <c r="M16" s="8" t="s">
+      <c r="M16" s="7" t="s">
         <v>220</v>
       </c>
-      <c r="N16" s="8" t="s">
+      <c r="N16" s="7" t="s">
         <v>222</v>
       </c>
-      <c r="O16" s="8" t="s">
+      <c r="O16" s="7" t="s">
         <v>445</v>
       </c>
-      <c r="P16" s="8" t="s">
+      <c r="P16" s="7" t="s">
         <v>221</v>
       </c>
     </row>
-    <row r="17" spans="1:16" s="9" customFormat="1" ht="379.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="8" t="s">
+    <row r="17" spans="1:16" s="8" customFormat="1" ht="379.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="B17" s="8" t="s">
+      <c r="B17" s="7" t="s">
         <v>139</v>
       </c>
-      <c r="C17" s="8" t="s">
+      <c r="C17" s="7" t="s">
         <v>140</v>
       </c>
-      <c r="D17" s="8" t="s">
+      <c r="D17" s="7" t="s">
         <v>141</v>
       </c>
-      <c r="E17" s="8" t="s">
+      <c r="E17" s="7" t="s">
         <v>415</v>
       </c>
-      <c r="F17" s="8" t="s">
+      <c r="F17" s="7" t="s">
         <v>396</v>
       </c>
-      <c r="G17" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="H17" s="8" t="s">
+      <c r="G17" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="H17" s="7" t="s">
         <v>414</v>
       </c>
-      <c r="I17" s="8" t="s">
+      <c r="I17" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="J17" s="8" t="s">
+      <c r="J17" s="7" t="s">
         <v>142</v>
       </c>
-      <c r="K17" s="8" t="s">
+      <c r="K17" s="7" t="s">
         <v>421</v>
       </c>
-      <c r="L17" s="8" t="s">
+      <c r="L17" s="7" t="s">
         <v>143</v>
       </c>
-      <c r="M17" s="8" t="s">
+      <c r="M17" s="7" t="s">
         <v>144</v>
       </c>
-      <c r="N17" s="8" t="s">
+      <c r="N17" s="7" t="s">
         <v>145</v>
       </c>
-      <c r="O17" s="8" t="s">
+      <c r="O17" s="7" t="s">
         <v>447</v>
       </c>
-      <c r="P17" s="9" t="s">
+      <c r="P17" s="8" t="s">
         <v>446</v>
       </c>
     </row>
-    <row r="18" spans="1:16" s="9" customFormat="1" ht="304.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="8" t="s">
+    <row r="18" spans="1:16" s="8" customFormat="1" ht="304.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="B18" s="8" t="s">
+      <c r="B18" s="7" t="s">
         <v>146</v>
       </c>
-      <c r="C18" s="8" t="s">
+      <c r="C18" s="7" t="s">
         <v>147</v>
       </c>
-      <c r="D18" s="8" t="s">
+      <c r="D18" s="7" t="s">
         <v>148</v>
       </c>
-      <c r="E18" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="F18" s="8" t="s">
+      <c r="E18" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="F18" s="7" t="s">
         <v>396</v>
       </c>
-      <c r="G18" s="8" t="s">
+      <c r="G18" s="7" t="s">
         <v>149</v>
       </c>
-      <c r="H18" s="8" t="s">
+      <c r="H18" s="7" t="s">
         <v>238</v>
       </c>
-      <c r="I18" s="8" t="s">
+      <c r="I18" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="J18" s="8" t="s">
+      <c r="J18" s="7" t="s">
         <v>150</v>
       </c>
-      <c r="K18" s="8" t="s">
+      <c r="K18" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="L18" s="8" t="s">
+      <c r="L18" s="7" t="s">
         <v>151</v>
       </c>
-      <c r="M18" s="8" t="s">
+      <c r="M18" s="7" t="s">
         <v>152</v>
       </c>
-      <c r="N18" s="8" t="s">
+      <c r="N18" s="7" t="s">
         <v>153</v>
       </c>
-      <c r="O18" s="8" t="s">
+      <c r="O18" s="7" t="s">
         <v>149</v>
       </c>
-      <c r="P18" s="9" t="s">
+      <c r="P18" s="8" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="19" spans="1:16" s="9" customFormat="1" ht="409.6" x14ac:dyDescent="0.25">
-      <c r="A19" s="8" t="s">
+    <row r="19" spans="1:16" s="8" customFormat="1" ht="409.6" x14ac:dyDescent="0.25">
+      <c r="A19" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="B19" s="8" t="s">
+      <c r="B19" s="7" t="s">
         <v>155</v>
       </c>
-      <c r="C19" s="8" t="s">
+      <c r="C19" s="7" t="s">
         <v>156</v>
       </c>
-      <c r="D19" s="8" t="s">
+      <c r="D19" s="7" t="s">
         <v>157</v>
       </c>
-      <c r="E19" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="F19" s="8" t="s">
+      <c r="E19" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="F19" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="G19" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="H19" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="I19" s="8" t="s">
+      <c r="G19" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="H19" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="I19" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="J19" s="8" t="s">
+      <c r="J19" s="7" t="s">
         <v>158</v>
       </c>
-      <c r="K19" s="8" t="s">
+      <c r="K19" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="L19" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="M19" s="8" t="s">
+      <c r="L19" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="M19" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="N19" s="8" t="s">
+      <c r="N19" s="7" t="s">
         <v>449</v>
       </c>
-      <c r="O19" s="8" t="s">
+      <c r="O19" s="7" t="s">
         <v>159</v>
       </c>
-      <c r="P19" s="9" t="s">
+      <c r="P19" s="8" t="s">
         <v>448</v>
       </c>
     </row>
-    <row r="20" spans="1:16" s="9" customFormat="1" ht="132" x14ac:dyDescent="0.25">
-      <c r="A20" s="8" t="s">
+    <row r="20" spans="1:16" s="8" customFormat="1" ht="132" x14ac:dyDescent="0.25">
+      <c r="A20" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B20" s="8" t="s">
+      <c r="B20" s="7" t="s">
         <v>224</v>
       </c>
-      <c r="C20" s="8" t="s">
+      <c r="C20" s="7" t="s">
         <v>225</v>
       </c>
-      <c r="D20" s="8" t="s">
+      <c r="D20" s="7" t="s">
         <v>226</v>
       </c>
-      <c r="E20" s="8" t="s">
+      <c r="E20" s="7" t="s">
         <v>416</v>
       </c>
-      <c r="F20" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="G20" s="8" t="s">
+      <c r="F20" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="G20" s="7" t="s">
         <v>201</v>
       </c>
-      <c r="H20" s="8" t="s">
+      <c r="H20" s="7" t="s">
         <v>238</v>
       </c>
-      <c r="I20" s="8" t="s">
+      <c r="I20" s="7" t="s">
         <v>244</v>
       </c>
-      <c r="J20" s="8" t="s">
+      <c r="J20" s="7" t="s">
         <v>227</v>
       </c>
-      <c r="K20" s="8" t="s">
+      <c r="K20" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="L20" s="8" t="s">
+      <c r="L20" s="7" t="s">
         <v>228</v>
       </c>
-      <c r="M20" s="8" t="s">
+      <c r="M20" s="7" t="s">
         <v>229</v>
       </c>
-      <c r="N20" s="8" t="s">
+      <c r="N20" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="O20" s="8" t="s">
+      <c r="O20" s="7" t="s">
         <v>230</v>
       </c>
-      <c r="P20" s="9" t="s">
+      <c r="P20" s="8" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="21" spans="1:16" s="9" customFormat="1" ht="189" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="8" t="s">
+    <row r="21" spans="1:16" s="8" customFormat="1" ht="189" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B21" s="8" t="s">
+      <c r="B21" s="7" t="s">
         <v>233</v>
       </c>
-      <c r="C21" s="8" t="s">
+      <c r="C21" s="7" t="s">
         <v>234</v>
       </c>
-      <c r="D21" s="8" t="s">
+      <c r="D21" s="7" t="s">
         <v>236</v>
       </c>
-      <c r="E21" s="8" t="s">
+      <c r="E21" s="7" t="s">
         <v>235</v>
       </c>
-      <c r="F21" s="8" t="s">
+      <c r="F21" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="G21" s="8" t="s">
+      <c r="G21" s="7" t="s">
         <v>237</v>
       </c>
-      <c r="H21" s="8" t="s">
+      <c r="H21" s="7" t="s">
         <v>238</v>
       </c>
-      <c r="I21" s="8" t="s">
+      <c r="I21" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="J21" s="8" t="s">
+      <c r="J21" s="7" t="s">
         <v>202</v>
       </c>
-      <c r="K21" s="8" t="s">
+      <c r="K21" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="L21" s="8" t="s">
+      <c r="L21" s="7" t="s">
         <v>239</v>
       </c>
-      <c r="M21" s="8" t="s">
+      <c r="M21" s="7" t="s">
         <v>240</v>
       </c>
-      <c r="N21" s="8" t="s">
+      <c r="N21" s="7" t="s">
         <v>241</v>
       </c>
-      <c r="O21" s="8" t="s">
+      <c r="O21" s="7" t="s">
         <v>242</v>
       </c>
-      <c r="P21" s="9" t="s">
+      <c r="P21" s="8" t="s">
         <v>243</v>
       </c>
     </row>
-    <row r="22" spans="1:16" s="9" customFormat="1" ht="250.8" x14ac:dyDescent="0.25">
-      <c r="A22" s="8" t="s">
+    <row r="22" spans="1:16" s="8" customFormat="1" ht="250.8" x14ac:dyDescent="0.25">
+      <c r="A22" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="B22" s="8" t="s">
+      <c r="B22" s="7" t="s">
         <v>160</v>
       </c>
-      <c r="C22" s="8" t="s">
+      <c r="C22" s="7" t="s">
         <v>161</v>
       </c>
-      <c r="D22" s="8" t="s">
+      <c r="D22" s="7" t="s">
         <v>162</v>
       </c>
-      <c r="E22" s="8" t="s">
+      <c r="E22" s="7" t="s">
         <v>235</v>
       </c>
-      <c r="F22" s="8" t="s">
+      <c r="F22" s="7" t="s">
         <v>163</v>
       </c>
-      <c r="G22" s="8" t="s">
+      <c r="G22" s="7" t="s">
         <v>163</v>
       </c>
-      <c r="H22" s="8" t="s">
+      <c r="H22" s="7" t="s">
         <v>238</v>
       </c>
-      <c r="I22" s="8" t="s">
+      <c r="I22" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="J22" s="8" t="s">
+      <c r="J22" s="7" t="s">
         <v>164</v>
       </c>
-      <c r="K22" s="8" t="s">
+      <c r="K22" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="L22" s="8" t="s">
+      <c r="L22" s="7" t="s">
         <v>451</v>
       </c>
-      <c r="M22" s="8" t="s">
+      <c r="M22" s="7" t="s">
         <v>165</v>
       </c>
-      <c r="N22" s="8" t="s">
+      <c r="N22" s="7" t="s">
         <v>450</v>
       </c>
-      <c r="O22" s="8" t="s">
+      <c r="O22" s="7" t="s">
         <v>166</v>
       </c>
-      <c r="P22" s="8" t="s">
+      <c r="P22" s="7" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="23" spans="1:16" s="9" customFormat="1" ht="145.19999999999999" x14ac:dyDescent="0.25">
-      <c r="A23" s="8" t="s">
+    <row r="23" spans="1:16" s="8" customFormat="1" ht="145.19999999999999" x14ac:dyDescent="0.25">
+      <c r="A23" s="7" t="s">
         <v>250</v>
       </c>
-      <c r="B23" s="8" t="s">
+      <c r="B23" s="7" t="s">
         <v>251</v>
       </c>
-      <c r="C23" s="8" t="s">
+      <c r="C23" s="7" t="s">
         <v>252</v>
       </c>
-      <c r="D23" s="8" t="s">
+      <c r="D23" s="7" t="s">
         <v>253</v>
       </c>
-      <c r="E23" s="8" t="s">
+      <c r="E23" s="7" t="s">
         <v>235</v>
       </c>
-      <c r="F23" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="G23" s="8" t="s">
+      <c r="F23" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="G23" s="7" t="s">
         <v>254</v>
       </c>
-      <c r="H23" s="8" t="s">
+      <c r="H23" s="7" t="s">
         <v>418</v>
       </c>
-      <c r="I23" s="8" t="s">
+      <c r="I23" s="7" t="s">
         <v>244</v>
       </c>
-      <c r="J23" s="8" t="s">
+      <c r="J23" s="7" t="s">
         <v>255</v>
       </c>
-      <c r="K23" s="8" t="s">
+      <c r="K23" s="7" t="s">
         <v>398</v>
       </c>
-      <c r="L23" s="8" t="s">
+      <c r="L23" s="7" t="s">
         <v>256</v>
       </c>
-      <c r="M23" s="8" t="s">
+      <c r="M23" s="7" t="s">
         <v>260</v>
       </c>
-      <c r="N23" s="8" t="s">
+      <c r="N23" s="7" t="s">
         <v>259</v>
       </c>
-      <c r="O23" s="8" t="s">
+      <c r="O23" s="7" t="s">
         <v>257</v>
       </c>
-      <c r="P23" s="9" t="s">
+      <c r="P23" s="8" t="s">
         <v>258</v>
       </c>
     </row>
-    <row r="24" spans="1:16" s="9" customFormat="1" ht="118.8" x14ac:dyDescent="0.25">
-      <c r="A24" s="8" t="s">
+    <row r="24" spans="1:16" s="8" customFormat="1" ht="118.8" x14ac:dyDescent="0.25">
+      <c r="A24" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="B24" s="8" t="s">
+      <c r="B24" s="7" t="s">
         <v>261</v>
       </c>
-      <c r="C24" s="8" t="s">
+      <c r="C24" s="7" t="s">
         <v>270</v>
       </c>
-      <c r="D24" s="8" t="s">
+      <c r="D24" s="7" t="s">
         <v>262</v>
       </c>
-      <c r="E24" s="9" t="s">
+      <c r="E24" s="8" t="s">
         <v>235</v>
       </c>
-      <c r="F24" s="8" t="s">
+      <c r="F24" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="G24" s="8" t="s">
+      <c r="G24" s="7" t="s">
         <v>263</v>
       </c>
-      <c r="H24" s="8" t="s">
+      <c r="H24" s="7" t="s">
         <v>264</v>
       </c>
-      <c r="I24" s="8" t="s">
+      <c r="I24" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="J24" s="8" t="s">
+      <c r="J24" s="7" t="s">
         <v>202</v>
       </c>
-      <c r="K24" s="8" t="s">
+      <c r="K24" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="L24" s="8" t="s">
+      <c r="L24" s="7" t="s">
         <v>265</v>
       </c>
-      <c r="M24" s="8" t="s">
+      <c r="M24" s="7" t="s">
         <v>266</v>
       </c>
-      <c r="N24" s="8" t="s">
+      <c r="N24" s="7" t="s">
         <v>267</v>
       </c>
-      <c r="O24" s="8" t="s">
+      <c r="O24" s="7" t="s">
         <v>268</v>
       </c>
-      <c r="P24" s="9" t="s">
+      <c r="P24" s="8" t="s">
         <v>269</v>
       </c>
     </row>
-    <row r="25" spans="1:16" s="9" customFormat="1" ht="184.8" x14ac:dyDescent="0.25">
-      <c r="A25" s="8" t="s">
+    <row r="25" spans="1:16" s="8" customFormat="1" ht="184.8" x14ac:dyDescent="0.25">
+      <c r="A25" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="B25" s="8" t="s">
+      <c r="B25" s="7" t="s">
         <v>293</v>
       </c>
-      <c r="C25" s="8" t="s">
+      <c r="C25" s="7" t="s">
         <v>168</v>
       </c>
-      <c r="D25" s="8" t="s">
+      <c r="D25" s="7" t="s">
         <v>169</v>
       </c>
-      <c r="E25" s="8" t="s">
+      <c r="E25" s="7" t="s">
         <v>170</v>
       </c>
-      <c r="F25" s="8" t="s">
+      <c r="F25" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="G25" s="8" t="s">
+      <c r="G25" s="7" t="s">
         <v>163</v>
       </c>
-      <c r="H25" s="8" t="s">
+      <c r="H25" s="7" t="s">
         <v>264</v>
       </c>
-      <c r="I25" s="8" t="s">
+      <c r="I25" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="J25" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="K25" s="8" t="s">
+      <c r="J25" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="K25" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="L25" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="M25" s="8" t="s">
+      <c r="L25" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="M25" s="7" t="s">
         <v>452</v>
       </c>
-      <c r="N25" s="8" t="s">
+      <c r="N25" s="7" t="s">
         <v>453</v>
       </c>
-      <c r="O25" s="8" t="s">
+      <c r="O25" s="7" t="s">
         <v>171</v>
       </c>
-      <c r="P25" s="9" t="s">
+      <c r="P25" s="8" t="s">
         <v>454</v>
       </c>
     </row>
-    <row r="26" spans="1:16" s="11" customFormat="1" ht="132" x14ac:dyDescent="0.25">
-      <c r="A26" s="10" t="s">
+    <row r="26" spans="1:16" s="10" customFormat="1" ht="132" x14ac:dyDescent="0.25">
+      <c r="A26" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="B26" s="10" t="s">
+      <c r="B26" s="9" t="s">
         <v>284</v>
       </c>
-      <c r="C26" s="10" t="s">
+      <c r="C26" s="9" t="s">
         <v>285</v>
       </c>
-      <c r="D26" s="10" t="s">
+      <c r="D26" s="9" t="s">
         <v>286</v>
       </c>
-      <c r="E26" s="10" t="s">
+      <c r="E26" s="9" t="s">
         <v>415</v>
       </c>
-      <c r="F26" s="10" t="s">
+      <c r="F26" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="G26" s="10" t="s">
+      <c r="G26" s="9" t="s">
         <v>163</v>
       </c>
-      <c r="H26" s="10" t="s">
+      <c r="H26" s="9" t="s">
         <v>287</v>
       </c>
-      <c r="I26" s="10" t="s">
+      <c r="I26" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="J26" s="10" t="s">
-        <v>56</v>
-      </c>
-      <c r="K26" s="10" t="s">
+      <c r="J26" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="K26" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="L26" s="10" t="s">
+      <c r="L26" s="9" t="s">
         <v>288</v>
       </c>
-      <c r="M26" s="10" t="s">
+      <c r="M26" s="9" t="s">
         <v>289</v>
       </c>
-      <c r="N26" s="10" t="s">
+      <c r="N26" s="9" t="s">
         <v>292</v>
       </c>
-      <c r="O26" s="10" t="s">
+      <c r="O26" s="9" t="s">
         <v>290</v>
       </c>
-      <c r="P26" s="11" t="s">
+      <c r="P26" s="10" t="s">
         <v>291</v>
       </c>
     </row>
-    <row r="27" spans="1:16" s="9" customFormat="1" ht="224.4" x14ac:dyDescent="0.25">
-      <c r="A27" s="8" t="s">
+    <row r="27" spans="1:16" s="8" customFormat="1" ht="224.4" x14ac:dyDescent="0.25">
+      <c r="A27" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B27" s="8" t="s">
+      <c r="B27" s="7" t="s">
         <v>172</v>
       </c>
-      <c r="C27" s="8" t="s">
+      <c r="C27" s="7" t="s">
         <v>173</v>
       </c>
-      <c r="D27" s="8" t="s">
+      <c r="D27" s="7" t="s">
         <v>174</v>
       </c>
-      <c r="E27" s="8" t="s">
+      <c r="E27" s="7" t="s">
         <v>415</v>
       </c>
-      <c r="F27" s="8" t="s">
+      <c r="F27" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="G27" s="8" t="s">
+      <c r="G27" s="7" t="s">
         <v>175</v>
       </c>
-      <c r="H27" s="8" t="s">
+      <c r="H27" s="7" t="s">
         <v>287</v>
       </c>
-      <c r="I27" s="8" t="s">
+      <c r="I27" s="7" t="s">
         <v>423</v>
       </c>
-      <c r="J27" s="8" t="s">
+      <c r="J27" s="7" t="s">
         <v>176</v>
       </c>
-      <c r="K27" s="8" t="s">
+      <c r="K27" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="L27" s="8" t="s">
+      <c r="L27" s="7" t="s">
         <v>177</v>
       </c>
-      <c r="M27" s="8" t="s">
+      <c r="M27" s="7" t="s">
         <v>178</v>
       </c>
-      <c r="N27" s="8" t="s">
+      <c r="N27" s="7" t="s">
         <v>179</v>
       </c>
-      <c r="O27" s="8" t="s">
+      <c r="O27" s="7" t="s">
         <v>180</v>
       </c>
-      <c r="P27" s="9" t="s">
+      <c r="P27" s="8" t="s">
         <v>455</v>
       </c>
     </row>
-    <row r="28" spans="1:16" s="9" customFormat="1" ht="409.6" x14ac:dyDescent="0.25">
-      <c r="A28" s="8" t="s">
+    <row r="28" spans="1:16" s="8" customFormat="1" ht="409.6" x14ac:dyDescent="0.25">
+      <c r="A28" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="B28" s="8" t="s">
+      <c r="B28" s="7" t="s">
         <v>181</v>
       </c>
-      <c r="C28" s="8" t="s">
+      <c r="C28" s="7" t="s">
         <v>182</v>
       </c>
-      <c r="D28" s="8" t="s">
+      <c r="D28" s="7" t="s">
         <v>183</v>
       </c>
-      <c r="E28" s="8" t="s">
+      <c r="E28" s="7" t="s">
         <v>235</v>
       </c>
-      <c r="F28" s="8" t="s">
+      <c r="F28" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="G28" s="8" t="s">
+      <c r="G28" s="7" t="s">
         <v>184</v>
       </c>
-      <c r="H28" s="8" t="s">
+      <c r="H28" s="7" t="s">
         <v>287</v>
       </c>
-      <c r="I28" s="8" t="s">
+      <c r="I28" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="J28" s="8" t="s">
+      <c r="J28" s="7" t="s">
         <v>185</v>
       </c>
-      <c r="K28" s="8" t="s">
+      <c r="K28" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="L28" s="8" t="s">
+      <c r="L28" s="7" t="s">
         <v>186</v>
       </c>
-      <c r="M28" s="8" t="s">
+      <c r="M28" s="7" t="s">
         <v>187</v>
       </c>
-      <c r="N28" s="8" t="s">
+      <c r="N28" s="7" t="s">
         <v>188</v>
       </c>
-      <c r="O28" s="8" t="s">
+      <c r="O28" s="7" t="s">
         <v>189</v>
       </c>
-      <c r="P28" s="9" t="s">
+      <c r="P28" s="8" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="29" spans="1:16" s="9" customFormat="1" ht="273.60000000000002" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="8" t="s">
+    <row r="29" spans="1:16" s="8" customFormat="1" ht="273.60000000000002" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="B29" s="8" t="s">
+      <c r="B29" s="7" t="s">
         <v>197</v>
       </c>
-      <c r="C29" s="8" t="s">
+      <c r="C29" s="7" t="s">
         <v>198</v>
       </c>
-      <c r="D29" s="8" t="s">
+      <c r="D29" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="E29" s="8" t="s">
+      <c r="E29" s="7" t="s">
         <v>235</v>
       </c>
-      <c r="F29" s="8" t="s">
+      <c r="F29" s="7" t="s">
         <v>200</v>
       </c>
-      <c r="G29" s="8" t="s">
+      <c r="G29" s="7" t="s">
         <v>201</v>
       </c>
-      <c r="H29" s="8" t="s">
+      <c r="H29" s="7" t="s">
         <v>238</v>
       </c>
-      <c r="I29" s="8" t="s">
+      <c r="I29" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="J29" s="8" t="s">
+      <c r="J29" s="7" t="s">
         <v>202</v>
       </c>
-      <c r="K29" s="8" t="s">
+      <c r="K29" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="L29" s="8" t="s">
+      <c r="L29" s="7" t="s">
         <v>203</v>
       </c>
-      <c r="M29" s="12" t="s">
+      <c r="M29" s="11" t="s">
         <v>271</v>
       </c>
-      <c r="N29" s="8" t="s">
+      <c r="N29" s="7" t="s">
         <v>204</v>
       </c>
-      <c r="O29" s="8" t="s">
+      <c r="O29" s="7" t="s">
         <v>206</v>
       </c>
-      <c r="P29" s="9" t="s">
+      <c r="P29" s="8" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="30" spans="1:16" s="3" customFormat="1" ht="155.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="2" t="s">
+    <row r="30" spans="1:16" s="8" customFormat="1" ht="155.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="B30" s="2" t="s">
+      <c r="B30" s="7" t="s">
         <v>207</v>
       </c>
-      <c r="C30" s="2" t="s">
+      <c r="C30" s="7" t="s">
         <v>399</v>
       </c>
-      <c r="D30" s="2" t="s">
+      <c r="D30" s="7" t="s">
         <v>208</v>
       </c>
-      <c r="E30" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="F30" s="2" t="s">
+      <c r="E30" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="F30" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="G30" s="2" t="s">
+      <c r="G30" s="7" t="s">
         <v>209</v>
       </c>
-      <c r="H30" s="2" t="s">
+      <c r="H30" s="7" t="s">
         <v>340</v>
       </c>
-      <c r="I30" s="2" t="s">
+      <c r="I30" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="J30" s="2" t="s">
+      <c r="J30" s="7" t="s">
         <v>202</v>
       </c>
-      <c r="K30" s="2" t="s">
+      <c r="K30" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="L30" s="2" t="s">
+      <c r="L30" s="7" t="s">
         <v>210</v>
       </c>
-      <c r="M30" s="2" t="s">
+      <c r="M30" s="7" t="s">
         <v>211</v>
       </c>
-      <c r="N30" s="2" t="s">
+      <c r="N30" s="7" t="s">
         <v>212</v>
       </c>
-      <c r="O30" s="2" t="s">
+      <c r="O30" s="7" t="s">
         <v>214</v>
       </c>
-      <c r="P30" s="2" t="s">
+      <c r="P30" s="7" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="31" spans="1:16" s="3" customFormat="1" ht="105.6" x14ac:dyDescent="0.25">
-      <c r="A31" s="2" t="s">
+    <row r="31" spans="1:16" s="8" customFormat="1" ht="105.6" x14ac:dyDescent="0.25">
+      <c r="A31" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B31" s="2" t="s">
+      <c r="B31" s="7" t="s">
         <v>272</v>
       </c>
-      <c r="C31" s="2" t="s">
+      <c r="C31" s="7" t="s">
         <v>273</v>
       </c>
-      <c r="D31" s="2" t="s">
+      <c r="D31" s="7" t="s">
         <v>274</v>
       </c>
-      <c r="E31" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="F31" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="G31" s="2" t="s">
+      <c r="E31" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="F31" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="G31" s="7" t="s">
         <v>276</v>
       </c>
-      <c r="H31" s="2" t="s">
+      <c r="H31" s="7" t="s">
         <v>277</v>
       </c>
-      <c r="I31" s="2" t="s">
+      <c r="I31" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="J31" s="2" t="s">
+      <c r="J31" s="7" t="s">
         <v>278</v>
       </c>
-      <c r="K31" s="2" t="s">
+      <c r="K31" s="7" t="s">
         <v>422</v>
       </c>
-      <c r="L31" s="2" t="s">
+      <c r="L31" s="7" t="s">
         <v>279</v>
       </c>
-      <c r="M31" s="2" t="s">
+      <c r="M31" s="7" t="s">
         <v>280</v>
       </c>
-      <c r="N31" s="2" t="s">
+      <c r="N31" s="7" t="s">
         <v>281</v>
       </c>
-      <c r="O31" s="2" t="s">
+      <c r="O31" s="7" t="s">
         <v>282</v>
       </c>
-      <c r="P31" s="3" t="s">
+      <c r="P31" s="8" t="s">
         <v>283</v>
       </c>
     </row>
-    <row r="32" spans="1:16" s="3" customFormat="1" ht="290.39999999999998" x14ac:dyDescent="0.25">
-      <c r="A32" s="2" t="s">
+    <row r="32" spans="1:16" s="8" customFormat="1" ht="290.39999999999998" x14ac:dyDescent="0.25">
+      <c r="A32" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="B32" s="2" t="s">
+      <c r="B32" s="7" t="s">
         <v>191</v>
       </c>
-      <c r="C32" s="2" t="s">
+      <c r="C32" s="7" t="s">
         <v>192</v>
       </c>
-      <c r="D32" s="2" t="s">
+      <c r="D32" s="7" t="s">
         <v>193</v>
       </c>
-      <c r="E32" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="F32" s="2" t="s">
+      <c r="E32" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="F32" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="G32" s="2" t="s">
+      <c r="G32" s="7" t="s">
         <v>163</v>
       </c>
-      <c r="H32" s="2" t="s">
+      <c r="H32" s="7" t="s">
         <v>287</v>
       </c>
-      <c r="I32" s="2" t="s">
+      <c r="I32" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="J32" s="2" t="s">
+      <c r="J32" s="7" t="s">
         <v>194</v>
       </c>
-      <c r="K32" s="2" t="s">
+      <c r="K32" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="L32" s="2" t="s">
+      <c r="L32" s="7" t="s">
         <v>163</v>
       </c>
-      <c r="M32" s="2" t="s">
+      <c r="M32" s="7" t="s">
         <v>195</v>
       </c>
-      <c r="N32" s="2" t="s">
+      <c r="N32" s="7" t="s">
         <v>196</v>
       </c>
-      <c r="O32" s="2"/>
+      <c r="O32" s="7" t="s">
+        <v>457</v>
+      </c>
+      <c r="P32" s="8" t="s">
+        <v>456</v>
+      </c>
     </row>
-    <row r="33" spans="1:16" s="3" customFormat="1" ht="120" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="2" t="s">
+    <row r="33" spans="1:16" s="8" customFormat="1" ht="120" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="B33" s="2" t="s">
+      <c r="B33" s="7" t="s">
         <v>294</v>
       </c>
-      <c r="C33" s="2" t="s">
+      <c r="C33" s="7" t="s">
         <v>295</v>
       </c>
-      <c r="D33" s="2" t="s">
+      <c r="D33" s="7" t="s">
         <v>296</v>
       </c>
-      <c r="E33" s="2" t="s">
+      <c r="E33" s="7" t="s">
         <v>235</v>
       </c>
-      <c r="F33" s="2" t="s">
+      <c r="F33" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="G33" s="2" t="s">
+      <c r="G33" s="7" t="s">
         <v>298</v>
       </c>
-      <c r="H33" s="2" t="s">
+      <c r="H33" s="7" t="s">
         <v>287</v>
       </c>
-      <c r="I33" s="2" t="s">
+      <c r="I33" s="7" t="s">
         <v>424</v>
       </c>
-      <c r="J33" s="2" t="s">
+      <c r="J33" s="7" t="s">
         <v>299</v>
       </c>
-      <c r="K33" s="2" t="s">
+      <c r="K33" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="L33" s="2" t="s">
+      <c r="L33" s="7" t="s">
         <v>300</v>
       </c>
-      <c r="M33" s="2" t="s">
+      <c r="M33" s="7" t="s">
         <v>301</v>
       </c>
-      <c r="N33" s="2" t="s">
+      <c r="N33" s="7" t="s">
         <v>302</v>
       </c>
-      <c r="O33" s="2" t="s">
+      <c r="O33" s="7" t="s">
         <v>303</v>
       </c>
-      <c r="P33" s="3" t="s">
+      <c r="P33" s="8" t="s">
         <v>304</v>
       </c>
     </row>
-    <row r="34" spans="1:16" s="3" customFormat="1" ht="79.2" x14ac:dyDescent="0.25">
-      <c r="A34" s="2" t="s">
+    <row r="34" spans="1:16" s="10" customFormat="1" ht="79.2" x14ac:dyDescent="0.25">
+      <c r="A34" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="B34" s="2" t="s">
+      <c r="B34" s="9" t="s">
         <v>305</v>
       </c>
-      <c r="C34" s="2" t="s">
+      <c r="C34" s="9" t="s">
         <v>306</v>
       </c>
-      <c r="D34" s="2" t="s">
+      <c r="D34" s="9" t="s">
         <v>307</v>
       </c>
-      <c r="E34" s="4" t="s">
+      <c r="E34" s="12" t="s">
         <v>235</v>
       </c>
-      <c r="F34" s="2" t="s">
+      <c r="F34" s="9" t="s">
         <v>397</v>
       </c>
-      <c r="G34" s="2" t="s">
+      <c r="G34" s="9" t="s">
         <v>297</v>
       </c>
-      <c r="H34" s="2" t="s">
+      <c r="H34" s="9" t="s">
         <v>309</v>
       </c>
-      <c r="I34" s="2" t="s">
+      <c r="I34" s="9" t="s">
         <v>424</v>
       </c>
-      <c r="J34" s="2" t="s">
+      <c r="J34" s="9" t="s">
         <v>310</v>
       </c>
-      <c r="K34" s="2" t="s">
+      <c r="K34" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="L34" s="2" t="s">
+      <c r="L34" s="9" t="s">
         <v>202</v>
       </c>
-      <c r="M34" s="2" t="s">
+      <c r="M34" s="9" t="s">
         <v>311</v>
       </c>
-      <c r="N34" s="2" t="s">
+      <c r="N34" s="9" t="s">
         <v>312</v>
       </c>
-      <c r="O34" s="2" t="s">
+      <c r="O34" s="9" t="s">
         <v>313</v>
       </c>
-      <c r="P34" s="3" t="s">
+      <c r="P34" s="10" t="s">
         <v>314</v>
       </c>
     </row>
-    <row r="35" spans="1:16" s="3" customFormat="1" ht="92.4" x14ac:dyDescent="0.25">
-      <c r="A35" s="2" t="s">
+    <row r="35" spans="1:16" s="8" customFormat="1" ht="92.4" x14ac:dyDescent="0.25">
+      <c r="A35" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="B35" s="2" t="s">
+      <c r="B35" s="7" t="s">
         <v>315</v>
       </c>
-      <c r="C35" s="2" t="s">
+      <c r="C35" s="7" t="s">
         <v>316</v>
       </c>
-      <c r="D35" s="2" t="s">
+      <c r="D35" s="7" t="s">
         <v>317</v>
       </c>
-      <c r="E35" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="F35" s="2" t="s">
+      <c r="E35" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="F35" s="7" t="s">
         <v>308</v>
       </c>
-      <c r="G35" s="2" t="s">
+      <c r="G35" s="7" t="s">
         <v>297</v>
       </c>
-      <c r="H35" s="2" t="s">
+      <c r="H35" s="7" t="s">
         <v>238</v>
       </c>
-      <c r="I35" s="2" t="s">
+      <c r="I35" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="J35" s="2" t="s">
+      <c r="J35" s="7" t="s">
         <v>318</v>
       </c>
-      <c r="K35" s="2" t="s">
+      <c r="K35" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="L35" s="2" t="s">
+      <c r="L35" s="7" t="s">
         <v>319</v>
       </c>
-      <c r="M35" s="2" t="s">
+      <c r="M35" s="7" t="s">
         <v>320</v>
       </c>
-      <c r="N35" s="2" t="s">
+      <c r="N35" s="7" t="s">
         <v>321</v>
       </c>
-      <c r="O35" s="2" t="s">
+      <c r="O35" s="7" t="s">
         <v>322</v>
       </c>
-      <c r="P35" s="3" t="s">
+      <c r="P35" s="8" t="s">
         <v>323</v>
       </c>
     </row>
-    <row r="36" spans="1:16" s="3" customFormat="1" ht="79.2" x14ac:dyDescent="0.25">
-      <c r="A36" s="2" t="s">
+    <row r="36" spans="1:16" s="8" customFormat="1" ht="79.2" x14ac:dyDescent="0.25">
+      <c r="A36" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="B36" s="2" t="s">
+      <c r="B36" s="7" t="s">
         <v>324</v>
       </c>
-      <c r="C36" s="2" t="s">
+      <c r="C36" s="7" t="s">
         <v>325</v>
       </c>
-      <c r="D36" s="2" t="s">
+      <c r="D36" s="7" t="s">
         <v>326</v>
       </c>
-      <c r="E36" s="2" t="s">
+      <c r="E36" s="7" t="s">
         <v>235</v>
       </c>
-      <c r="F36" s="2" t="s">
+      <c r="F36" s="7" t="s">
         <v>328</v>
       </c>
-      <c r="G36" s="2" t="s">
+      <c r="G36" s="7" t="s">
         <v>327</v>
       </c>
-      <c r="H36" s="2" t="s">
+      <c r="H36" s="7" t="s">
         <v>238</v>
       </c>
-      <c r="I36" s="2" t="s">
+      <c r="I36" s="7" t="s">
         <v>424</v>
       </c>
-      <c r="J36" s="2" t="s">
+      <c r="J36" s="7" t="s">
         <v>329</v>
       </c>
-      <c r="K36" s="2" t="s">
+      <c r="K36" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="L36" s="2" t="s">
+      <c r="L36" s="7" t="s">
         <v>330</v>
       </c>
-      <c r="M36" s="2" t="s">
+      <c r="M36" s="7" t="s">
         <v>331</v>
       </c>
-      <c r="N36" s="2" t="s">
+      <c r="N36" s="7" t="s">
         <v>332</v>
       </c>
-      <c r="O36" s="2" t="s">
+      <c r="O36" s="7" t="s">
         <v>333</v>
       </c>
-      <c r="P36" s="3" t="s">
+      <c r="P36" s="8" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="37" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="10" t="s">
+    <row r="37" spans="1:16" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="B37" s="10" t="s">
+      <c r="B37" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="C37" s="10" t="s">
+      <c r="C37" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="D37" s="10" t="s">
+      <c r="D37" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="E37" s="10" t="s">
+      <c r="E37" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="F37" s="10" t="s">
+      <c r="F37" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="G37" s="10" t="s">
+      <c r="G37" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="H37" s="10" t="s">
+      <c r="H37" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="I37" s="10" t="s">
+      <c r="I37" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="J37" s="10" t="s">
+      <c r="J37" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="K37" s="10" t="s">
+      <c r="K37" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="L37" s="10" t="s">
+      <c r="L37" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="M37" s="10" t="s">
+      <c r="M37" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="N37" s="10"/>
-      <c r="O37" s="10" t="s">
+      <c r="N37" s="9"/>
+      <c r="O37" s="9" t="s">
         <v>46</v>
       </c>
     </row>
@@ -4109,53 +4120,53 @@
         <v>350</v>
       </c>
     </row>
-    <row r="40" spans="1:16" s="9" customFormat="1" ht="145.19999999999999" x14ac:dyDescent="0.25">
-      <c r="A40" s="8" t="s">
+    <row r="40" spans="1:16" s="8" customFormat="1" ht="145.19999999999999" x14ac:dyDescent="0.25">
+      <c r="A40" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="B40" s="8" t="s">
+      <c r="B40" s="7" t="s">
         <v>351</v>
       </c>
-      <c r="C40" s="8" t="s">
+      <c r="C40" s="7" t="s">
         <v>352</v>
       </c>
-      <c r="D40" s="8" t="s">
+      <c r="D40" s="7" t="s">
         <v>353</v>
       </c>
-      <c r="E40" s="8" t="s">
+      <c r="E40" s="7" t="s">
         <v>415</v>
       </c>
-      <c r="F40" s="8" t="s">
+      <c r="F40" s="7" t="s">
         <v>354</v>
       </c>
-      <c r="G40" s="8" t="s">
+      <c r="G40" s="7" t="s">
         <v>297</v>
       </c>
-      <c r="H40" s="8" t="s">
+      <c r="H40" s="7" t="s">
         <v>238</v>
       </c>
-      <c r="I40" s="8" t="s">
+      <c r="I40" s="7" t="s">
         <v>244</v>
       </c>
-      <c r="J40" s="8" t="s">
+      <c r="J40" s="7" t="s">
         <v>355</v>
       </c>
-      <c r="K40" s="8" t="s">
+      <c r="K40" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="L40" s="8" t="s">
+      <c r="L40" s="7" t="s">
         <v>356</v>
       </c>
-      <c r="M40" s="8" t="s">
+      <c r="M40" s="7" t="s">
         <v>357</v>
       </c>
-      <c r="N40" s="8" t="s">
+      <c r="N40" s="7" t="s">
         <v>358</v>
       </c>
-      <c r="O40" s="8" t="s">
+      <c r="O40" s="7" t="s">
         <v>359</v>
       </c>
-      <c r="P40" s="9" t="s">
+      <c r="P40" s="8" t="s">
         <v>360</v>
       </c>
     </row>
@@ -4359,53 +4370,53 @@
         <v>394</v>
       </c>
     </row>
-    <row r="45" spans="1:16" s="11" customFormat="1" ht="145.19999999999999" x14ac:dyDescent="0.25">
-      <c r="A45" s="10" t="s">
+    <row r="45" spans="1:16" s="10" customFormat="1" ht="145.19999999999999" x14ac:dyDescent="0.25">
+      <c r="A45" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="B45" s="10" t="s">
+      <c r="B45" s="9" t="s">
         <v>368</v>
       </c>
-      <c r="C45" s="10" t="s">
+      <c r="C45" s="9" t="s">
         <v>369</v>
       </c>
-      <c r="D45" s="10" t="s">
+      <c r="D45" s="9" t="s">
         <v>370</v>
       </c>
-      <c r="E45" s="10" t="s">
+      <c r="E45" s="9" t="s">
         <v>235</v>
       </c>
-      <c r="F45" s="10" t="s">
+      <c r="F45" s="9" t="s">
         <v>339</v>
       </c>
-      <c r="G45" s="10" t="s">
+      <c r="G45" s="9" t="s">
         <v>338</v>
       </c>
-      <c r="H45" s="10" t="s">
+      <c r="H45" s="9" t="s">
         <v>238</v>
       </c>
-      <c r="I45" s="10" t="s">
+      <c r="I45" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="J45" s="10" t="s">
+      <c r="J45" s="9" t="s">
         <v>371</v>
       </c>
-      <c r="K45" s="10" t="s">
+      <c r="K45" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="L45" s="10" t="s">
+      <c r="L45" s="9" t="s">
         <v>372</v>
       </c>
-      <c r="M45" s="10" t="s">
+      <c r="M45" s="9" t="s">
         <v>373</v>
       </c>
-      <c r="N45" s="10" t="s">
+      <c r="N45" s="9" t="s">
         <v>374</v>
       </c>
-      <c r="O45" s="10" t="s">
+      <c r="O45" s="9" t="s">
         <v>375</v>
       </c>
-      <c r="P45" s="11" t="s">
+      <c r="P45" s="10" t="s">
         <v>376</v>
       </c>
     </row>
@@ -4416,18 +4427,18 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4575,18 +4586,18 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1160EB8C-E200-4916-A3B3-9BF8115D37F8}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24F2579D-323E-48EA-8FED-D372AFFF0A04}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24F2579D-323E-48EA-8FED-D372AFFF0A04}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1160EB8C-E200-4916-A3B3-9BF8115D37F8}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Update Individual Annotations file with new data
</commit_message>
<xml_diff>
--- a/main/05_data_charting/data/Individual_Annotations.xlsx
+++ b/main/05_data_charting/data/Individual_Annotations.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27830"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\orincon\scoping-ml-wave-seismology\main\05_data_charting\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E1DFBFF-5CE3-415B-9780-6C6921C7F2F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1ED36729-46E7-4EEA-B662-F3A6BA8B2FF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{115BB8D9-8B86-4726-97F8-E06477FD353D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{115BB8D9-8B86-4726-97F8-E06477FD353D}"/>
   </bookViews>
   <sheets>
     <sheet name="Oscar" sheetId="4" r:id="rId1"/>
@@ -1782,15 +1782,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1838,10 +1835,7 @@
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <person displayName="Oscar Andres Rincon Cardeño" id="{89B996A1-6F87-4193-876B-892C93859AA0}" userId="S::orincon@eafit.edu.co::0eb7a243-0e55-4e0b-bc15-7fcfa587c292" providerId="AD"/>
-  <person displayName="Silvana Montoya Noguera" id="{08EE124C-73D2-424F-BF73-5FA5ED1E280C}" userId="S::smontoyan@eafit.edu.co::4cc234ee-4981-4b01-b85e-fd14b0eb0f53" providerId="AD"/>
-</personList>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2162,1865 +2156,1865 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C33CE99-2E5D-4F6C-B637-1B3AEFE552A0}">
   <dimension ref="A1:P45"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.09765625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="36.59765625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="39.296875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="36.59765625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="24.8984375" style="1" customWidth="1"/>
-    <col min="5" max="8" width="36.59765625" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="35.69921875" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="15" width="36.59765625" style="1" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="32.296875" style="1" bestFit="1" customWidth="1"/>
-    <col min="17" max="16384" width="9.09765625" style="1"/>
+    <col min="1" max="1" width="36.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="39.28515625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="36.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="24.85546875" style="1" customWidth="1"/>
+    <col min="5" max="8" width="36.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="35.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="15" width="36.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="32.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="17" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
+    <row r="1" spans="1:16" ht="26.45" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
         <v>400</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="4" t="s">
         <v>401</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="5" t="s">
         <v>402</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="5" t="s">
         <v>404</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="F1" s="5" t="s">
         <v>403</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="G1" s="5" t="s">
         <v>405</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="H1" s="5" t="s">
         <v>406</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="I1" s="5" t="s">
         <v>407</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="J1" s="5" t="s">
         <v>408</v>
       </c>
-      <c r="K1" s="6" t="s">
+      <c r="K1" s="5" t="s">
         <v>409</v>
       </c>
-      <c r="L1" s="6" t="s">
+      <c r="L1" s="5" t="s">
         <v>410</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="M1" s="4" t="s">
         <v>411</v>
       </c>
-      <c r="N1" s="5" t="s">
+      <c r="N1" s="4" t="s">
         <v>412</v>
       </c>
-      <c r="O1" s="5" t="s">
+      <c r="O1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="P1" s="4" t="s">
+      <c r="P1" s="3" t="s">
         <v>413</v>
       </c>
     </row>
-    <row r="2" spans="1:16" s="8" customFormat="1" ht="250.8" x14ac:dyDescent="0.25">
-      <c r="A2" s="7" t="s">
+    <row r="2" spans="1:16" s="7" customFormat="1" ht="267.75" x14ac:dyDescent="0.25">
+      <c r="A2" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="D2" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="E2" s="7" t="s">
+      <c r="E2" s="6" t="s">
         <v>417</v>
       </c>
-      <c r="F2" s="7" t="s">
+      <c r="F2" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="G2" s="7" t="s">
+      <c r="G2" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="H2" s="7" t="s">
+      <c r="H2" s="6" t="s">
         <v>238</v>
       </c>
-      <c r="I2" s="7" t="s">
+      <c r="I2" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="J2" s="7" t="s">
+      <c r="J2" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="K2" s="7" t="s">
+      <c r="K2" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="L2" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="M2" s="7" t="s">
+      <c r="L2" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="M2" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="N2" s="7" t="s">
+      <c r="N2" s="6" t="s">
         <v>425</v>
       </c>
-      <c r="O2" s="7" t="s">
+      <c r="O2" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="P2" s="8" t="s">
+      <c r="P2" s="7" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="3" spans="1:16" s="8" customFormat="1" ht="184.8" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
+    <row r="3" spans="1:16" s="7" customFormat="1" ht="204" x14ac:dyDescent="0.25">
+      <c r="A3" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D3" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="6" t="s">
         <v>415</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="F3" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="G3" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="H3" s="7" t="s">
+      <c r="G3" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="H3" s="6" t="s">
         <v>238</v>
       </c>
-      <c r="I3" s="7" t="s">
+      <c r="I3" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="J3" s="7" t="s">
+      <c r="J3" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="K3" s="7" t="s">
+      <c r="K3" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="L3" s="7" t="s">
+      <c r="L3" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="M3" s="7" t="s">
+      <c r="M3" s="6" t="s">
         <v>425</v>
       </c>
-      <c r="N3" s="7" t="s">
+      <c r="N3" s="6" t="s">
         <v>425</v>
       </c>
-      <c r="O3" s="7" t="s">
+      <c r="O3" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="P3" s="8" t="s">
+      <c r="P3" s="7" t="s">
         <v>426</v>
       </c>
     </row>
-    <row r="4" spans="1:16" s="8" customFormat="1" ht="201" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="7" t="s">
+    <row r="4" spans="1:16" s="7" customFormat="1" ht="201" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="E4" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="F4" s="7" t="s">
+      <c r="E4" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="F4" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="G4" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="H4" s="7" t="s">
+      <c r="G4" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="H4" s="6" t="s">
         <v>238</v>
       </c>
-      <c r="I4" s="7" t="s">
+      <c r="I4" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="J4" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="K4" s="7" t="s">
+      <c r="J4" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="K4" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="L4" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="M4" s="7" t="s">
+      <c r="L4" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="M4" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="N4" s="7" t="s">
+      <c r="N4" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="O4" s="7" t="s">
+      <c r="O4" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="P4" s="8" t="s">
+      <c r="P4" s="7" t="s">
         <v>427</v>
       </c>
     </row>
-    <row r="5" spans="1:16" s="8" customFormat="1" ht="210" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="7" t="s">
+    <row r="5" spans="1:16" s="7" customFormat="1" ht="210" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="D5" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="E5" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="F5" s="7" t="s">
+      <c r="E5" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="F5" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="G5" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="H5" s="7" t="s">
+      <c r="G5" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="H5" s="6" t="s">
         <v>238</v>
       </c>
-      <c r="I5" s="7" t="s">
+      <c r="I5" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="J5" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="K5" s="7" t="s">
+      <c r="J5" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="K5" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="L5" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="M5" s="7" t="s">
+      <c r="L5" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="M5" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="N5" s="7" t="s">
+      <c r="N5" s="6" t="s">
         <v>425</v>
       </c>
-      <c r="O5" s="7" t="s">
+      <c r="O5" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="P5" s="8" t="s">
+      <c r="P5" s="7" t="s">
         <v>428</v>
       </c>
     </row>
-    <row r="6" spans="1:16" s="8" customFormat="1" ht="250.8" x14ac:dyDescent="0.25">
-      <c r="A6" s="7" t="s">
+    <row r="6" spans="1:16" s="7" customFormat="1" ht="280.5" x14ac:dyDescent="0.25">
+      <c r="A6" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="E6" s="6" t="s">
         <v>170</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="F6" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="G6" s="7" t="s">
+      <c r="G6" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="H6" s="7" t="s">
+      <c r="H6" s="6" t="s">
         <v>238</v>
       </c>
-      <c r="I6" s="7" t="s">
+      <c r="I6" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="J6" s="7" t="s">
+      <c r="J6" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="K6" s="7" t="s">
+      <c r="K6" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="L6" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="M6" s="7" t="s">
+      <c r="L6" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="M6" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="N6" s="7" t="s">
+      <c r="N6" s="6" t="s">
         <v>425</v>
       </c>
-      <c r="O6" s="7" t="s">
+      <c r="O6" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="P6" s="8" t="s">
+      <c r="P6" s="7" t="s">
         <v>429</v>
       </c>
     </row>
-    <row r="7" spans="1:16" s="8" customFormat="1" ht="250.8" x14ac:dyDescent="0.25">
-      <c r="A7" s="7" t="s">
+    <row r="7" spans="1:16" s="7" customFormat="1" ht="280.5" x14ac:dyDescent="0.25">
+      <c r="A7" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D7" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="F7" s="7" t="s">
+      <c r="F7" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="G7" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="H7" s="7" t="s">
+      <c r="G7" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="H7" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="I7" s="7" t="s">
+      <c r="I7" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="J7" s="7" t="s">
+      <c r="J7" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="K7" s="7" t="s">
+      <c r="K7" s="6" t="s">
         <v>419</v>
       </c>
-      <c r="L7" s="7" t="s">
+      <c r="L7" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="M7" s="7" t="s">
+      <c r="M7" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="N7" s="7" t="s">
+      <c r="N7" s="6" t="s">
         <v>425</v>
       </c>
-      <c r="O7" s="7" t="s">
+      <c r="O7" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="P7" s="8" t="s">
+      <c r="P7" s="7" t="s">
         <v>430</v>
       </c>
     </row>
-    <row r="8" spans="1:16" s="8" customFormat="1" ht="184.8" x14ac:dyDescent="0.25">
-      <c r="A8" s="7" t="s">
+    <row r="8" spans="1:16" s="7" customFormat="1" ht="204" x14ac:dyDescent="0.25">
+      <c r="A8" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="6" t="s">
         <v>94</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="E8" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="F8" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="G8" s="7" t="s">
+      <c r="G8" s="6" t="s">
         <v>122</v>
       </c>
-      <c r="H8" s="7" t="s">
+      <c r="H8" s="6" t="s">
         <v>238</v>
       </c>
-      <c r="I8" s="7" t="s">
+      <c r="I8" s="6" t="s">
         <v>244</v>
       </c>
-      <c r="J8" s="7" t="s">
+      <c r="J8" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="K8" s="7" t="s">
+      <c r="K8" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="L8" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="M8" s="7" t="s">
+      <c r="L8" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="M8" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="N8" s="7" t="s">
+      <c r="N8" s="6" t="s">
         <v>425</v>
       </c>
-      <c r="O8" s="7" t="s">
+      <c r="O8" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="P8" s="8" t="s">
+      <c r="P8" s="7" t="s">
         <v>431</v>
       </c>
     </row>
-    <row r="9" spans="1:16" s="8" customFormat="1" ht="303.60000000000002" x14ac:dyDescent="0.25">
-      <c r="A9" s="7" t="s">
+    <row r="9" spans="1:16" s="7" customFormat="1" ht="344.25" x14ac:dyDescent="0.25">
+      <c r="A9" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="D9" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="E9" s="6" t="s">
         <v>235</v>
       </c>
-      <c r="F9" s="7" t="s">
+      <c r="F9" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="G9" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="H9" s="7" t="s">
+      <c r="G9" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="H9" s="6" t="s">
         <v>414</v>
       </c>
-      <c r="I9" s="7" t="s">
+      <c r="I9" s="6" t="s">
         <v>244</v>
       </c>
-      <c r="J9" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="K9" s="7" t="s">
+      <c r="J9" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="K9" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="L9" s="7" t="s">
+      <c r="L9" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="M9" s="7" t="s">
+      <c r="M9" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="N9" s="7" t="s">
+      <c r="N9" s="6" t="s">
         <v>425</v>
       </c>
-      <c r="O9" s="7" t="s">
+      <c r="O9" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="P9" s="8" t="s">
+      <c r="P9" s="7" t="s">
         <v>432</v>
       </c>
     </row>
-    <row r="10" spans="1:16" s="8" customFormat="1" ht="211.2" x14ac:dyDescent="0.25">
-      <c r="A10" s="7" t="s">
+    <row r="10" spans="1:16" s="7" customFormat="1" ht="229.5" x14ac:dyDescent="0.25">
+      <c r="A10" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="6" t="s">
         <v>108</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="D10" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="E10" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="F10" s="7" t="s">
+      <c r="E10" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="F10" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="G10" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="H10" s="7" t="s">
+      <c r="G10" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="H10" s="6" t="s">
         <v>238</v>
       </c>
-      <c r="I10" s="7" t="s">
+      <c r="I10" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="J10" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="K10" s="7" t="s">
+      <c r="J10" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="K10" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="L10" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="M10" s="7" t="s">
+      <c r="L10" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="M10" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="N10" s="7" t="s">
+      <c r="N10" s="6" t="s">
         <v>425</v>
       </c>
-      <c r="O10" s="7" t="s">
+      <c r="O10" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="P10" s="8" t="s">
+      <c r="P10" s="7" t="s">
         <v>433</v>
       </c>
     </row>
-    <row r="11" spans="1:16" s="8" customFormat="1" ht="198" x14ac:dyDescent="0.25">
-      <c r="A11" s="7" t="s">
+    <row r="11" spans="1:16" s="7" customFormat="1" ht="216.75" x14ac:dyDescent="0.25">
+      <c r="A11" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="6" t="s">
         <v>112</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="C11" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="D11" s="7" t="s">
+      <c r="D11" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="E11" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="F11" s="7" t="s">
+      <c r="E11" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="F11" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="G11" s="7" t="s">
+      <c r="G11" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="H11" s="7" t="s">
+      <c r="H11" s="6" t="s">
         <v>238</v>
       </c>
-      <c r="I11" s="7" t="s">
+      <c r="I11" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="J11" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="K11" s="7" t="s">
+      <c r="J11" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="K11" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="L11" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="M11" s="7" t="s">
+      <c r="L11" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="M11" s="6" t="s">
         <v>117</v>
       </c>
-      <c r="N11" s="7" t="s">
+      <c r="N11" s="6" t="s">
         <v>425</v>
       </c>
-      <c r="O11" s="7" t="s">
+      <c r="O11" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="P11" s="8" t="s">
+      <c r="P11" s="7" t="s">
         <v>434</v>
       </c>
     </row>
-    <row r="12" spans="1:16" s="8" customFormat="1" ht="264" x14ac:dyDescent="0.25">
-      <c r="A12" s="7" t="s">
+    <row r="12" spans="1:16" s="7" customFormat="1" ht="264" x14ac:dyDescent="0.25">
+      <c r="A12" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="C12" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="D12" s="6" t="s">
         <v>121</v>
       </c>
-      <c r="E12" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="F12" s="7" t="s">
+      <c r="E12" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="F12" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="G12" s="7" t="s">
+      <c r="G12" s="6" t="s">
         <v>122</v>
       </c>
-      <c r="H12" s="7" t="s">
+      <c r="H12" s="6" t="s">
         <v>238</v>
       </c>
-      <c r="I12" s="7" t="s">
+      <c r="I12" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="J12" s="7" t="s">
+      <c r="J12" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="K12" s="7" t="s">
+      <c r="K12" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="L12" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="M12" s="7" t="s">
+      <c r="L12" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="M12" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="N12" s="7" t="s">
+      <c r="N12" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="O12" s="7" t="s">
+      <c r="O12" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="P12" s="8" t="s">
+      <c r="P12" s="7" t="s">
         <v>435</v>
       </c>
     </row>
-    <row r="13" spans="1:16" s="8" customFormat="1" ht="303.60000000000002" x14ac:dyDescent="0.25">
-      <c r="A13" s="7" t="s">
+    <row r="13" spans="1:16" s="7" customFormat="1" ht="344.25" x14ac:dyDescent="0.25">
+      <c r="A13" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B13" s="7" t="s">
+      <c r="B13" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="C13" s="7" t="s">
+      <c r="C13" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="D13" s="7" t="s">
+      <c r="D13" s="6" t="s">
         <v>129</v>
       </c>
-      <c r="E13" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="F13" s="7" t="s">
+      <c r="E13" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="F13" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="G13" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="H13" s="7" t="s">
+      <c r="G13" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="H13" s="6" t="s">
         <v>238</v>
       </c>
-      <c r="I13" s="7" t="s">
+      <c r="I13" s="6" t="s">
         <v>244</v>
       </c>
-      <c r="J13" s="7" t="s">
+      <c r="J13" s="6" t="s">
         <v>130</v>
       </c>
-      <c r="K13" s="7" t="s">
+      <c r="K13" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="L13" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="M13" s="7" t="s">
+      <c r="L13" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="M13" s="6" t="s">
         <v>438</v>
       </c>
-      <c r="N13" s="7" t="s">
+      <c r="N13" s="6" t="s">
         <v>437</v>
       </c>
-      <c r="O13" s="7" t="s">
+      <c r="O13" s="6" t="s">
         <v>131</v>
       </c>
-      <c r="P13" s="8" t="s">
+      <c r="P13" s="7" t="s">
         <v>436</v>
       </c>
     </row>
-    <row r="14" spans="1:16" s="8" customFormat="1" ht="198" x14ac:dyDescent="0.25">
-      <c r="A14" s="7" t="s">
+    <row r="14" spans="1:16" s="7" customFormat="1" ht="204" x14ac:dyDescent="0.25">
+      <c r="A14" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="B14" s="6" t="s">
         <v>132</v>
       </c>
-      <c r="C14" s="7" t="s">
+      <c r="C14" s="6" t="s">
         <v>443</v>
       </c>
-      <c r="D14" s="7" t="s">
+      <c r="D14" s="6" t="s">
         <v>444</v>
       </c>
-      <c r="E14" s="7" t="s">
+      <c r="E14" s="6" t="s">
         <v>235</v>
       </c>
-      <c r="F14" s="7" t="s">
+      <c r="F14" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="G14" s="7" t="s">
+      <c r="G14" s="6" t="s">
         <v>246</v>
       </c>
-      <c r="H14" s="7" t="s">
+      <c r="H14" s="6" t="s">
         <v>309</v>
       </c>
-      <c r="I14" s="7" t="s">
+      <c r="I14" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="J14" s="7" t="s">
+      <c r="J14" s="6" t="s">
         <v>439</v>
       </c>
-      <c r="K14" s="7" t="s">
+      <c r="K14" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="L14" s="7" t="s">
+      <c r="L14" s="6" t="s">
         <v>133</v>
       </c>
-      <c r="M14" s="7" t="s">
+      <c r="M14" s="6" t="s">
         <v>440</v>
       </c>
-      <c r="N14" s="7" t="s">
+      <c r="N14" s="6" t="s">
         <v>441</v>
       </c>
-      <c r="O14" s="7" t="s">
+      <c r="O14" s="6" t="s">
         <v>134</v>
       </c>
-      <c r="P14" s="8" t="s">
+      <c r="P14" s="7" t="s">
         <v>442</v>
       </c>
     </row>
-    <row r="15" spans="1:16" s="8" customFormat="1" ht="290.39999999999998" x14ac:dyDescent="0.25">
-      <c r="A15" s="7" t="s">
+    <row r="15" spans="1:16" s="7" customFormat="1" ht="318.75" x14ac:dyDescent="0.25">
+      <c r="A15" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B15" s="7" t="s">
+      <c r="B15" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="C15" s="7" t="s">
+      <c r="C15" s="6" t="s">
         <v>245</v>
       </c>
-      <c r="D15" s="7" t="s">
+      <c r="D15" s="6" t="s">
         <v>136</v>
       </c>
-      <c r="E15" s="7" t="s">
+      <c r="E15" s="6" t="s">
         <v>235</v>
       </c>
-      <c r="F15" s="7" t="s">
+      <c r="F15" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="G15" s="7" t="s">
+      <c r="G15" s="6" t="s">
         <v>246</v>
       </c>
-      <c r="H15" s="7" t="s">
+      <c r="H15" s="6" t="s">
         <v>238</v>
       </c>
-      <c r="I15" s="7" t="s">
+      <c r="I15" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="J15" s="7" t="s">
+      <c r="J15" s="6" t="s">
         <v>247</v>
       </c>
-      <c r="K15" s="7" t="s">
+      <c r="K15" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="L15" s="7" t="s">
+      <c r="L15" s="6" t="s">
         <v>248</v>
       </c>
-      <c r="M15" s="7" t="s">
+      <c r="M15" s="6" t="s">
         <v>249</v>
       </c>
-      <c r="N15" s="7" t="s">
+      <c r="N15" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="O15" s="7" t="s">
+      <c r="O15" s="6" t="s">
         <v>138</v>
       </c>
-      <c r="P15" s="8" t="s">
+      <c r="P15" s="7" t="s">
         <v>442</v>
       </c>
     </row>
-    <row r="16" spans="1:16" s="8" customFormat="1" ht="152.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="7" t="s">
+    <row r="16" spans="1:16" s="7" customFormat="1" ht="152.44999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B16" s="7" t="s">
+      <c r="B16" s="6" t="s">
         <v>223</v>
       </c>
-      <c r="C16" s="7" t="s">
+      <c r="C16" s="6" t="s">
         <v>215</v>
       </c>
-      <c r="D16" s="7" t="s">
+      <c r="D16" s="6" t="s">
         <v>216</v>
       </c>
-      <c r="E16" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="F16" s="7" t="s">
+      <c r="E16" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="F16" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="G16" s="7" t="s">
+      <c r="G16" s="6" t="s">
         <v>217</v>
       </c>
-      <c r="H16" s="7" t="s">
+      <c r="H16" s="6" t="s">
         <v>238</v>
       </c>
-      <c r="I16" s="7" t="s">
+      <c r="I16" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="J16" s="7" t="s">
+      <c r="J16" s="6" t="s">
         <v>218</v>
       </c>
-      <c r="K16" s="7" t="s">
+      <c r="K16" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="L16" s="7" t="s">
+      <c r="L16" s="6" t="s">
         <v>219</v>
       </c>
-      <c r="M16" s="7" t="s">
+      <c r="M16" s="6" t="s">
         <v>220</v>
       </c>
-      <c r="N16" s="7" t="s">
+      <c r="N16" s="6" t="s">
         <v>222</v>
       </c>
-      <c r="O16" s="7" t="s">
+      <c r="O16" s="6" t="s">
         <v>445</v>
       </c>
-      <c r="P16" s="7" t="s">
+      <c r="P16" s="6" t="s">
         <v>221</v>
       </c>
     </row>
-    <row r="17" spans="1:16" s="8" customFormat="1" ht="379.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="7" t="s">
+    <row r="17" spans="1:16" s="7" customFormat="1" ht="379.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B17" s="7" t="s">
+      <c r="B17" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="C17" s="7" t="s">
+      <c r="C17" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="D17" s="7" t="s">
+      <c r="D17" s="6" t="s">
         <v>141</v>
       </c>
-      <c r="E17" s="7" t="s">
+      <c r="E17" s="6" t="s">
         <v>415</v>
       </c>
-      <c r="F17" s="7" t="s">
+      <c r="F17" s="6" t="s">
         <v>396</v>
       </c>
-      <c r="G17" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="H17" s="7" t="s">
+      <c r="G17" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="H17" s="6" t="s">
         <v>414</v>
       </c>
-      <c r="I17" s="7" t="s">
+      <c r="I17" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="J17" s="7" t="s">
+      <c r="J17" s="6" t="s">
         <v>142</v>
       </c>
-      <c r="K17" s="7" t="s">
+      <c r="K17" s="6" t="s">
         <v>421</v>
       </c>
-      <c r="L17" s="7" t="s">
+      <c r="L17" s="6" t="s">
         <v>143</v>
       </c>
-      <c r="M17" s="7" t="s">
+      <c r="M17" s="6" t="s">
         <v>144</v>
       </c>
-      <c r="N17" s="7" t="s">
+      <c r="N17" s="6" t="s">
         <v>145</v>
       </c>
-      <c r="O17" s="7" t="s">
+      <c r="O17" s="6" t="s">
         <v>447</v>
       </c>
-      <c r="P17" s="8" t="s">
+      <c r="P17" s="7" t="s">
         <v>446</v>
       </c>
     </row>
-    <row r="18" spans="1:16" s="8" customFormat="1" ht="304.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="7" t="s">
+    <row r="18" spans="1:16" s="7" customFormat="1" ht="304.14999999999998" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="B18" s="6" t="s">
         <v>146</v>
       </c>
-      <c r="C18" s="7" t="s">
+      <c r="C18" s="6" t="s">
         <v>147</v>
       </c>
-      <c r="D18" s="7" t="s">
+      <c r="D18" s="6" t="s">
         <v>148</v>
       </c>
-      <c r="E18" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="F18" s="7" t="s">
+      <c r="E18" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="F18" s="6" t="s">
         <v>396</v>
       </c>
-      <c r="G18" s="7" t="s">
+      <c r="G18" s="6" t="s">
         <v>149</v>
       </c>
-      <c r="H18" s="7" t="s">
+      <c r="H18" s="6" t="s">
         <v>238</v>
       </c>
-      <c r="I18" s="7" t="s">
+      <c r="I18" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="J18" s="7" t="s">
+      <c r="J18" s="6" t="s">
         <v>150</v>
       </c>
-      <c r="K18" s="7" t="s">
+      <c r="K18" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="L18" s="7" t="s">
+      <c r="L18" s="6" t="s">
         <v>151</v>
       </c>
-      <c r="M18" s="7" t="s">
+      <c r="M18" s="6" t="s">
         <v>152</v>
       </c>
-      <c r="N18" s="7" t="s">
+      <c r="N18" s="6" t="s">
         <v>153</v>
       </c>
-      <c r="O18" s="7" t="s">
+      <c r="O18" s="6" t="s">
         <v>149</v>
       </c>
-      <c r="P18" s="8" t="s">
+      <c r="P18" s="7" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="19" spans="1:16" s="8" customFormat="1" ht="409.6" x14ac:dyDescent="0.25">
-      <c r="A19" s="7" t="s">
+    <row r="19" spans="1:16" s="7" customFormat="1" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A19" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B19" s="7" t="s">
+      <c r="B19" s="6" t="s">
         <v>155</v>
       </c>
-      <c r="C19" s="7" t="s">
+      <c r="C19" s="6" t="s">
         <v>156</v>
       </c>
-      <c r="D19" s="7" t="s">
+      <c r="D19" s="6" t="s">
         <v>157</v>
       </c>
-      <c r="E19" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="F19" s="7" t="s">
+      <c r="E19" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="F19" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="G19" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="H19" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="I19" s="7" t="s">
+      <c r="G19" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="H19" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="I19" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="J19" s="7" t="s">
+      <c r="J19" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="K19" s="7" t="s">
+      <c r="K19" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="L19" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="M19" s="7" t="s">
+      <c r="L19" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="M19" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="N19" s="7" t="s">
+      <c r="N19" s="6" t="s">
         <v>449</v>
       </c>
-      <c r="O19" s="7" t="s">
+      <c r="O19" s="6" t="s">
         <v>159</v>
       </c>
-      <c r="P19" s="8" t="s">
+      <c r="P19" s="7" t="s">
         <v>448</v>
       </c>
     </row>
-    <row r="20" spans="1:16" s="8" customFormat="1" ht="132" x14ac:dyDescent="0.25">
-      <c r="A20" s="7" t="s">
+    <row r="20" spans="1:16" s="7" customFormat="1" ht="127.5" x14ac:dyDescent="0.25">
+      <c r="A20" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B20" s="7" t="s">
+      <c r="B20" s="6" t="s">
         <v>224</v>
       </c>
-      <c r="C20" s="7" t="s">
+      <c r="C20" s="6" t="s">
         <v>225</v>
       </c>
-      <c r="D20" s="7" t="s">
+      <c r="D20" s="6" t="s">
         <v>226</v>
       </c>
-      <c r="E20" s="7" t="s">
+      <c r="E20" s="6" t="s">
         <v>416</v>
       </c>
-      <c r="F20" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="G20" s="7" t="s">
+      <c r="F20" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="G20" s="6" t="s">
         <v>201</v>
       </c>
-      <c r="H20" s="7" t="s">
+      <c r="H20" s="6" t="s">
         <v>238</v>
       </c>
-      <c r="I20" s="7" t="s">
+      <c r="I20" s="6" t="s">
         <v>244</v>
       </c>
-      <c r="J20" s="7" t="s">
+      <c r="J20" s="6" t="s">
         <v>227</v>
       </c>
-      <c r="K20" s="7" t="s">
+      <c r="K20" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="L20" s="7" t="s">
+      <c r="L20" s="6" t="s">
         <v>228</v>
       </c>
-      <c r="M20" s="7" t="s">
+      <c r="M20" s="6" t="s">
         <v>229</v>
       </c>
-      <c r="N20" s="7" t="s">
+      <c r="N20" s="6" t="s">
         <v>232</v>
       </c>
-      <c r="O20" s="7" t="s">
+      <c r="O20" s="6" t="s">
         <v>230</v>
       </c>
-      <c r="P20" s="8" t="s">
+      <c r="P20" s="7" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="21" spans="1:16" s="8" customFormat="1" ht="189" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="7" t="s">
+    <row r="21" spans="1:16" s="7" customFormat="1" ht="189" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="B21" s="7" t="s">
+      <c r="B21" s="6" t="s">
         <v>233</v>
       </c>
-      <c r="C21" s="7" t="s">
+      <c r="C21" s="6" t="s">
         <v>234</v>
       </c>
-      <c r="D21" s="7" t="s">
+      <c r="D21" s="6" t="s">
         <v>236</v>
       </c>
-      <c r="E21" s="7" t="s">
+      <c r="E21" s="6" t="s">
         <v>235</v>
       </c>
-      <c r="F21" s="7" t="s">
+      <c r="F21" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="G21" s="7" t="s">
+      <c r="G21" s="6" t="s">
         <v>237</v>
       </c>
-      <c r="H21" s="7" t="s">
+      <c r="H21" s="6" t="s">
         <v>238</v>
       </c>
-      <c r="I21" s="7" t="s">
+      <c r="I21" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="J21" s="7" t="s">
+      <c r="J21" s="6" t="s">
         <v>202</v>
       </c>
-      <c r="K21" s="7" t="s">
+      <c r="K21" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="L21" s="7" t="s">
+      <c r="L21" s="6" t="s">
         <v>239</v>
       </c>
-      <c r="M21" s="7" t="s">
+      <c r="M21" s="6" t="s">
         <v>240</v>
       </c>
-      <c r="N21" s="7" t="s">
+      <c r="N21" s="6" t="s">
         <v>241</v>
       </c>
-      <c r="O21" s="7" t="s">
+      <c r="O21" s="6" t="s">
         <v>242</v>
       </c>
-      <c r="P21" s="8" t="s">
+      <c r="P21" s="7" t="s">
         <v>243</v>
       </c>
     </row>
-    <row r="22" spans="1:16" s="8" customFormat="1" ht="250.8" x14ac:dyDescent="0.25">
-      <c r="A22" s="7" t="s">
+    <row r="22" spans="1:16" s="7" customFormat="1" ht="267.75" x14ac:dyDescent="0.25">
+      <c r="A22" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B22" s="7" t="s">
+      <c r="B22" s="6" t="s">
         <v>160</v>
       </c>
-      <c r="C22" s="7" t="s">
+      <c r="C22" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="D22" s="7" t="s">
+      <c r="D22" s="6" t="s">
         <v>162</v>
       </c>
-      <c r="E22" s="7" t="s">
+      <c r="E22" s="6" t="s">
         <v>235</v>
       </c>
-      <c r="F22" s="7" t="s">
+      <c r="F22" s="6" t="s">
         <v>163</v>
       </c>
-      <c r="G22" s="7" t="s">
+      <c r="G22" s="6" t="s">
         <v>163</v>
       </c>
-      <c r="H22" s="7" t="s">
+      <c r="H22" s="6" t="s">
         <v>238</v>
       </c>
-      <c r="I22" s="7" t="s">
+      <c r="I22" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="J22" s="7" t="s">
+      <c r="J22" s="6" t="s">
         <v>164</v>
       </c>
-      <c r="K22" s="7" t="s">
+      <c r="K22" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="L22" s="7" t="s">
+      <c r="L22" s="6" t="s">
         <v>451</v>
       </c>
-      <c r="M22" s="7" t="s">
+      <c r="M22" s="6" t="s">
         <v>165</v>
       </c>
-      <c r="N22" s="7" t="s">
+      <c r="N22" s="6" t="s">
         <v>450</v>
       </c>
-      <c r="O22" s="7" t="s">
+      <c r="O22" s="6" t="s">
         <v>166</v>
       </c>
-      <c r="P22" s="7" t="s">
+      <c r="P22" s="6" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="23" spans="1:16" s="8" customFormat="1" ht="145.19999999999999" x14ac:dyDescent="0.25">
-      <c r="A23" s="7" t="s">
+    <row r="23" spans="1:16" s="7" customFormat="1" ht="153" x14ac:dyDescent="0.25">
+      <c r="A23" s="6" t="s">
         <v>250</v>
       </c>
-      <c r="B23" s="7" t="s">
+      <c r="B23" s="6" t="s">
         <v>251</v>
       </c>
-      <c r="C23" s="7" t="s">
+      <c r="C23" s="6" t="s">
         <v>252</v>
       </c>
-      <c r="D23" s="7" t="s">
+      <c r="D23" s="6" t="s">
         <v>253</v>
       </c>
-      <c r="E23" s="7" t="s">
+      <c r="E23" s="6" t="s">
         <v>235</v>
       </c>
-      <c r="F23" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="G23" s="7" t="s">
+      <c r="F23" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="G23" s="6" t="s">
         <v>254</v>
       </c>
-      <c r="H23" s="7" t="s">
+      <c r="H23" s="6" t="s">
         <v>418</v>
       </c>
-      <c r="I23" s="7" t="s">
+      <c r="I23" s="6" t="s">
         <v>244</v>
       </c>
-      <c r="J23" s="7" t="s">
+      <c r="J23" s="6" t="s">
         <v>255</v>
       </c>
-      <c r="K23" s="7" t="s">
+      <c r="K23" s="6" t="s">
         <v>398</v>
       </c>
-      <c r="L23" s="7" t="s">
+      <c r="L23" s="6" t="s">
         <v>256</v>
       </c>
-      <c r="M23" s="7" t="s">
+      <c r="M23" s="6" t="s">
         <v>260</v>
       </c>
-      <c r="N23" s="7" t="s">
+      <c r="N23" s="6" t="s">
         <v>259</v>
       </c>
-      <c r="O23" s="7" t="s">
+      <c r="O23" s="6" t="s">
         <v>257</v>
       </c>
-      <c r="P23" s="8" t="s">
+      <c r="P23" s="7" t="s">
         <v>258</v>
       </c>
     </row>
-    <row r="24" spans="1:16" s="8" customFormat="1" ht="118.8" x14ac:dyDescent="0.25">
-      <c r="A24" s="7" t="s">
+    <row r="24" spans="1:16" s="7" customFormat="1" ht="114.75" x14ac:dyDescent="0.25">
+      <c r="A24" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="B24" s="7" t="s">
+      <c r="B24" s="6" t="s">
         <v>261</v>
       </c>
-      <c r="C24" s="7" t="s">
+      <c r="C24" s="6" t="s">
         <v>270</v>
       </c>
-      <c r="D24" s="7" t="s">
+      <c r="D24" s="6" t="s">
         <v>262</v>
       </c>
-      <c r="E24" s="8" t="s">
+      <c r="E24" s="7" t="s">
         <v>235</v>
       </c>
-      <c r="F24" s="7" t="s">
+      <c r="F24" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="G24" s="7" t="s">
+      <c r="G24" s="6" t="s">
         <v>263</v>
       </c>
-      <c r="H24" s="7" t="s">
+      <c r="H24" s="6" t="s">
         <v>264</v>
       </c>
-      <c r="I24" s="7" t="s">
+      <c r="I24" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="J24" s="7" t="s">
+      <c r="J24" s="6" t="s">
         <v>202</v>
       </c>
-      <c r="K24" s="7" t="s">
+      <c r="K24" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="L24" s="7" t="s">
+      <c r="L24" s="6" t="s">
         <v>265</v>
       </c>
-      <c r="M24" s="7" t="s">
+      <c r="M24" s="6" t="s">
         <v>266</v>
       </c>
-      <c r="N24" s="7" t="s">
+      <c r="N24" s="6" t="s">
         <v>267</v>
       </c>
-      <c r="O24" s="7" t="s">
+      <c r="O24" s="6" t="s">
         <v>268</v>
       </c>
-      <c r="P24" s="8" t="s">
+      <c r="P24" s="7" t="s">
         <v>269</v>
       </c>
     </row>
-    <row r="25" spans="1:16" s="8" customFormat="1" ht="184.8" x14ac:dyDescent="0.25">
-      <c r="A25" s="7" t="s">
+    <row r="25" spans="1:16" s="7" customFormat="1" ht="191.25" x14ac:dyDescent="0.25">
+      <c r="A25" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="B25" s="7" t="s">
+      <c r="B25" s="6" t="s">
         <v>293</v>
       </c>
-      <c r="C25" s="7" t="s">
+      <c r="C25" s="6" t="s">
         <v>168</v>
       </c>
-      <c r="D25" s="7" t="s">
+      <c r="D25" s="6" t="s">
         <v>169</v>
       </c>
-      <c r="E25" s="7" t="s">
+      <c r="E25" s="6" t="s">
         <v>170</v>
       </c>
-      <c r="F25" s="7" t="s">
+      <c r="F25" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="G25" s="7" t="s">
+      <c r="G25" s="6" t="s">
         <v>163</v>
       </c>
-      <c r="H25" s="7" t="s">
+      <c r="H25" s="6" t="s">
         <v>264</v>
       </c>
-      <c r="I25" s="7" t="s">
+      <c r="I25" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="J25" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="K25" s="7" t="s">
+      <c r="J25" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="K25" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="L25" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="M25" s="7" t="s">
+      <c r="L25" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="M25" s="6" t="s">
         <v>452</v>
       </c>
-      <c r="N25" s="7" t="s">
+      <c r="N25" s="6" t="s">
         <v>453</v>
       </c>
-      <c r="O25" s="7" t="s">
+      <c r="O25" s="6" t="s">
         <v>171</v>
       </c>
-      <c r="P25" s="8" t="s">
+      <c r="P25" s="7" t="s">
         <v>454</v>
       </c>
     </row>
-    <row r="26" spans="1:16" s="10" customFormat="1" ht="132" x14ac:dyDescent="0.25">
-      <c r="A26" s="9" t="s">
+    <row r="26" spans="1:16" s="9" customFormat="1" ht="140.25" x14ac:dyDescent="0.25">
+      <c r="A26" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="B26" s="9" t="s">
+      <c r="B26" s="8" t="s">
         <v>284</v>
       </c>
-      <c r="C26" s="9" t="s">
+      <c r="C26" s="8" t="s">
         <v>285</v>
       </c>
-      <c r="D26" s="9" t="s">
+      <c r="D26" s="8" t="s">
         <v>286</v>
       </c>
-      <c r="E26" s="9" t="s">
+      <c r="E26" s="8" t="s">
         <v>415</v>
       </c>
-      <c r="F26" s="9" t="s">
+      <c r="F26" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="G26" s="9" t="s">
+      <c r="G26" s="8" t="s">
         <v>163</v>
       </c>
-      <c r="H26" s="9" t="s">
+      <c r="H26" s="8" t="s">
         <v>287</v>
       </c>
-      <c r="I26" s="9" t="s">
+      <c r="I26" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="J26" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="K26" s="9" t="s">
+      <c r="J26" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="K26" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="L26" s="9" t="s">
+      <c r="L26" s="8" t="s">
         <v>288</v>
       </c>
-      <c r="M26" s="9" t="s">
+      <c r="M26" s="8" t="s">
         <v>289</v>
       </c>
-      <c r="N26" s="9" t="s">
+      <c r="N26" s="8" t="s">
         <v>292</v>
       </c>
-      <c r="O26" s="9" t="s">
+      <c r="O26" s="8" t="s">
         <v>290</v>
       </c>
-      <c r="P26" s="10" t="s">
+      <c r="P26" s="9" t="s">
         <v>291</v>
       </c>
     </row>
-    <row r="27" spans="1:16" s="8" customFormat="1" ht="224.4" x14ac:dyDescent="0.25">
-      <c r="A27" s="7" t="s">
+    <row r="27" spans="1:16" s="7" customFormat="1" ht="255" x14ac:dyDescent="0.25">
+      <c r="A27" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="B27" s="7" t="s">
+      <c r="B27" s="6" t="s">
         <v>172</v>
       </c>
-      <c r="C27" s="7" t="s">
+      <c r="C27" s="6" t="s">
         <v>173</v>
       </c>
-      <c r="D27" s="7" t="s">
+      <c r="D27" s="6" t="s">
         <v>174</v>
       </c>
-      <c r="E27" s="7" t="s">
+      <c r="E27" s="6" t="s">
         <v>415</v>
       </c>
-      <c r="F27" s="7" t="s">
+      <c r="F27" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="G27" s="7" t="s">
+      <c r="G27" s="6" t="s">
         <v>175</v>
       </c>
-      <c r="H27" s="7" t="s">
+      <c r="H27" s="6" t="s">
         <v>287</v>
       </c>
-      <c r="I27" s="7" t="s">
+      <c r="I27" s="6" t="s">
         <v>423</v>
       </c>
-      <c r="J27" s="7" t="s">
+      <c r="J27" s="6" t="s">
         <v>176</v>
       </c>
-      <c r="K27" s="7" t="s">
+      <c r="K27" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="L27" s="7" t="s">
+      <c r="L27" s="6" t="s">
         <v>177</v>
       </c>
-      <c r="M27" s="7" t="s">
+      <c r="M27" s="6" t="s">
         <v>178</v>
       </c>
-      <c r="N27" s="7" t="s">
+      <c r="N27" s="6" t="s">
         <v>179</v>
       </c>
-      <c r="O27" s="7" t="s">
+      <c r="O27" s="6" t="s">
         <v>180</v>
       </c>
-      <c r="P27" s="8" t="s">
+      <c r="P27" s="7" t="s">
         <v>455</v>
       </c>
     </row>
-    <row r="28" spans="1:16" s="8" customFormat="1" ht="409.6" x14ac:dyDescent="0.25">
-      <c r="A28" s="7" t="s">
+    <row r="28" spans="1:16" s="7" customFormat="1" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A28" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="B28" s="7" t="s">
+      <c r="B28" s="6" t="s">
         <v>181</v>
       </c>
-      <c r="C28" s="7" t="s">
+      <c r="C28" s="6" t="s">
         <v>182</v>
       </c>
-      <c r="D28" s="7" t="s">
+      <c r="D28" s="6" t="s">
         <v>183</v>
       </c>
-      <c r="E28" s="7" t="s">
+      <c r="E28" s="6" t="s">
         <v>235</v>
       </c>
-      <c r="F28" s="7" t="s">
+      <c r="F28" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="G28" s="7" t="s">
+      <c r="G28" s="6" t="s">
         <v>184</v>
       </c>
-      <c r="H28" s="7" t="s">
+      <c r="H28" s="6" t="s">
         <v>287</v>
       </c>
-      <c r="I28" s="7" t="s">
+      <c r="I28" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="J28" s="7" t="s">
+      <c r="J28" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="K28" s="7" t="s">
+      <c r="K28" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="L28" s="7" t="s">
+      <c r="L28" s="6" t="s">
         <v>186</v>
       </c>
-      <c r="M28" s="7" t="s">
+      <c r="M28" s="6" t="s">
         <v>187</v>
       </c>
-      <c r="N28" s="7" t="s">
+      <c r="N28" s="6" t="s">
         <v>188</v>
       </c>
-      <c r="O28" s="7" t="s">
+      <c r="O28" s="6" t="s">
         <v>189</v>
       </c>
-      <c r="P28" s="8" t="s">
+      <c r="P28" s="7" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="29" spans="1:16" s="8" customFormat="1" ht="273.60000000000002" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="7" t="s">
+    <row r="29" spans="1:16" s="7" customFormat="1" ht="273.60000000000002" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B29" s="7" t="s">
+      <c r="B29" s="6" t="s">
         <v>197</v>
       </c>
-      <c r="C29" s="7" t="s">
+      <c r="C29" s="6" t="s">
         <v>198</v>
       </c>
-      <c r="D29" s="7" t="s">
+      <c r="D29" s="6" t="s">
         <v>199</v>
       </c>
-      <c r="E29" s="7" t="s">
+      <c r="E29" s="6" t="s">
         <v>235</v>
       </c>
-      <c r="F29" s="7" t="s">
+      <c r="F29" s="6" t="s">
         <v>200</v>
       </c>
-      <c r="G29" s="7" t="s">
+      <c r="G29" s="6" t="s">
         <v>201</v>
       </c>
-      <c r="H29" s="7" t="s">
+      <c r="H29" s="6" t="s">
         <v>238</v>
       </c>
-      <c r="I29" s="7" t="s">
+      <c r="I29" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="J29" s="7" t="s">
+      <c r="J29" s="6" t="s">
         <v>202</v>
       </c>
-      <c r="K29" s="7" t="s">
+      <c r="K29" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="L29" s="7" t="s">
+      <c r="L29" s="6" t="s">
         <v>203</v>
       </c>
-      <c r="M29" s="11" t="s">
+      <c r="M29" s="10" t="s">
         <v>271</v>
       </c>
-      <c r="N29" s="7" t="s">
+      <c r="N29" s="6" t="s">
         <v>204</v>
       </c>
-      <c r="O29" s="7" t="s">
+      <c r="O29" s="6" t="s">
         <v>206</v>
       </c>
-      <c r="P29" s="8" t="s">
+      <c r="P29" s="7" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="30" spans="1:16" s="8" customFormat="1" ht="155.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="7" t="s">
+    <row r="30" spans="1:16" s="7" customFormat="1" ht="155.44999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="B30" s="7" t="s">
+      <c r="B30" s="6" t="s">
         <v>207</v>
       </c>
-      <c r="C30" s="7" t="s">
+      <c r="C30" s="6" t="s">
         <v>399</v>
       </c>
-      <c r="D30" s="7" t="s">
+      <c r="D30" s="6" t="s">
         <v>208</v>
       </c>
-      <c r="E30" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="F30" s="7" t="s">
+      <c r="E30" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="F30" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="G30" s="7" t="s">
+      <c r="G30" s="6" t="s">
         <v>209</v>
       </c>
-      <c r="H30" s="7" t="s">
+      <c r="H30" s="6" t="s">
         <v>340</v>
       </c>
-      <c r="I30" s="7" t="s">
+      <c r="I30" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="J30" s="7" t="s">
+      <c r="J30" s="6" t="s">
         <v>202</v>
       </c>
-      <c r="K30" s="7" t="s">
+      <c r="K30" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="L30" s="7" t="s">
+      <c r="L30" s="6" t="s">
         <v>210</v>
       </c>
-      <c r="M30" s="7" t="s">
+      <c r="M30" s="6" t="s">
         <v>211</v>
       </c>
-      <c r="N30" s="7" t="s">
+      <c r="N30" s="6" t="s">
         <v>212</v>
       </c>
-      <c r="O30" s="7" t="s">
+      <c r="O30" s="6" t="s">
         <v>214</v>
       </c>
-      <c r="P30" s="7" t="s">
+      <c r="P30" s="6" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="31" spans="1:16" s="8" customFormat="1" ht="105.6" x14ac:dyDescent="0.25">
-      <c r="A31" s="7" t="s">
+    <row r="31" spans="1:16" s="7" customFormat="1" ht="102" x14ac:dyDescent="0.25">
+      <c r="A31" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="B31" s="7" t="s">
+      <c r="B31" s="6" t="s">
         <v>272</v>
       </c>
-      <c r="C31" s="7" t="s">
+      <c r="C31" s="6" t="s">
         <v>273</v>
       </c>
-      <c r="D31" s="7" t="s">
+      <c r="D31" s="6" t="s">
         <v>274</v>
       </c>
-      <c r="E31" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="F31" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="G31" s="7" t="s">
+      <c r="E31" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="F31" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="G31" s="6" t="s">
         <v>276</v>
       </c>
-      <c r="H31" s="7" t="s">
+      <c r="H31" s="6" t="s">
         <v>277</v>
       </c>
-      <c r="I31" s="7" t="s">
+      <c r="I31" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="J31" s="7" t="s">
+      <c r="J31" s="6" t="s">
         <v>278</v>
       </c>
-      <c r="K31" s="7" t="s">
+      <c r="K31" s="6" t="s">
         <v>422</v>
       </c>
-      <c r="L31" s="7" t="s">
+      <c r="L31" s="6" t="s">
         <v>279</v>
       </c>
-      <c r="M31" s="7" t="s">
+      <c r="M31" s="6" t="s">
         <v>280</v>
       </c>
-      <c r="N31" s="7" t="s">
+      <c r="N31" s="6" t="s">
         <v>281</v>
       </c>
-      <c r="O31" s="7" t="s">
+      <c r="O31" s="6" t="s">
         <v>282</v>
       </c>
-      <c r="P31" s="8" t="s">
+      <c r="P31" s="7" t="s">
         <v>283</v>
       </c>
     </row>
-    <row r="32" spans="1:16" s="8" customFormat="1" ht="290.39999999999998" x14ac:dyDescent="0.25">
-      <c r="A32" s="7" t="s">
+    <row r="32" spans="1:16" s="7" customFormat="1" ht="306" x14ac:dyDescent="0.25">
+      <c r="A32" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B32" s="7" t="s">
+      <c r="B32" s="6" t="s">
         <v>191</v>
       </c>
-      <c r="C32" s="7" t="s">
+      <c r="C32" s="6" t="s">
         <v>192</v>
       </c>
-      <c r="D32" s="7" t="s">
+      <c r="D32" s="6" t="s">
         <v>193</v>
       </c>
-      <c r="E32" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="F32" s="7" t="s">
+      <c r="E32" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="F32" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="G32" s="7" t="s">
+      <c r="G32" s="6" t="s">
         <v>163</v>
       </c>
-      <c r="H32" s="7" t="s">
+      <c r="H32" s="6" t="s">
         <v>287</v>
       </c>
-      <c r="I32" s="7" t="s">
+      <c r="I32" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="J32" s="7" t="s">
+      <c r="J32" s="6" t="s">
         <v>194</v>
       </c>
-      <c r="K32" s="7" t="s">
+      <c r="K32" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="L32" s="7" t="s">
+      <c r="L32" s="6" t="s">
         <v>163</v>
       </c>
-      <c r="M32" s="7" t="s">
+      <c r="M32" s="6" t="s">
         <v>195</v>
       </c>
-      <c r="N32" s="7" t="s">
+      <c r="N32" s="6" t="s">
         <v>196</v>
       </c>
-      <c r="O32" s="7" t="s">
+      <c r="O32" s="6" t="s">
         <v>457</v>
       </c>
-      <c r="P32" s="8" t="s">
+      <c r="P32" s="7" t="s">
         <v>456</v>
       </c>
     </row>
-    <row r="33" spans="1:16" s="8" customFormat="1" ht="120" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="7" t="s">
+    <row r="33" spans="1:16" s="7" customFormat="1" ht="120" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B33" s="7" t="s">
+      <c r="B33" s="6" t="s">
         <v>294</v>
       </c>
-      <c r="C33" s="7" t="s">
+      <c r="C33" s="6" t="s">
         <v>295</v>
       </c>
-      <c r="D33" s="7" t="s">
+      <c r="D33" s="6" t="s">
         <v>296</v>
       </c>
-      <c r="E33" s="7" t="s">
+      <c r="E33" s="6" t="s">
         <v>235</v>
       </c>
-      <c r="F33" s="7" t="s">
+      <c r="F33" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="G33" s="7" t="s">
+      <c r="G33" s="6" t="s">
         <v>298</v>
       </c>
-      <c r="H33" s="7" t="s">
+      <c r="H33" s="6" t="s">
         <v>287</v>
       </c>
-      <c r="I33" s="7" t="s">
+      <c r="I33" s="6" t="s">
         <v>424</v>
       </c>
-      <c r="J33" s="7" t="s">
+      <c r="J33" s="6" t="s">
         <v>299</v>
       </c>
-      <c r="K33" s="7" t="s">
+      <c r="K33" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="L33" s="7" t="s">
+      <c r="L33" s="6" t="s">
         <v>300</v>
       </c>
-      <c r="M33" s="7" t="s">
+      <c r="M33" s="6" t="s">
         <v>301</v>
       </c>
-      <c r="N33" s="7" t="s">
+      <c r="N33" s="6" t="s">
         <v>302</v>
       </c>
-      <c r="O33" s="7" t="s">
+      <c r="O33" s="6" t="s">
         <v>303</v>
       </c>
-      <c r="P33" s="8" t="s">
+      <c r="P33" s="7" t="s">
         <v>304</v>
       </c>
     </row>
-    <row r="34" spans="1:16" s="10" customFormat="1" ht="79.2" x14ac:dyDescent="0.25">
-      <c r="A34" s="9" t="s">
+    <row r="34" spans="1:16" s="9" customFormat="1" ht="76.5" x14ac:dyDescent="0.25">
+      <c r="A34" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="B34" s="9" t="s">
+      <c r="B34" s="8" t="s">
         <v>305</v>
       </c>
-      <c r="C34" s="9" t="s">
+      <c r="C34" s="8" t="s">
         <v>306</v>
       </c>
-      <c r="D34" s="9" t="s">
+      <c r="D34" s="8" t="s">
         <v>307</v>
       </c>
-      <c r="E34" s="12" t="s">
+      <c r="E34" s="11" t="s">
         <v>235</v>
       </c>
-      <c r="F34" s="9" t="s">
+      <c r="F34" s="8" t="s">
         <v>397</v>
       </c>
-      <c r="G34" s="9" t="s">
+      <c r="G34" s="8" t="s">
         <v>297</v>
       </c>
-      <c r="H34" s="9" t="s">
+      <c r="H34" s="8" t="s">
         <v>309</v>
       </c>
-      <c r="I34" s="9" t="s">
+      <c r="I34" s="8" t="s">
         <v>424</v>
       </c>
-      <c r="J34" s="9" t="s">
+      <c r="J34" s="8" t="s">
         <v>310</v>
       </c>
-      <c r="K34" s="9" t="s">
+      <c r="K34" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="L34" s="9" t="s">
+      <c r="L34" s="8" t="s">
         <v>202</v>
       </c>
-      <c r="M34" s="9" t="s">
+      <c r="M34" s="8" t="s">
         <v>311</v>
       </c>
-      <c r="N34" s="9" t="s">
+      <c r="N34" s="8" t="s">
         <v>312</v>
       </c>
-      <c r="O34" s="9" t="s">
+      <c r="O34" s="8" t="s">
         <v>313</v>
       </c>
-      <c r="P34" s="10" t="s">
+      <c r="P34" s="9" t="s">
         <v>314</v>
       </c>
     </row>
-    <row r="35" spans="1:16" s="8" customFormat="1" ht="92.4" x14ac:dyDescent="0.25">
-      <c r="A35" s="7" t="s">
+    <row r="35" spans="1:16" s="7" customFormat="1" ht="89.25" x14ac:dyDescent="0.25">
+      <c r="A35" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="B35" s="7" t="s">
+      <c r="B35" s="6" t="s">
         <v>315</v>
       </c>
-      <c r="C35" s="7" t="s">
+      <c r="C35" s="6" t="s">
         <v>316</v>
       </c>
-      <c r="D35" s="7" t="s">
+      <c r="D35" s="6" t="s">
         <v>317</v>
       </c>
-      <c r="E35" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="F35" s="7" t="s">
+      <c r="E35" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="F35" s="6" t="s">
         <v>308</v>
       </c>
-      <c r="G35" s="7" t="s">
+      <c r="G35" s="6" t="s">
         <v>297</v>
       </c>
-      <c r="H35" s="7" t="s">
+      <c r="H35" s="6" t="s">
         <v>238</v>
       </c>
-      <c r="I35" s="7" t="s">
+      <c r="I35" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="J35" s="7" t="s">
+      <c r="J35" s="6" t="s">
         <v>318</v>
       </c>
-      <c r="K35" s="7" t="s">
+      <c r="K35" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="L35" s="7" t="s">
+      <c r="L35" s="6" t="s">
         <v>319</v>
       </c>
-      <c r="M35" s="7" t="s">
+      <c r="M35" s="6" t="s">
         <v>320</v>
       </c>
-      <c r="N35" s="7" t="s">
+      <c r="N35" s="6" t="s">
         <v>321</v>
       </c>
-      <c r="O35" s="7" t="s">
+      <c r="O35" s="6" t="s">
         <v>322</v>
       </c>
-      <c r="P35" s="8" t="s">
+      <c r="P35" s="7" t="s">
         <v>323</v>
       </c>
     </row>
-    <row r="36" spans="1:16" s="8" customFormat="1" ht="79.2" x14ac:dyDescent="0.25">
-      <c r="A36" s="7" t="s">
+    <row r="36" spans="1:16" s="7" customFormat="1" ht="76.5" x14ac:dyDescent="0.25">
+      <c r="A36" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="B36" s="7" t="s">
+      <c r="B36" s="6" t="s">
         <v>324</v>
       </c>
-      <c r="C36" s="7" t="s">
+      <c r="C36" s="6" t="s">
         <v>325</v>
       </c>
-      <c r="D36" s="7" t="s">
+      <c r="D36" s="6" t="s">
         <v>326</v>
       </c>
-      <c r="E36" s="7" t="s">
+      <c r="E36" s="6" t="s">
         <v>235</v>
       </c>
-      <c r="F36" s="7" t="s">
+      <c r="F36" s="6" t="s">
         <v>328</v>
       </c>
-      <c r="G36" s="7" t="s">
+      <c r="G36" s="6" t="s">
         <v>327</v>
       </c>
-      <c r="H36" s="7" t="s">
+      <c r="H36" s="6" t="s">
         <v>238</v>
       </c>
-      <c r="I36" s="7" t="s">
+      <c r="I36" s="6" t="s">
         <v>424</v>
       </c>
-      <c r="J36" s="7" t="s">
+      <c r="J36" s="6" t="s">
         <v>329</v>
       </c>
-      <c r="K36" s="7" t="s">
+      <c r="K36" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="L36" s="7" t="s">
+      <c r="L36" s="6" t="s">
         <v>330</v>
       </c>
-      <c r="M36" s="7" t="s">
+      <c r="M36" s="6" t="s">
         <v>331</v>
       </c>
-      <c r="N36" s="7" t="s">
+      <c r="N36" s="6" t="s">
         <v>332</v>
       </c>
-      <c r="O36" s="7" t="s">
+      <c r="O36" s="6" t="s">
         <v>333</v>
       </c>
-      <c r="P36" s="8" t="s">
+      <c r="P36" s="7" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="37" spans="1:16" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="9" t="s">
+    <row r="37" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="B37" s="9" t="s">
+      <c r="B37" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="C37" s="9" t="s">
+      <c r="C37" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="D37" s="9" t="s">
+      <c r="D37" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="E37" s="9" t="s">
+      <c r="E37" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="F37" s="9" t="s">
+      <c r="F37" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="G37" s="9" t="s">
+      <c r="G37" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="H37" s="9" t="s">
+      <c r="H37" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="I37" s="9" t="s">
+      <c r="I37" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="J37" s="9" t="s">
+      <c r="J37" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="K37" s="9" t="s">
+      <c r="K37" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="L37" s="9" t="s">
+      <c r="L37" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="M37" s="9" t="s">
+      <c r="M37" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="N37" s="9"/>
-      <c r="O37" s="9" t="s">
+      <c r="N37" s="8"/>
+      <c r="O37" s="8" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="38" spans="1:16" s="3" customFormat="1" ht="132" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:16" ht="153" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>37</v>
       </c>
@@ -4066,11 +4060,11 @@
       <c r="O38" s="2" t="s">
         <v>343</v>
       </c>
-      <c r="P38" s="3" t="s">
+      <c r="P38" s="1" t="s">
         <v>344</v>
       </c>
     </row>
-    <row r="39" spans="1:16" s="3" customFormat="1" ht="132" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:16" ht="165.75" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>38</v>
       </c>
@@ -4116,61 +4110,61 @@
       <c r="O39" s="2" t="s">
         <v>349</v>
       </c>
-      <c r="P39" s="3" t="s">
+      <c r="P39" s="1" t="s">
         <v>350</v>
       </c>
     </row>
-    <row r="40" spans="1:16" s="8" customFormat="1" ht="145.19999999999999" x14ac:dyDescent="0.25">
-      <c r="A40" s="7" t="s">
+    <row r="40" spans="1:16" s="7" customFormat="1" ht="140.25" x14ac:dyDescent="0.25">
+      <c r="A40" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="B40" s="7" t="s">
+      <c r="B40" s="6" t="s">
         <v>351</v>
       </c>
-      <c r="C40" s="7" t="s">
+      <c r="C40" s="6" t="s">
         <v>352</v>
       </c>
-      <c r="D40" s="7" t="s">
+      <c r="D40" s="6" t="s">
         <v>353</v>
       </c>
-      <c r="E40" s="7" t="s">
+      <c r="E40" s="6" t="s">
         <v>415</v>
       </c>
-      <c r="F40" s="7" t="s">
+      <c r="F40" s="6" t="s">
         <v>354</v>
       </c>
-      <c r="G40" s="7" t="s">
+      <c r="G40" s="6" t="s">
         <v>297</v>
       </c>
-      <c r="H40" s="7" t="s">
+      <c r="H40" s="6" t="s">
         <v>238</v>
       </c>
-      <c r="I40" s="7" t="s">
+      <c r="I40" s="6" t="s">
         <v>244</v>
       </c>
-      <c r="J40" s="7" t="s">
+      <c r="J40" s="6" t="s">
         <v>355</v>
       </c>
-      <c r="K40" s="7" t="s">
+      <c r="K40" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="L40" s="7" t="s">
+      <c r="L40" s="6" t="s">
         <v>356</v>
       </c>
-      <c r="M40" s="7" t="s">
+      <c r="M40" s="6" t="s">
         <v>357</v>
       </c>
-      <c r="N40" s="7" t="s">
+      <c r="N40" s="6" t="s">
         <v>358</v>
       </c>
-      <c r="O40" s="7" t="s">
+      <c r="O40" s="6" t="s">
         <v>359</v>
       </c>
-      <c r="P40" s="8" t="s">
+      <c r="P40" s="7" t="s">
         <v>360</v>
       </c>
     </row>
-    <row r="41" spans="1:16" s="3" customFormat="1" ht="118.8" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:16" ht="114.75" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>40</v>
       </c>
@@ -4216,11 +4210,11 @@
       <c r="O41" s="2" t="s">
         <v>366</v>
       </c>
-      <c r="P41" s="3" t="s">
+      <c r="P41" s="1" t="s">
         <v>367</v>
       </c>
     </row>
-    <row r="42" spans="1:16" s="3" customFormat="1" ht="145.19999999999999" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:16" ht="153" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>41</v>
       </c>
@@ -4266,11 +4260,11 @@
       <c r="O42" s="2" t="s">
         <v>375</v>
       </c>
-      <c r="P42" s="3" t="s">
+      <c r="P42" s="1" t="s">
         <v>376</v>
       </c>
     </row>
-    <row r="43" spans="1:16" s="3" customFormat="1" ht="145.19999999999999" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:16" ht="153" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>42</v>
       </c>
@@ -4316,11 +4310,11 @@
       <c r="O43" s="2" t="s">
         <v>384</v>
       </c>
-      <c r="P43" s="3" t="s">
+      <c r="P43" s="1" t="s">
         <v>385</v>
       </c>
     </row>
-    <row r="44" spans="1:16" s="3" customFormat="1" ht="171.6" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:16" ht="178.5" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>43</v>
       </c>
@@ -4366,57 +4360,57 @@
       <c r="O44" s="2" t="s">
         <v>393</v>
       </c>
-      <c r="P44" s="3" t="s">
+      <c r="P44" s="1" t="s">
         <v>394</v>
       </c>
     </row>
-    <row r="45" spans="1:16" s="10" customFormat="1" ht="145.19999999999999" x14ac:dyDescent="0.25">
-      <c r="A45" s="9" t="s">
+    <row r="45" spans="1:16" s="9" customFormat="1" ht="153" x14ac:dyDescent="0.25">
+      <c r="A45" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="B45" s="9" t="s">
+      <c r="B45" s="8" t="s">
         <v>368</v>
       </c>
-      <c r="C45" s="9" t="s">
+      <c r="C45" s="8" t="s">
         <v>369</v>
       </c>
-      <c r="D45" s="9" t="s">
+      <c r="D45" s="8" t="s">
         <v>370</v>
       </c>
-      <c r="E45" s="9" t="s">
+      <c r="E45" s="8" t="s">
         <v>235</v>
       </c>
-      <c r="F45" s="9" t="s">
+      <c r="F45" s="8" t="s">
         <v>339</v>
       </c>
-      <c r="G45" s="9" t="s">
+      <c r="G45" s="8" t="s">
         <v>338</v>
       </c>
-      <c r="H45" s="9" t="s">
+      <c r="H45" s="8" t="s">
         <v>238</v>
       </c>
-      <c r="I45" s="9" t="s">
+      <c r="I45" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="J45" s="9" t="s">
+      <c r="J45" s="8" t="s">
         <v>371</v>
       </c>
-      <c r="K45" s="9" t="s">
+      <c r="K45" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="L45" s="9" t="s">
+      <c r="L45" s="8" t="s">
         <v>372</v>
       </c>
-      <c r="M45" s="9" t="s">
+      <c r="M45" s="8" t="s">
         <v>373</v>
       </c>
-      <c r="N45" s="9" t="s">
+      <c r="N45" s="8" t="s">
         <v>374</v>
       </c>
-      <c r="O45" s="9" t="s">
+      <c r="O45" s="8" t="s">
         <v>375</v>
       </c>
-      <c r="P45" s="10" t="s">
+      <c r="P45" s="9" t="s">
         <v>376</v>
       </c>
     </row>
@@ -4427,18 +4421,18 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4586,18 +4580,18 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24F2579D-323E-48EA-8FED-D372AFFF0A04}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1160EB8C-E200-4916-A3B3-9BF8115D37F8}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1160EB8C-E200-4916-A3B3-9BF8115D37F8}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24F2579D-323E-48EA-8FED-D372AFFF0A04}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>